<commit_message>
feat: add survey status sorting to UI and implement session-aware scraper initialization with manual confirmation support
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -16,28 +16,28 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1450" uniqueCount="501">
   <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>company_name</t>
-  </si>
-  <si>
-    <t>survey_status</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>global_status</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>timestamp</t>
-  </si>
-  <si>
-    <t>order</t>
+    <t>Kode Identitas</t>
+  </si>
+  <si>
+    <t>Nama Perusahaan</t>
+  </si>
+  <si>
+    <t>Status Dokumen</t>
+  </si>
+  <si>
+    <t>Email Tujuan</t>
+  </si>
+  <si>
+    <t>Status terakhir</t>
+  </si>
+  <si>
+    <t>Status History</t>
+  </si>
+  <si>
+    <t>Timestamp History</t>
+  </si>
+  <si>
+    <t>Urutan History</t>
   </si>
   <si>
     <t>7207011006001000 - UB - 1</t>
@@ -985,538 +985,538 @@
     <t>19 Mei 2026, 11:14:37</t>
   </si>
   <si>
+    <t>19 Mei 2026, 09:51:11</t>
+  </si>
+  <si>
     <t>19 Mei 2026, 09:51:10</t>
   </si>
   <si>
-    <t>19 Mei 2026, 09:51:11</t>
-  </si>
-  <si>
     <t>19 Mei 2026, 11:14:34</t>
   </si>
   <si>
+    <t>02 Jun 2026, 07:57:37</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 07:57:15</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:57:37</t>
-  </si>
-  <si>
     <t>01 Jun 2026, 23:07:49</t>
   </si>
   <si>
+    <t>02 Jun 2026, 07:38:30</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 07:38:27</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:38:30</t>
+    <t>02 Jun 2026, 07:23:56</t>
   </si>
   <si>
     <t>02 Jun 2026, 07:23:53</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:23:56</t>
+    <t>02 Jun 2026, 08:58:37</t>
   </si>
   <si>
     <t>02 Jun 2026, 08:56:24</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:58:37</t>
+    <t>02 Jun 2026, 03:53:26</t>
   </si>
   <si>
     <t>02 Jun 2026, 03:51:54</t>
   </si>
   <si>
-    <t>02 Jun 2026, 03:53:26</t>
+    <t>02 Jun 2026, 01:14:20</t>
   </si>
   <si>
     <t>02 Jun 2026, 01:14:16</t>
   </si>
   <si>
-    <t>02 Jun 2026, 01:14:20</t>
+    <t>02 Jun 2026, 04:33:23</t>
   </si>
   <si>
     <t>02 Jun 2026, 04:32:41</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:33:23</t>
+    <t>01 Jun 2026, 23:17:00</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:15:52</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:17:00</t>
+    <t>02 Jun 2026, 02:09:06</t>
   </si>
   <si>
     <t>02 Jun 2026, 02:09:05</t>
   </si>
   <si>
-    <t>02 Jun 2026, 02:09:06</t>
+    <t>01 Jun 2026, 23:00:27</t>
   </si>
   <si>
     <t>01 Jun 2026, 22:59:43</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:00:27</t>
+    <t>02 Jun 2026, 01:10:45</t>
   </si>
   <si>
     <t>02 Jun 2026, 01:10:14</t>
   </si>
   <si>
-    <t>02 Jun 2026, 01:10:45</t>
+    <t>02 Jun 2026, 07:48:23</t>
   </si>
   <si>
     <t>02 Jun 2026, 07:47:46</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:48:23</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 02:23:23</t>
   </si>
   <si>
     <t>01 Jun 2026, 22:48:15</t>
   </si>
   <si>
+    <t>02 Jun 2026, 04:39:27</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 04:39:23</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:39:27</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 08:57:51</t>
   </si>
   <si>
+    <t>02 Jun 2026, 09:04:21</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 09:04:02</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:04:21</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 00:55:50</t>
   </si>
   <si>
+    <t>02 Jun 2026, 02:30:55</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 02:29:47</t>
   </si>
   <si>
-    <t>02 Jun 2026, 02:30:55</t>
+    <t>02 Jun 2026, 04:02:15</t>
   </si>
   <si>
     <t>02 Jun 2026, 03:59:51</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:02:15</t>
+    <t>01 Jun 2026, 23:16:31</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:16:27</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:16:31</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 06:50:12</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:47:52</t>
   </si>
   <si>
+    <t>02 Jun 2026, 08:35:20</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 08:34:32</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:35:20</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 04:22:11</t>
   </si>
   <si>
+    <t>02 Jun 2026, 06:59:00</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 06:58:39</t>
   </si>
   <si>
-    <t>02 Jun 2026, 06:59:00</t>
+    <t>02 Jun 2026, 08:55:13</t>
   </si>
   <si>
     <t>02 Jun 2026, 08:52:30</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:55:13</t>
+    <t>01 Jun 2026, 23:34:59</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:34:56</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:34:59</t>
+    <t>02 Jun 2026, 03:44:55</t>
   </si>
   <si>
     <t>02 Jun 2026, 03:44:52</t>
   </si>
   <si>
-    <t>02 Jun 2026, 03:44:55</t>
+    <t>02 Jun 2026, 00:49:30</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:49:31</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:49:30</t>
+    <t>02 Jun 2026, 01:23:29</t>
   </si>
   <si>
     <t>02 Jun 2026, 01:23:24</t>
   </si>
   <si>
-    <t>02 Jun 2026, 01:23:29</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 06:19:08</t>
   </si>
   <si>
+    <t>02 Jun 2026, 09:06:32</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 09:04:47</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:06:32</t>
+    <t>02 Jun 2026, 06:33:41</t>
   </si>
   <si>
     <t>02 Jun 2026, 06:32:51</t>
   </si>
   <si>
-    <t>02 Jun 2026, 06:33:41</t>
+    <t>02 Jun 2026, 10:08:22</t>
   </si>
   <si>
     <t>02 Jun 2026, 10:04:58</t>
   </si>
   <si>
-    <t>02 Jun 2026, 10:08:22</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 06:31:35</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:35:32</t>
   </si>
   <si>
+    <t>02 Jun 2026, 08:52:48</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 08:52:14</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:52:48</t>
+    <t>02 Jun 2026, 00:41:02</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:41:01</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:41:02</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 09:17:21</t>
   </si>
   <si>
+    <t>02 Jun 2026, 09:12:41</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 09:11:39</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:12:41</t>
+    <t>02 Jun 2026, 05:22:20</t>
   </si>
   <si>
     <t>02 Jun 2026, 05:21:43</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:22:20</t>
+    <t>02 Jun 2026, 07:08:36</t>
   </si>
   <si>
     <t>02 Jun 2026, 07:08:18</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:08:36</t>
+    <t>01 Jun 2026, 23:30:02</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:29:34</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:30:02</t>
+    <t>02 Jun 2026, 11:53:38</t>
   </si>
   <si>
     <t>02 Jun 2026, 11:53:36</t>
   </si>
   <si>
-    <t>02 Jun 2026, 11:53:38</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 02:01:57</t>
   </si>
   <si>
+    <t>01 Jun 2026, 23:06:38</t>
+  </si>
+  <si>
     <t>01 Jun 2026, 23:06:35</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:06:38</t>
+    <t>02 Jun 2026, 10:34:01</t>
   </si>
   <si>
     <t>02 Jun 2026, 10:33:19</t>
   </si>
   <si>
-    <t>02 Jun 2026, 10:34:01</t>
+    <t>02 Jun 2026, 11:57:49</t>
   </si>
   <si>
     <t>02 Jun 2026, 11:49:47</t>
   </si>
   <si>
-    <t>02 Jun 2026, 11:57:49</t>
+    <t>02 Jun 2026, 00:34:13</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:34:08</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:34:13</t>
+    <t>02 Jun 2026, 03:39:29</t>
   </si>
   <si>
     <t>02 Jun 2026, 03:39:18</t>
   </si>
   <si>
-    <t>02 Jun 2026, 03:39:29</t>
+    <t>02 Jun 2026, 06:22:28</t>
   </si>
   <si>
     <t>02 Jun 2026, 06:22:25</t>
   </si>
   <si>
-    <t>02 Jun 2026, 06:22:28</t>
+    <t>02 Jun 2026, 00:06:29</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:06:21</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:06:29</t>
+    <t>02 Jun 2026, 04:45:27</t>
   </si>
   <si>
     <t>02 Jun 2026, 04:43:12</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:45:27</t>
+    <t>02 Jun 2026, 05:52:54</t>
   </si>
   <si>
     <t>02 Jun 2026, 05:52:21</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:52:54</t>
-  </si>
-  <si>
     <t>01 Jun 2026, 23:01:16</t>
   </si>
   <si>
+    <t>02 Jun 2026, 05:46:05</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 05:45:34</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:46:05</t>
+    <t>02 Jun 2026, 07:00:54</t>
   </si>
   <si>
     <t>02 Jun 2026, 07:00:24</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:00:54</t>
+    <t>02 Jun 2026, 09:00:10</t>
   </si>
   <si>
     <t>02 Jun 2026, 08:59:36</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:00:10</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 08:50:41</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:04:03</t>
   </si>
   <si>
+    <t>01 Jun 2026, 22:58:30</t>
+  </si>
+  <si>
     <t>01 Jun 2026, 22:57:07</t>
   </si>
   <si>
-    <t>01 Jun 2026, 22:58:30</t>
+    <t>02 Jun 2026, 03:10:04</t>
   </si>
   <si>
     <t>02 Jun 2026, 03:09:36</t>
   </si>
   <si>
-    <t>02 Jun 2026, 03:10:04</t>
+    <t>02 Jun 2026, 04:12:10</t>
   </si>
   <si>
     <t>02 Jun 2026, 04:11:35</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:12:10</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 01:06:09</t>
   </si>
   <si>
+    <t>02 Jun 2026, 00:37:51</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 00:37:47</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:37:51</t>
+    <t>02 Jun 2026, 11:37:42</t>
   </si>
   <si>
     <t>02 Jun 2026, 11:37:41</t>
   </si>
   <si>
-    <t>02 Jun 2026, 11:37:42</t>
+    <t>02 Jun 2026, 07:11:36</t>
   </si>
   <si>
     <t>02 Jun 2026, 07:11:00</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:11:36</t>
+    <t>02 Jun 2026, 09:45:54</t>
   </si>
   <si>
     <t>02 Jun 2026, 09:45:51</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:45:54</t>
+    <t>02 Jun 2026, 05:08:43</t>
   </si>
   <si>
     <t>02 Jun 2026, 05:07:16</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:08:43</t>
+    <t>02 Jun 2026, 06:39:45</t>
   </si>
   <si>
     <t>02 Jun 2026, 06:36:13</t>
   </si>
   <si>
-    <t>02 Jun 2026, 06:39:45</t>
+    <t>01 Jun 2026, 23:26:06</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:23:45</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:26:06</t>
+    <t>02 Jun 2026, 05:59:58</t>
   </si>
   <si>
     <t>02 Jun 2026, 05:59:12</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:59:58</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 07:10:57</t>
   </si>
   <si>
+    <t>02 Jun 2026, 11:47:27</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 11:47:26</t>
   </si>
   <si>
-    <t>02 Jun 2026, 11:47:27</t>
-  </si>
-  <si>
     <t>01 Jun 2026, 22:58:46</t>
   </si>
   <si>
+    <t>02 Jun 2026, 11:35:03</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 11:35:02</t>
   </si>
   <si>
-    <t>02 Jun 2026, 11:35:03</t>
+    <t>02 Jun 2026, 09:36:45</t>
   </si>
   <si>
     <t>02 Jun 2026, 09:36:44</t>
   </si>
   <si>
-    <t>02 Jun 2026, 09:36:45</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 03:21:19</t>
   </si>
   <si>
+    <t>02 Jun 2026, 07:01:31</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 07:01:30</t>
   </si>
   <si>
-    <t>02 Jun 2026, 07:01:31</t>
+    <t>01 Jun 2026, 23:00:08</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:00:04</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:00:08</t>
+    <t>02 Jun 2026, 00:12:21</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:11:48</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:12:21</t>
+    <t>02 Jun 2026, 04:58:35</t>
   </si>
   <si>
     <t>02 Jun 2026, 04:58:16</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:58:35</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 00:59:01</t>
   </si>
   <si>
+    <t>02 Jun 2026, 01:44:11</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 01:44:10</t>
   </si>
   <si>
-    <t>02 Jun 2026, 01:44:11</t>
+    <t>02 Jun 2026, 00:39:39</t>
   </si>
   <si>
     <t>02 Jun 2026, 00:39:34</t>
   </si>
   <si>
-    <t>02 Jun 2026, 00:39:39</t>
+    <t>02 Jun 2026, 05:57:24</t>
   </si>
   <si>
     <t>02 Jun 2026, 05:57:20</t>
   </si>
   <si>
-    <t>02 Jun 2026, 05:57:24</t>
+    <t>01 Jun 2026, 23:49:00</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:48:57</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:49:00</t>
-  </si>
-  <si>
     <t>02 Jun 2026, 07:31:06</t>
   </si>
   <si>
+    <t>02 Jun 2026, 03:12:01</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 03:11:28</t>
   </si>
   <si>
-    <t>02 Jun 2026, 03:12:01</t>
+    <t>02 Jun 2026, 08:35:38</t>
   </si>
   <si>
     <t>02 Jun 2026, 08:35:37</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:35:38</t>
+    <t>02 Jun 2026, 08:38:05</t>
   </si>
   <si>
     <t>02 Jun 2026, 08:37:43</t>
   </si>
   <si>
-    <t>02 Jun 2026, 08:38:05</t>
+    <t>02 Jun 2026, 10:28:53</t>
   </si>
   <si>
     <t>02 Jun 2026, 10:28:18</t>
   </si>
   <si>
-    <t>02 Jun 2026, 10:28:53</t>
+    <t>01 Jun 2026, 23:02:12</t>
   </si>
   <si>
     <t>01 Jun 2026, 23:02:08</t>
   </si>
   <si>
-    <t>01 Jun 2026, 23:02:12</t>
+    <t>02 Jun 2026, 01:30:50</t>
   </si>
   <si>
     <t>02 Jun 2026, 01:29:43</t>
   </si>
   <si>
-    <t>02 Jun 2026, 01:30:50</t>
-  </si>
-  <si>
     <t>01 Jun 2026, 23:53:12</t>
   </si>
   <si>
+    <t>02 Jun 2026, 04:55:14</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 04:54:25</t>
   </si>
   <si>
-    <t>02 Jun 2026, 04:55:14</t>
+    <t>02 Jun 2026, 02:20:17</t>
   </si>
   <si>
     <t>02 Jun 2026, 02:20:10</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 02:20:17</t>
   </si>
 </sst>
 </file>
@@ -1920,7 +1920,7 @@
         <v>320</v>
       </c>
       <c r="F2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G2" t="s">
         <v>322</v>
@@ -1946,7 +1946,7 @@
         <v>320</v>
       </c>
       <c r="F3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G3" t="s">
         <v>322</v>
@@ -1969,10 +1969,10 @@
         <v>218</v>
       </c>
       <c r="E4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G4" t="s">
         <v>323</v>
@@ -1995,10 +1995,10 @@
         <v>218</v>
       </c>
       <c r="E5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G5" t="s">
         <v>324</v>
@@ -2021,10 +2021,10 @@
         <v>219</v>
       </c>
       <c r="E6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G6" t="s">
         <v>325</v>
@@ -2047,10 +2047,10 @@
         <v>219</v>
       </c>
       <c r="E7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G7" t="s">
         <v>325</v>
@@ -2076,7 +2076,7 @@
         <v>320</v>
       </c>
       <c r="F8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G8" t="s">
         <v>326</v>
@@ -2102,7 +2102,7 @@
         <v>320</v>
       </c>
       <c r="F9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G9" t="s">
         <v>327</v>
@@ -2128,7 +2128,7 @@
         <v>320</v>
       </c>
       <c r="F10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G10" t="s">
         <v>328</v>
@@ -2154,7 +2154,7 @@
         <v>320</v>
       </c>
       <c r="F11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G11" t="s">
         <v>328</v>
@@ -2180,7 +2180,7 @@
         <v>320</v>
       </c>
       <c r="F12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G12" t="s">
         <v>329</v>
@@ -2206,7 +2206,7 @@
         <v>320</v>
       </c>
       <c r="F13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G13" t="s">
         <v>330</v>
@@ -2232,7 +2232,7 @@
         <v>320</v>
       </c>
       <c r="F14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G14" t="s">
         <v>331</v>
@@ -2258,7 +2258,7 @@
         <v>320</v>
       </c>
       <c r="F15" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G15" t="s">
         <v>332</v>
@@ -2284,7 +2284,7 @@
         <v>320</v>
       </c>
       <c r="F16" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G16" t="s">
         <v>333</v>
@@ -2310,7 +2310,7 @@
         <v>320</v>
       </c>
       <c r="F17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G17" t="s">
         <v>334</v>
@@ -2336,7 +2336,7 @@
         <v>320</v>
       </c>
       <c r="F18" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G18" t="s">
         <v>335</v>
@@ -2362,7 +2362,7 @@
         <v>320</v>
       </c>
       <c r="F19" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G19" t="s">
         <v>336</v>
@@ -2388,7 +2388,7 @@
         <v>320</v>
       </c>
       <c r="F20" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G20" t="s">
         <v>337</v>
@@ -2414,7 +2414,7 @@
         <v>320</v>
       </c>
       <c r="F21" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G21" t="s">
         <v>338</v>
@@ -2440,7 +2440,7 @@
         <v>320</v>
       </c>
       <c r="F22" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G22" t="s">
         <v>339</v>
@@ -2466,7 +2466,7 @@
         <v>320</v>
       </c>
       <c r="F23" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G23" t="s">
         <v>340</v>
@@ -2492,7 +2492,7 @@
         <v>320</v>
       </c>
       <c r="F24" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G24" t="s">
         <v>341</v>
@@ -2518,7 +2518,7 @@
         <v>320</v>
       </c>
       <c r="F25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G25" t="s">
         <v>342</v>
@@ -2544,7 +2544,7 @@
         <v>320</v>
       </c>
       <c r="F26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G26" t="s">
         <v>343</v>
@@ -2570,7 +2570,7 @@
         <v>320</v>
       </c>
       <c r="F27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G27" t="s">
         <v>344</v>
@@ -2596,7 +2596,7 @@
         <v>320</v>
       </c>
       <c r="F28" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G28" t="s">
         <v>345</v>
@@ -2622,7 +2622,7 @@
         <v>320</v>
       </c>
       <c r="F29" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G29" t="s">
         <v>346</v>
@@ -2648,7 +2648,7 @@
         <v>320</v>
       </c>
       <c r="F30" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G30" t="s">
         <v>347</v>
@@ -2674,7 +2674,7 @@
         <v>320</v>
       </c>
       <c r="F31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G31" t="s">
         <v>348</v>
@@ -2700,7 +2700,7 @@
         <v>320</v>
       </c>
       <c r="F32" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G32" t="s">
         <v>349</v>
@@ -2726,7 +2726,7 @@
         <v>320</v>
       </c>
       <c r="F33" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G33" t="s">
         <v>350</v>
@@ -2749,10 +2749,10 @@
         <v>233</v>
       </c>
       <c r="E34" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F34" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G34" t="s">
         <v>351</v>
@@ -2775,10 +2775,10 @@
         <v>233</v>
       </c>
       <c r="E35" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F35" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G35" t="s">
         <v>351</v>
@@ -2804,7 +2804,7 @@
         <v>320</v>
       </c>
       <c r="F36" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G36" t="s">
         <v>352</v>
@@ -2830,7 +2830,7 @@
         <v>320</v>
       </c>
       <c r="F37" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G37" t="s">
         <v>352</v>
@@ -2856,7 +2856,7 @@
         <v>320</v>
       </c>
       <c r="F38" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G38" t="s">
         <v>353</v>
@@ -2882,7 +2882,7 @@
         <v>320</v>
       </c>
       <c r="F39" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G39" t="s">
         <v>354</v>
@@ -2905,10 +2905,10 @@
         <v>236</v>
       </c>
       <c r="E40" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F40" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G40" t="s">
         <v>355</v>
@@ -2931,10 +2931,10 @@
         <v>236</v>
       </c>
       <c r="E41" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F41" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G41" t="s">
         <v>355</v>
@@ -2960,7 +2960,7 @@
         <v>320</v>
       </c>
       <c r="F42" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G42" t="s">
         <v>356</v>
@@ -2986,7 +2986,7 @@
         <v>320</v>
       </c>
       <c r="F43" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G43" t="s">
         <v>357</v>
@@ -3009,10 +3009,10 @@
         <v>238</v>
       </c>
       <c r="E44" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F44" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G44" t="s">
         <v>358</v>
@@ -3035,10 +3035,10 @@
         <v>238</v>
       </c>
       <c r="E45" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F45" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G45" t="s">
         <v>358</v>
@@ -3064,7 +3064,7 @@
         <v>320</v>
       </c>
       <c r="F46" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G46" t="s">
         <v>359</v>
@@ -3090,7 +3090,7 @@
         <v>320</v>
       </c>
       <c r="F47" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G47" t="s">
         <v>360</v>
@@ -3116,7 +3116,7 @@
         <v>320</v>
       </c>
       <c r="F48" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G48" t="s">
         <v>361</v>
@@ -3142,7 +3142,7 @@
         <v>320</v>
       </c>
       <c r="F49" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G49" t="s">
         <v>362</v>
@@ -3168,7 +3168,7 @@
         <v>320</v>
       </c>
       <c r="F50" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G50" t="s">
         <v>363</v>
@@ -3194,7 +3194,7 @@
         <v>320</v>
       </c>
       <c r="F51" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G51" t="s">
         <v>364</v>
@@ -3217,10 +3217,10 @@
         <v>242</v>
       </c>
       <c r="E52" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F52" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G52" t="s">
         <v>365</v>
@@ -3243,10 +3243,10 @@
         <v>242</v>
       </c>
       <c r="E53" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F53" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G53" t="s">
         <v>365</v>
@@ -3272,7 +3272,7 @@
         <v>320</v>
       </c>
       <c r="F54" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G54" t="s">
         <v>366</v>
@@ -3298,7 +3298,7 @@
         <v>320</v>
       </c>
       <c r="F55" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G55" t="s">
         <v>366</v>
@@ -3324,7 +3324,7 @@
         <v>320</v>
       </c>
       <c r="F56" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G56" t="s">
         <v>367</v>
@@ -3350,7 +3350,7 @@
         <v>320</v>
       </c>
       <c r="F57" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G57" t="s">
         <v>368</v>
@@ -3373,10 +3373,10 @@
         <v>245</v>
       </c>
       <c r="E58" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F58" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G58" t="s">
         <v>369</v>
@@ -3399,10 +3399,10 @@
         <v>245</v>
       </c>
       <c r="E59" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F59" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G59" t="s">
         <v>369</v>
@@ -3428,7 +3428,7 @@
         <v>320</v>
       </c>
       <c r="F60" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G60" t="s">
         <v>370</v>
@@ -3454,7 +3454,7 @@
         <v>320</v>
       </c>
       <c r="F61" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G61" t="s">
         <v>371</v>
@@ -3480,7 +3480,7 @@
         <v>320</v>
       </c>
       <c r="F62" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G62" t="s">
         <v>372</v>
@@ -3506,7 +3506,7 @@
         <v>320</v>
       </c>
       <c r="F63" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G63" t="s">
         <v>373</v>
@@ -3532,7 +3532,7 @@
         <v>320</v>
       </c>
       <c r="F64" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G64" t="s">
         <v>374</v>
@@ -3558,7 +3558,7 @@
         <v>320</v>
       </c>
       <c r="F65" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G65" t="s">
         <v>375</v>
@@ -3584,7 +3584,7 @@
         <v>320</v>
       </c>
       <c r="F66" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G66" t="s">
         <v>376</v>
@@ -3610,7 +3610,7 @@
         <v>320</v>
       </c>
       <c r="F67" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G67" t="s">
         <v>377</v>
@@ -3633,10 +3633,10 @@
         <v>250</v>
       </c>
       <c r="E68" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F68" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G68" t="s">
         <v>378</v>
@@ -3659,10 +3659,10 @@
         <v>250</v>
       </c>
       <c r="E69" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F69" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G69" t="s">
         <v>379</v>
@@ -3688,7 +3688,7 @@
         <v>320</v>
       </c>
       <c r="F70" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G70" t="s">
         <v>380</v>
@@ -3714,7 +3714,7 @@
         <v>320</v>
       </c>
       <c r="F71" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G71" t="s">
         <v>381</v>
@@ -3740,7 +3740,7 @@
         <v>320</v>
       </c>
       <c r="F72" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G72" t="s">
         <v>382</v>
@@ -3766,7 +3766,7 @@
         <v>320</v>
       </c>
       <c r="F73" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G73" t="s">
         <v>382</v>
@@ -3792,7 +3792,7 @@
         <v>320</v>
       </c>
       <c r="F74" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G74" t="s">
         <v>383</v>
@@ -3818,7 +3818,7 @@
         <v>320</v>
       </c>
       <c r="F75" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G75" t="s">
         <v>384</v>
@@ -3844,7 +3844,7 @@
         <v>320</v>
       </c>
       <c r="F76" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G76" t="s">
         <v>385</v>
@@ -3870,7 +3870,7 @@
         <v>320</v>
       </c>
       <c r="F77" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G77" t="s">
         <v>386</v>
@@ -3896,7 +3896,7 @@
         <v>320</v>
       </c>
       <c r="F78" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G78" t="s">
         <v>387</v>
@@ -3922,7 +3922,7 @@
         <v>320</v>
       </c>
       <c r="F79" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G79" t="s">
         <v>388</v>
@@ -3945,10 +3945,10 @@
         <v>256</v>
       </c>
       <c r="E80" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F80" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G80" t="s">
         <v>389</v>
@@ -3971,10 +3971,10 @@
         <v>256</v>
       </c>
       <c r="E81" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F81" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G81" t="s">
         <v>389</v>
@@ -4000,7 +4000,7 @@
         <v>320</v>
       </c>
       <c r="F82" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G82" t="s">
         <v>390</v>
@@ -4026,7 +4026,7 @@
         <v>320</v>
       </c>
       <c r="F83" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G83" t="s">
         <v>390</v>
@@ -4052,7 +4052,7 @@
         <v>320</v>
       </c>
       <c r="F84" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G84" t="s">
         <v>391</v>
@@ -4078,7 +4078,7 @@
         <v>320</v>
       </c>
       <c r="F85" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G85" t="s">
         <v>392</v>
@@ -4104,7 +4104,7 @@
         <v>320</v>
       </c>
       <c r="F86" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G86" t="s">
         <v>393</v>
@@ -4130,7 +4130,7 @@
         <v>320</v>
       </c>
       <c r="F87" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G87" t="s">
         <v>394</v>
@@ -4156,7 +4156,7 @@
         <v>320</v>
       </c>
       <c r="F88" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G88" t="s">
         <v>395</v>
@@ -4182,7 +4182,7 @@
         <v>320</v>
       </c>
       <c r="F89" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G89" t="s">
         <v>395</v>
@@ -4208,7 +4208,7 @@
         <v>320</v>
       </c>
       <c r="F90" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G90" t="s">
         <v>396</v>
@@ -4234,7 +4234,7 @@
         <v>320</v>
       </c>
       <c r="F91" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G91" t="s">
         <v>397</v>
@@ -4260,7 +4260,7 @@
         <v>320</v>
       </c>
       <c r="F92" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G92" t="s">
         <v>398</v>
@@ -4286,7 +4286,7 @@
         <v>320</v>
       </c>
       <c r="F93" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G93" t="s">
         <v>399</v>
@@ -4312,7 +4312,7 @@
         <v>320</v>
       </c>
       <c r="F94" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G94" t="s">
         <v>400</v>
@@ -4338,7 +4338,7 @@
         <v>320</v>
       </c>
       <c r="F95" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G95" t="s">
         <v>401</v>
@@ -4364,7 +4364,7 @@
         <v>320</v>
       </c>
       <c r="F96" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G96" t="s">
         <v>402</v>
@@ -4390,7 +4390,7 @@
         <v>320</v>
       </c>
       <c r="F97" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G97" t="s">
         <v>403</v>
@@ -4413,10 +4413,10 @@
         <v>265</v>
       </c>
       <c r="E98" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F98" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G98" t="s">
         <v>404</v>
@@ -4439,10 +4439,10 @@
         <v>265</v>
       </c>
       <c r="E99" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F99" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G99" t="s">
         <v>405</v>
@@ -4468,7 +4468,7 @@
         <v>320</v>
       </c>
       <c r="F100" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G100" t="s">
         <v>406</v>
@@ -4494,7 +4494,7 @@
         <v>320</v>
       </c>
       <c r="F101" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G101" t="s">
         <v>406</v>
@@ -4520,7 +4520,7 @@
         <v>320</v>
       </c>
       <c r="F102" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G102" t="s">
         <v>407</v>
@@ -4546,7 +4546,7 @@
         <v>320</v>
       </c>
       <c r="F103" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G103" t="s">
         <v>408</v>
@@ -4572,7 +4572,7 @@
         <v>320</v>
       </c>
       <c r="F104" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G104" t="s">
         <v>409</v>
@@ -4598,7 +4598,7 @@
         <v>320</v>
       </c>
       <c r="F105" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G105" t="s">
         <v>410</v>
@@ -4624,7 +4624,7 @@
         <v>320</v>
       </c>
       <c r="F106" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G106" t="s">
         <v>411</v>
@@ -4650,7 +4650,7 @@
         <v>320</v>
       </c>
       <c r="F107" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G107" t="s">
         <v>412</v>
@@ -4676,7 +4676,7 @@
         <v>320</v>
       </c>
       <c r="F108" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G108" t="s">
         <v>413</v>
@@ -4702,7 +4702,7 @@
         <v>320</v>
       </c>
       <c r="F109" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G109" t="s">
         <v>414</v>
@@ -4728,7 +4728,7 @@
         <v>320</v>
       </c>
       <c r="F110" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G110" t="s">
         <v>415</v>
@@ -4754,7 +4754,7 @@
         <v>320</v>
       </c>
       <c r="F111" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G111" t="s">
         <v>416</v>
@@ -4780,7 +4780,7 @@
         <v>320</v>
       </c>
       <c r="F112" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G112" t="s">
         <v>417</v>
@@ -4806,7 +4806,7 @@
         <v>320</v>
       </c>
       <c r="F113" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G113" t="s">
         <v>418</v>
@@ -4832,7 +4832,7 @@
         <v>320</v>
       </c>
       <c r="F114" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G114" t="s">
         <v>419</v>
@@ -4858,7 +4858,7 @@
         <v>320</v>
       </c>
       <c r="F115" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G115" t="s">
         <v>420</v>
@@ -4884,7 +4884,7 @@
         <v>320</v>
       </c>
       <c r="F116" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G116" t="s">
         <v>421</v>
@@ -4910,7 +4910,7 @@
         <v>320</v>
       </c>
       <c r="F117" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G117" t="s">
         <v>422</v>
@@ -4936,7 +4936,7 @@
         <v>320</v>
       </c>
       <c r="F118" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G118" t="s">
         <v>423</v>
@@ -4962,7 +4962,7 @@
         <v>320</v>
       </c>
       <c r="F119" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G119" t="s">
         <v>424</v>
@@ -4988,10 +4988,10 @@
         <v>320</v>
       </c>
       <c r="F120" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G120" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H120">
         <v>1</v>
@@ -5014,10 +5014,10 @@
         <v>320</v>
       </c>
       <c r="F121" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G121" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H121">
         <v>2</v>
@@ -5040,7 +5040,7 @@
         <v>320</v>
       </c>
       <c r="F122" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G122" t="s">
         <v>425</v>
@@ -5066,7 +5066,7 @@
         <v>320</v>
       </c>
       <c r="F123" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G123" t="s">
         <v>425</v>
@@ -5092,7 +5092,7 @@
         <v>320</v>
       </c>
       <c r="F124" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G124" t="s">
         <v>426</v>
@@ -5118,7 +5118,7 @@
         <v>320</v>
       </c>
       <c r="F125" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G125" t="s">
         <v>427</v>
@@ -5144,7 +5144,7 @@
         <v>320</v>
       </c>
       <c r="F126" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G126" t="s">
         <v>428</v>
@@ -5170,7 +5170,7 @@
         <v>320</v>
       </c>
       <c r="F127" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G127" t="s">
         <v>429</v>
@@ -5196,7 +5196,7 @@
         <v>320</v>
       </c>
       <c r="F128" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G128" t="s">
         <v>430</v>
@@ -5222,7 +5222,7 @@
         <v>320</v>
       </c>
       <c r="F129" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G129" t="s">
         <v>431</v>
@@ -5248,7 +5248,7 @@
         <v>320</v>
       </c>
       <c r="F130" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G130" t="s">
         <v>432</v>
@@ -5274,7 +5274,7 @@
         <v>320</v>
       </c>
       <c r="F131" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G131" t="s">
         <v>432</v>
@@ -5297,10 +5297,10 @@
         <v>282</v>
       </c>
       <c r="E132" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F132" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G132" t="s">
         <v>433</v>
@@ -5323,10 +5323,10 @@
         <v>282</v>
       </c>
       <c r="E133" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F133" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G133" t="s">
         <v>433</v>
@@ -5352,7 +5352,7 @@
         <v>320</v>
       </c>
       <c r="F134" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G134" t="s">
         <v>434</v>
@@ -5378,7 +5378,7 @@
         <v>320</v>
       </c>
       <c r="F135" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G135" t="s">
         <v>435</v>
@@ -5404,7 +5404,7 @@
         <v>320</v>
       </c>
       <c r="F136" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G136" t="s">
         <v>436</v>
@@ -5430,7 +5430,7 @@
         <v>320</v>
       </c>
       <c r="F137" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G137" t="s">
         <v>437</v>
@@ -5456,7 +5456,7 @@
         <v>320</v>
       </c>
       <c r="F138" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G138" t="s">
         <v>438</v>
@@ -5482,7 +5482,7 @@
         <v>320</v>
       </c>
       <c r="F139" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G139" t="s">
         <v>439</v>
@@ -5505,10 +5505,10 @@
         <v>286</v>
       </c>
       <c r="E140" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F140" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G140" t="s">
         <v>440</v>
@@ -5531,10 +5531,10 @@
         <v>286</v>
       </c>
       <c r="E141" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F141" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G141" t="s">
         <v>440</v>
@@ -5560,7 +5560,7 @@
         <v>320</v>
       </c>
       <c r="F142" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G142" t="s">
         <v>441</v>
@@ -5586,7 +5586,7 @@
         <v>320</v>
       </c>
       <c r="F143" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G143" t="s">
         <v>442</v>
@@ -5612,7 +5612,7 @@
         <v>320</v>
       </c>
       <c r="F144" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G144" t="s">
         <v>443</v>
@@ -5638,7 +5638,7 @@
         <v>320</v>
       </c>
       <c r="F145" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G145" t="s">
         <v>444</v>
@@ -5664,7 +5664,7 @@
         <v>320</v>
       </c>
       <c r="F146" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G146" t="s">
         <v>445</v>
@@ -5690,7 +5690,7 @@
         <v>320</v>
       </c>
       <c r="F147" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G147" t="s">
         <v>446</v>
@@ -5716,7 +5716,7 @@
         <v>320</v>
       </c>
       <c r="F148" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G148" t="s">
         <v>447</v>
@@ -5742,7 +5742,7 @@
         <v>320</v>
       </c>
       <c r="F149" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G149" t="s">
         <v>448</v>
@@ -5768,7 +5768,7 @@
         <v>320</v>
       </c>
       <c r="F150" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G150" t="s">
         <v>449</v>
@@ -5794,7 +5794,7 @@
         <v>320</v>
       </c>
       <c r="F151" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G151" t="s">
         <v>450</v>
@@ -5820,7 +5820,7 @@
         <v>320</v>
       </c>
       <c r="F152" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G152" t="s">
         <v>451</v>
@@ -5846,7 +5846,7 @@
         <v>320</v>
       </c>
       <c r="F153" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G153" t="s">
         <v>452</v>
@@ -5872,7 +5872,7 @@
         <v>320</v>
       </c>
       <c r="F154" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G154" t="s">
         <v>453</v>
@@ -5898,7 +5898,7 @@
         <v>320</v>
       </c>
       <c r="F155" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G155" t="s">
         <v>454</v>
@@ -5924,7 +5924,7 @@
         <v>320</v>
       </c>
       <c r="F156" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G156" t="s">
         <v>455</v>
@@ -5950,7 +5950,7 @@
         <v>320</v>
       </c>
       <c r="F157" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G157" t="s">
         <v>456</v>
@@ -5976,7 +5976,7 @@
         <v>320</v>
       </c>
       <c r="F158" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G158" t="s">
         <v>457</v>
@@ -6002,7 +6002,7 @@
         <v>320</v>
       </c>
       <c r="F159" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G159" t="s">
         <v>457</v>
@@ -6028,7 +6028,7 @@
         <v>320</v>
       </c>
       <c r="F160" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G160" t="s">
         <v>458</v>
@@ -6054,7 +6054,7 @@
         <v>320</v>
       </c>
       <c r="F161" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G161" t="s">
         <v>459</v>
@@ -6080,10 +6080,10 @@
         <v>320</v>
       </c>
       <c r="F162" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G162" t="s">
-        <v>460</v>
+        <v>346</v>
       </c>
       <c r="H162">
         <v>1</v>
@@ -6106,10 +6106,10 @@
         <v>320</v>
       </c>
       <c r="F163" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G163" t="s">
-        <v>345</v>
+        <v>460</v>
       </c>
       <c r="H163">
         <v>2</v>
@@ -6129,10 +6129,10 @@
         <v>298</v>
       </c>
       <c r="E164" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F164" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G164" t="s">
         <v>461</v>
@@ -6155,10 +6155,10 @@
         <v>298</v>
       </c>
       <c r="E165" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F165" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G165" t="s">
         <v>462</v>
@@ -6184,7 +6184,7 @@
         <v>320</v>
       </c>
       <c r="F166" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G166" t="s">
         <v>463</v>
@@ -6210,7 +6210,7 @@
         <v>320</v>
       </c>
       <c r="F167" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G167" t="s">
         <v>464</v>
@@ -6236,7 +6236,7 @@
         <v>320</v>
       </c>
       <c r="F168" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G168" t="s">
         <v>465</v>
@@ -6262,7 +6262,7 @@
         <v>320</v>
       </c>
       <c r="F169" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G169" t="s">
         <v>465</v>
@@ -6288,7 +6288,7 @@
         <v>320</v>
       </c>
       <c r="F170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G170" t="s">
         <v>466</v>
@@ -6314,7 +6314,7 @@
         <v>320</v>
       </c>
       <c r="F171" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G171" t="s">
         <v>467</v>
@@ -6340,7 +6340,7 @@
         <v>320</v>
       </c>
       <c r="F172" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G172" t="s">
         <v>468</v>
@@ -6366,7 +6366,7 @@
         <v>320</v>
       </c>
       <c r="F173" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G173" t="s">
         <v>469</v>
@@ -6392,7 +6392,7 @@
         <v>320</v>
       </c>
       <c r="F174" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G174" t="s">
         <v>470</v>
@@ -6418,7 +6418,7 @@
         <v>320</v>
       </c>
       <c r="F175" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G175" t="s">
         <v>471</v>
@@ -6444,7 +6444,7 @@
         <v>320</v>
       </c>
       <c r="F176" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G176" t="s">
         <v>472</v>
@@ -6470,7 +6470,7 @@
         <v>320</v>
       </c>
       <c r="F177" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G177" t="s">
         <v>473</v>
@@ -6496,7 +6496,7 @@
         <v>320</v>
       </c>
       <c r="F178" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G178" t="s">
         <v>474</v>
@@ -6522,7 +6522,7 @@
         <v>320</v>
       </c>
       <c r="F179" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G179" t="s">
         <v>474</v>
@@ -6548,7 +6548,7 @@
         <v>320</v>
       </c>
       <c r="F180" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G180" t="s">
         <v>475</v>
@@ -6574,7 +6574,7 @@
         <v>320</v>
       </c>
       <c r="F181" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G181" t="s">
         <v>476</v>
@@ -6600,7 +6600,7 @@
         <v>320</v>
       </c>
       <c r="F182" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G182" t="s">
         <v>477</v>
@@ -6626,7 +6626,7 @@
         <v>320</v>
       </c>
       <c r="F183" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G183" t="s">
         <v>478</v>
@@ -6652,7 +6652,7 @@
         <v>320</v>
       </c>
       <c r="F184" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G184" t="s">
         <v>479</v>
@@ -6678,7 +6678,7 @@
         <v>320</v>
       </c>
       <c r="F185" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G185" t="s">
         <v>480</v>
@@ -6704,7 +6704,7 @@
         <v>320</v>
       </c>
       <c r="F186" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G186" t="s">
         <v>481</v>
@@ -6730,7 +6730,7 @@
         <v>320</v>
       </c>
       <c r="F187" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G187" t="s">
         <v>482</v>
@@ -6753,10 +6753,10 @@
         <v>310</v>
       </c>
       <c r="E188" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F188" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G188" t="s">
         <v>483</v>
@@ -6779,10 +6779,10 @@
         <v>310</v>
       </c>
       <c r="E189" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F189" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G189" t="s">
         <v>483</v>
@@ -6808,7 +6808,7 @@
         <v>320</v>
       </c>
       <c r="F190" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G190" t="s">
         <v>484</v>
@@ -6834,7 +6834,7 @@
         <v>320</v>
       </c>
       <c r="F191" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G191" t="s">
         <v>485</v>
@@ -6860,7 +6860,7 @@
         <v>320</v>
       </c>
       <c r="F192" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G192" t="s">
         <v>486</v>
@@ -6886,7 +6886,7 @@
         <v>320</v>
       </c>
       <c r="F193" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G193" t="s">
         <v>487</v>
@@ -6912,7 +6912,7 @@
         <v>320</v>
       </c>
       <c r="F194" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G194" t="s">
         <v>488</v>
@@ -6938,7 +6938,7 @@
         <v>320</v>
       </c>
       <c r="F195" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G195" t="s">
         <v>489</v>
@@ -6964,7 +6964,7 @@
         <v>320</v>
       </c>
       <c r="F196" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G196" t="s">
         <v>490</v>
@@ -6990,7 +6990,7 @@
         <v>320</v>
       </c>
       <c r="F197" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G197" t="s">
         <v>491</v>
@@ -7016,7 +7016,7 @@
         <v>320</v>
       </c>
       <c r="F198" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G198" t="s">
         <v>492</v>
@@ -7042,7 +7042,7 @@
         <v>320</v>
       </c>
       <c r="F199" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G199" t="s">
         <v>493</v>
@@ -7068,7 +7068,7 @@
         <v>320</v>
       </c>
       <c r="F200" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G200" t="s">
         <v>494</v>
@@ -7094,7 +7094,7 @@
         <v>320</v>
       </c>
       <c r="F201" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G201" t="s">
         <v>495</v>
@@ -7120,7 +7120,7 @@
         <v>320</v>
       </c>
       <c r="F202" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G202" t="s">
         <v>496</v>
@@ -7146,7 +7146,7 @@
         <v>320</v>
       </c>
       <c r="F203" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G203" t="s">
         <v>496</v>
@@ -7172,7 +7172,7 @@
         <v>320</v>
       </c>
       <c r="F204" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G204" t="s">
         <v>497</v>
@@ -7198,7 +7198,7 @@
         <v>320</v>
       </c>
       <c r="F205" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G205" t="s">
         <v>498</v>
@@ -7224,7 +7224,7 @@
         <v>320</v>
       </c>
       <c r="F206" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G206" t="s">
         <v>499</v>
@@ -7250,7 +7250,7 @@
         <v>320</v>
       </c>
       <c r="F207" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G207" t="s">
         <v>500</v>

</xml_diff>

<commit_message>
feat: add dashboard monitoring tools and update survey data records
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -139,12 +139,12 @@
     <t>7204070009001200 - UB - 1</t>
   </si>
   <si>
+    <t>7204070012000800 - UB - 1</t>
+  </si>
+  <si>
     <t>7204070011000301 - UB - 3</t>
   </si>
   <si>
-    <t>7204070012000800 - UB - 1</t>
-  </si>
-  <si>
     <t>7205090009000301 - UB - 1</t>
   </si>
   <si>
@@ -490,12 +490,12 @@
     <t>PNM MODAL MIKRO</t>
   </si>
   <si>
+    <t>Balindo Manunggal Bersama, PT</t>
+  </si>
+  <si>
     <t>FIF, PT</t>
   </si>
   <si>
-    <t>Balindo Manunggal Bersama, PT</t>
-  </si>
-  <si>
     <t>SEKOLAH POLISI NEGARA</t>
   </si>
   <si>
@@ -850,12 +850,12 @@
     <t>ulamposo@gmail.com</t>
   </si>
   <si>
+    <t>gracekayupa@gmail.com</t>
+  </si>
+  <si>
     <t>dewiputrihilika90@gmail.com</t>
   </si>
   <si>
-    <t>gracekayupa@gmail.com</t>
-  </si>
-  <si>
     <t>kppnpalu651707@yahoo.com</t>
   </si>
   <si>
@@ -1300,6 +1300,12 @@
     <t>26 May 2026, 08:34:35</t>
   </si>
   <si>
+    <t>26 May 2026, 07:30:38</t>
+  </si>
+  <si>
+    <t>26 May 2026, 07:30:35</t>
+  </si>
+  <si>
     <t>31 May 2026, 12:04:58</t>
   </si>
   <si>
@@ -1334,12 +1340,6 @@
   </si>
   <si>
     <t>02 Jun 2026, 11:53:24</t>
-  </si>
-  <si>
-    <t>26 May 2026, 07:30:38</t>
-  </si>
-  <si>
-    <t>26 May 2026, 07:30:35</t>
   </si>
   <si>
     <t>02 Jun 2026, 02:30:55</t>
@@ -3975,7 +3975,7 @@
         <v>364</v>
       </c>
       <c r="F68" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="G68" t="s">
         <v>428</v>
@@ -4001,7 +4001,7 @@
         <v>364</v>
       </c>
       <c r="F69" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="G69" t="s">
         <v>429</v>
@@ -4012,42 +4012,42 @@
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B70" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C70" t="s">
         <v>242</v>
       </c>
       <c r="D70" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E70" t="s">
         <v>364</v>
       </c>
       <c r="F70" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G70" t="s">
         <v>430</v>
       </c>
       <c r="H70">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C71" t="s">
         <v>242</v>
       </c>
       <c r="D71" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E71" t="s">
         <v>364</v>
@@ -4059,99 +4059,99 @@
         <v>431</v>
       </c>
       <c r="H71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B72" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C72" t="s">
         <v>242</v>
       </c>
       <c r="D72" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E72" t="s">
         <v>364</v>
       </c>
       <c r="F72" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G72" t="s">
         <v>432</v>
       </c>
       <c r="H72">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B73" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C73" t="s">
         <v>242</v>
       </c>
       <c r="D73" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E73" t="s">
         <v>364</v>
       </c>
       <c r="F73" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G73" t="s">
         <v>433</v>
       </c>
       <c r="H73">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C74" t="s">
         <v>242</v>
       </c>
       <c r="D74" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E74" t="s">
         <v>364</v>
       </c>
       <c r="F74" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="G74" t="s">
         <v>434</v>
       </c>
       <c r="H74">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B75" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C75" t="s">
         <v>242</v>
       </c>
       <c r="D75" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E75" t="s">
         <v>364</v>
@@ -4163,111 +4163,111 @@
         <v>435</v>
       </c>
       <c r="H75">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C76" t="s">
         <v>242</v>
       </c>
       <c r="D76" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E76" t="s">
         <v>364</v>
       </c>
       <c r="F76" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="G76" t="s">
         <v>436</v>
       </c>
       <c r="H76">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B77" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C77" t="s">
         <v>242</v>
       </c>
       <c r="D77" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E77" t="s">
         <v>364</v>
       </c>
       <c r="F77" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="G77" t="s">
         <v>437</v>
       </c>
       <c r="H77">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B78" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C78" t="s">
         <v>242</v>
       </c>
       <c r="D78" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E78" t="s">
         <v>364</v>
       </c>
       <c r="F78" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G78" t="s">
         <v>438</v>
       </c>
       <c r="H78">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B79" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C79" t="s">
         <v>242</v>
       </c>
       <c r="D79" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E79" t="s">
         <v>364</v>
       </c>
       <c r="F79" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G79" t="s">
         <v>439</v>
       </c>
       <c r="H79">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -4287,13 +4287,13 @@
         <v>364</v>
       </c>
       <c r="F80" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="G80" t="s">
         <v>440</v>
       </c>
       <c r="H80">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -4319,7 +4319,7 @@
         <v>441</v>
       </c>
       <c r="H81">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="82" spans="1:8">

</xml_diff>

<commit_message>
feat: implement data cleaning scripts and update email interaction records
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="168">
   <si>
     <t>code</t>
   </si>
@@ -40,9 +40,15 @@
     <t>order</t>
   </si>
   <si>
+    <t>4b3d4210-f21f-43bc-90cb-365395f8d755</t>
+  </si>
+  <si>
     <t>ec2ea21f-b88a-400a-8f3d-a03562ff60ad</t>
   </si>
   <si>
+    <t>0d4bfa96-7cd5-47d9-b366-e133f6ea27c4</t>
+  </si>
+  <si>
     <t>ca7ed898-5339-4d22-8a89-b89adc186705</t>
   </si>
   <si>
@@ -61,9 +67,81 @@
     <t>bcd04260-5f2a-4732-99e6-e2a415b8b206</t>
   </si>
   <si>
+    <t>19131aed-4f2e-465e-a7f6-9c0d50cbf975</t>
+  </si>
+  <si>
+    <t>5ed2770d-9be6-4fc1-bf70-0d4e10c482c8</t>
+  </si>
+  <si>
+    <t>2b350499-a5b6-45ce-97b3-88359725419f</t>
+  </si>
+  <si>
+    <t>ad55d177-41a1-444e-ae54-8c6807aee095</t>
+  </si>
+  <si>
+    <t>2155505c-bb3d-48ec-ba48-ac98edbdca95</t>
+  </si>
+  <si>
+    <t>abbb91f7-66fb-497f-87e0-235b843068fd</t>
+  </si>
+  <si>
+    <t>64348838-c95b-4e73-8c90-1539e49a8fa6</t>
+  </si>
+  <si>
+    <t>0219fe15-1f5c-4cd7-96f0-734727640195</t>
+  </si>
+  <si>
+    <t>208ebcc6-9881-4752-a982-5d8825476be0</t>
+  </si>
+  <si>
+    <t>df965e5e-d457-436c-a65a-af7726c7ce2b</t>
+  </si>
+  <si>
+    <t>0c6fcc80-9ea0-43b2-8775-cb18edc33d25</t>
+  </si>
+  <si>
+    <t>b2cf42e6-965c-49fa-abac-9af54426d0cc</t>
+  </si>
+  <si>
+    <t>e0e3282e-4685-4ad8-b636-6449ef659410</t>
+  </si>
+  <si>
+    <t>9818074f-7f62-4f6f-8a12-7b9ec153718e</t>
+  </si>
+  <si>
+    <t>2676b7e4-6dca-4e7f-991e-6ae27b0b0c85</t>
+  </si>
+  <si>
+    <t>9b9e29d1-fc1e-4b2d-99d7-838fde85299c</t>
+  </si>
+  <si>
+    <t>e807b2d0-c9e8-4158-bc0a-301bcc232add</t>
+  </si>
+  <si>
+    <t>22df9424-5a77-4276-ab7d-9c4bc6b29108</t>
+  </si>
+  <si>
+    <t>cfb263a1-8db1-46b4-9417-0a2e529be838</t>
+  </si>
+  <si>
+    <t>b58860b3-d502-48de-bf29-ebc5b51b0389</t>
+  </si>
+  <si>
+    <t>cf953441-4548-4748-b059-68c60a1c9312</t>
+  </si>
+  <si>
+    <t>befe39ef-4187-40aa-9e99-fef88d32baa1</t>
+  </si>
+  <si>
+    <t>BPR Syariah  &lt;Agus Supriadi&gt;</t>
+  </si>
+  <si>
     <t>BRI UNIT SALAKAN</t>
   </si>
   <si>
+    <t>BANK DANAMON INDONESIA, PT TBK KCP LUWUK</t>
+  </si>
+  <si>
     <t>BANK PERKREDITAN RAKYAT PALU LOKADANA UTAMA</t>
   </si>
   <si>
@@ -82,12 +160,81 @@
     <t>BRI UNIT BUALEMO</t>
   </si>
   <si>
+    <t>BANK CENTRAL ASIA TBK. CABANG LUWUK</t>
+  </si>
+  <si>
+    <t>BANK PERKREDITAN RAKYAT MITRA NIAGA BANGGAI</t>
+  </si>
+  <si>
+    <t>BANK SULTENG</t>
+  </si>
+  <si>
+    <t>TOTALINDO BANGGAI PERKASA</t>
+  </si>
+  <si>
+    <t>REKAYASA INDUSTRI PT</t>
+  </si>
+  <si>
+    <t>JOB PERTAMINA - MEDCO E&amp;P TOMORI SULAWESI</t>
+  </si>
+  <si>
+    <t>INDONESIA TSINGSHAN STAINLESS STEEL</t>
+  </si>
+  <si>
+    <t>HUA CHIN ALUMINUM  INDONESIA</t>
+  </si>
+  <si>
+    <t>TIGA BAJI, PT</t>
+  </si>
+  <si>
+    <t>MCC15 ENGINEERING AND CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>BROLY NICKEL INDUSTRY</t>
+  </si>
+  <si>
+    <t>BANK SYARIAH INDONESIA, PT</t>
+  </si>
+  <si>
+    <t>HADJI KALLA</t>
+  </si>
+  <si>
+    <t>Detian Coking Indonesia</t>
+  </si>
+  <si>
+    <t>JEMBATAN MAS ENGINEERING</t>
+  </si>
+  <si>
+    <t>INDONESIA RUIPU NICKEL AND CROME ALLOY, PT</t>
+  </si>
+  <si>
+    <t>THE SIXTH CHEMICAL ENGINEERING CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>KENCANA BUMI MINERAL</t>
+  </si>
+  <si>
+    <t>CIPTA MANDIRI MOROWALI</t>
+  </si>
+  <si>
+    <t>INDONESIA GUANG CHING NICKEL AND STAINLESS STEEL INDUSTRY TKA</t>
+  </si>
+  <si>
+    <t>KINRUI NEW ENERGY TECHNOLOGIES  INDONESIA</t>
+  </si>
+  <si>
     <t>OPEN</t>
   </si>
   <si>
+    <t>avatarcrue@gmail.com</t>
+  </si>
+  <si>
     <t>n5164@corp.bri.com</t>
   </si>
   <si>
+    <t>bankdanamon.admin@gmail.com</t>
+  </si>
+  <si>
     <t>kc.luwuk@bprpalulokadanautama.com</t>
   </si>
   <si>
@@ -106,18 +253,102 @@
     <t>nbobs@corp.brico.id</t>
   </si>
   <si>
+    <t>bca_luwuk_pajak@gmail.com</t>
+  </si>
+  <si>
+    <t>toili@mailnesia.com</t>
+  </si>
+  <si>
+    <t>banksulteng.toili@yahoo.com</t>
+  </si>
+  <si>
+    <t>totalindobatbperkasa@gmail.com</t>
+  </si>
+  <si>
+    <t>wandysendjaja@yahoo.com</t>
+  </si>
+  <si>
+    <t>haris.ismail@job-tomori.com</t>
+  </si>
+  <si>
+    <t>secretariat@it-stainlesssteel.com</t>
+  </si>
+  <si>
+    <t>secretariathuachinind@gmail.com</t>
+  </si>
+  <si>
+    <t>aka-hamsah@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>mccmorowali@yahoo.com</t>
+  </si>
+  <si>
+    <t>hengjayasite@yahoo.com</t>
+  </si>
+  <si>
+    <t>sapriliya@bsm.co.id</t>
+  </si>
+  <si>
+    <t>nur.salam.coning@kallagroup.co.id</t>
+  </si>
+  <si>
+    <t>secretariat@detiancoking-ind.com</t>
+  </si>
+  <si>
+    <t>jembatanmas579@yahoo.com</t>
+  </si>
+  <si>
+    <t>smaalkhairatkolono@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>sobeh@ppc-adulsory.com</t>
+  </si>
+  <si>
+    <t>acctaxkbm@yahoo.com</t>
+  </si>
+  <si>
+    <t>kc.morowali@bprpalulokadanautama.com</t>
+  </si>
+  <si>
+    <t>ciptamandiri@yahoo.com</t>
+  </si>
+  <si>
+    <t>rukun@bd.em.com</t>
+  </si>
+  <si>
+    <t>secretariatkinrui@gmail.com</t>
+  </si>
+  <si>
+    <t>Permanent_fail</t>
+  </si>
+  <si>
     <t>Bounced</t>
   </si>
   <si>
     <t>Queued</t>
   </si>
   <si>
+    <t>09 Jun 2026, 11:19:15</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:35:03</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:35:02</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 09:36:45</t>
   </si>
   <si>
     <t>02 Jun 2026, 09:36:44</t>
   </si>
   <si>
+    <t>09 Jun 2026, 11:00:04</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:07:49</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 07:38:30</t>
   </si>
   <si>
@@ -149,6 +380,144 @@
   </si>
   <si>
     <t>02 Jun 2026, 06:50:12</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:02:57</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:34:59</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:34:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:11:11</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:10:03</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 00:12:21</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 00:11:48</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:57:24</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:57:20</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:05:04</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:49:00</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:48:57</t>
+  </si>
+  <si>
+    <t>18 May 2026, 12:37:49</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 09:53:25</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:51:24</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:23:23</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:57:25</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 22:48:15</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:04:32</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:47:52</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:55:13</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:52:30</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:00:02</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:38</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:57:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:49:47</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:57:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:45:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:43:12</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:08:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:11:39</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:16</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:22:02</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:06:55</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:52:15</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:52:11</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:55:41</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:55:37</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:29:20</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:28:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:54:53</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:54:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:59:29</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:59:25</t>
   </si>
 </sst>
 </file>
@@ -506,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -540,22 +909,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>104</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -566,22 +935,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -589,28 +958,28 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -618,51 +987,51 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>102</v>
       </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -670,100 +1039,100 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>109</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
-        <v>39</v>
+        <v>110</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
-        <v>40</v>
+        <v>111</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -771,25 +1140,25 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="H11">
         <v>2</v>
@@ -797,25 +1166,25 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="E12" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
+        <v>113</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -823,25 +1192,25 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="G13" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -849,25 +1218,25 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>102</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -875,27 +1244,1483 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G15" t="s">
+        <v>116</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" t="s">
+        <v>102</v>
+      </c>
+      <c r="G16" t="s">
+        <v>117</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" t="s">
+        <v>118</v>
+      </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" t="s">
+        <v>119</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" t="s">
+        <v>121</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" t="s">
+        <v>121</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
+        <v>69</v>
+      </c>
+      <c r="D22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" t="s">
+        <v>101</v>
+      </c>
+      <c r="G22" t="s">
+        <v>122</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" t="s">
+        <v>101</v>
+      </c>
+      <c r="F23" t="s">
+        <v>102</v>
+      </c>
+      <c r="G23" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" t="s">
+        <v>101</v>
+      </c>
+      <c r="F24" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" t="s">
+        <v>101</v>
+      </c>
+      <c r="F25" t="s">
+        <v>101</v>
+      </c>
+      <c r="G25" t="s">
+        <v>125</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" t="s">
+        <v>101</v>
+      </c>
+      <c r="F26" t="s">
+        <v>101</v>
+      </c>
+      <c r="G26" t="s">
+        <v>126</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" t="s">
+        <v>69</v>
+      </c>
+      <c r="D27" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" t="s">
+        <v>127</v>
+      </c>
+      <c r="H27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" t="s">
+        <v>103</v>
+      </c>
+      <c r="G28" t="s">
+        <v>128</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" t="s">
+        <v>102</v>
+      </c>
+      <c r="F29" t="s">
+        <v>102</v>
+      </c>
+      <c r="G29" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" t="s">
+        <v>103</v>
+      </c>
+      <c r="G30" t="s">
+        <v>130</v>
+      </c>
+      <c r="H30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" t="s">
         <v>21</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" t="s">
+        <v>101</v>
+      </c>
+      <c r="G31" t="s">
+        <v>131</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B32" t="s">
+        <v>52</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32" t="s">
+        <v>101</v>
+      </c>
+      <c r="F32" t="s">
+        <v>102</v>
+      </c>
+      <c r="G32" t="s">
+        <v>132</v>
+      </c>
+      <c r="H32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33" t="s">
+        <v>101</v>
+      </c>
+      <c r="F33" t="s">
+        <v>103</v>
+      </c>
+      <c r="G33" t="s">
+        <v>133</v>
+      </c>
+      <c r="H33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
         <v>22</v>
       </c>
-      <c r="D15" t="s">
+      <c r="B34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" t="s">
+        <v>84</v>
+      </c>
+      <c r="E34" t="s">
+        <v>101</v>
+      </c>
+      <c r="F34" t="s">
+        <v>101</v>
+      </c>
+      <c r="G34" t="s">
+        <v>134</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" t="s">
+        <v>101</v>
+      </c>
+      <c r="F35" t="s">
+        <v>101</v>
+      </c>
+      <c r="G35" t="s">
+        <v>135</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36" t="s">
+        <v>84</v>
+      </c>
+      <c r="E36" t="s">
+        <v>101</v>
+      </c>
+      <c r="F36" t="s">
+        <v>101</v>
+      </c>
+      <c r="G36" t="s">
+        <v>136</v>
+      </c>
+      <c r="H36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
+        <v>23</v>
+      </c>
+      <c r="B37" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" t="s">
+        <v>102</v>
+      </c>
+      <c r="F37" t="s">
+        <v>103</v>
+      </c>
+      <c r="G37" t="s">
+        <v>137</v>
+      </c>
+      <c r="H37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C38" t="s">
+        <v>69</v>
+      </c>
+      <c r="D38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E38" t="s">
+        <v>102</v>
+      </c>
+      <c r="F38" t="s">
+        <v>102</v>
+      </c>
+      <c r="G38" t="s">
+        <v>137</v>
+      </c>
+      <c r="H38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" t="s">
+        <v>69</v>
+      </c>
+      <c r="D39" t="s">
+        <v>86</v>
+      </c>
+      <c r="E39" t="s">
+        <v>101</v>
+      </c>
+      <c r="F39" t="s">
+        <v>101</v>
+      </c>
+      <c r="G39" t="s">
+        <v>138</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" t="s">
+        <v>69</v>
+      </c>
+      <c r="D40" t="s">
+        <v>86</v>
+      </c>
+      <c r="E40" t="s">
+        <v>101</v>
+      </c>
+      <c r="F40" t="s">
+        <v>102</v>
+      </c>
+      <c r="G40" t="s">
+        <v>139</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" t="s">
+        <v>86</v>
+      </c>
+      <c r="E41" t="s">
+        <v>101</v>
+      </c>
+      <c r="F41" t="s">
+        <v>103</v>
+      </c>
+      <c r="G41" t="s">
+        <v>139</v>
+      </c>
+      <c r="H41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" t="s">
+        <v>69</v>
+      </c>
+      <c r="D42" t="s">
+        <v>87</v>
+      </c>
+      <c r="E42" t="s">
+        <v>101</v>
+      </c>
+      <c r="F42" t="s">
+        <v>101</v>
+      </c>
+      <c r="G42" t="s">
+        <v>140</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43" t="s">
+        <v>69</v>
+      </c>
+      <c r="D43" t="s">
+        <v>87</v>
+      </c>
+      <c r="E43" t="s">
+        <v>101</v>
+      </c>
+      <c r="F43" t="s">
+        <v>102</v>
+      </c>
+      <c r="G43" t="s">
+        <v>141</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" t="s">
+        <v>69</v>
+      </c>
+      <c r="D44" t="s">
+        <v>87</v>
+      </c>
+      <c r="E44" t="s">
+        <v>101</v>
+      </c>
+      <c r="F44" t="s">
+        <v>103</v>
+      </c>
+      <c r="G44" t="s">
+        <v>141</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" t="s">
+        <v>69</v>
+      </c>
+      <c r="D45" t="s">
+        <v>88</v>
+      </c>
+      <c r="E45" t="s">
+        <v>102</v>
+      </c>
+      <c r="F45" t="s">
+        <v>102</v>
+      </c>
+      <c r="G45" t="s">
+        <v>142</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" t="s">
+        <v>69</v>
+      </c>
+      <c r="D46" t="s">
+        <v>88</v>
+      </c>
+      <c r="E46" t="s">
+        <v>102</v>
+      </c>
+      <c r="F46" t="s">
+        <v>103</v>
+      </c>
+      <c r="G46" t="s">
+        <v>143</v>
+      </c>
+      <c r="H46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
+        <v>27</v>
+      </c>
+      <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>69</v>
+      </c>
+      <c r="D47" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" t="s">
+        <v>101</v>
+      </c>
+      <c r="F47" t="s">
+        <v>101</v>
+      </c>
+      <c r="G47" t="s">
+        <v>144</v>
+      </c>
+      <c r="H47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48" t="s">
+        <v>58</v>
+      </c>
+      <c r="C48" t="s">
+        <v>69</v>
+      </c>
+      <c r="D48" t="s">
+        <v>89</v>
+      </c>
+      <c r="E48" t="s">
+        <v>101</v>
+      </c>
+      <c r="F48" t="s">
+        <v>102</v>
+      </c>
+      <c r="G48" t="s">
+        <v>145</v>
+      </c>
+      <c r="H48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" t="s">
+        <v>27</v>
+      </c>
+      <c r="B49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" t="s">
+        <v>89</v>
+      </c>
+      <c r="E49" t="s">
+        <v>101</v>
+      </c>
+      <c r="F49" t="s">
+        <v>103</v>
+      </c>
+      <c r="G49" t="s">
+        <v>146</v>
+      </c>
+      <c r="H49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" t="s">
+        <v>59</v>
+      </c>
+      <c r="C50" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E50" t="s">
+        <v>102</v>
+      </c>
+      <c r="F50" t="s">
+        <v>102</v>
+      </c>
+      <c r="G50" t="s">
+        <v>147</v>
+      </c>
+      <c r="H50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" t="s">
+        <v>102</v>
+      </c>
+      <c r="F51" t="s">
+        <v>103</v>
+      </c>
+      <c r="G51" t="s">
+        <v>148</v>
+      </c>
+      <c r="H51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" t="s">
         <v>29</v>
       </c>
-      <c r="E15" t="s">
+      <c r="B52" t="s">
+        <v>60</v>
+      </c>
+      <c r="C52" t="s">
+        <v>69</v>
+      </c>
+      <c r="D52" t="s">
+        <v>91</v>
+      </c>
+      <c r="E52" t="s">
+        <v>101</v>
+      </c>
+      <c r="F52" t="s">
+        <v>101</v>
+      </c>
+      <c r="G52" t="s">
+        <v>149</v>
+      </c>
+      <c r="H52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" t="s">
         <v>30</v>
       </c>
-      <c r="F15" t="s">
+      <c r="B53" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" t="s">
+        <v>92</v>
+      </c>
+      <c r="E53" t="s">
+        <v>102</v>
+      </c>
+      <c r="F53" t="s">
+        <v>102</v>
+      </c>
+      <c r="G53" t="s">
+        <v>150</v>
+      </c>
+      <c r="H53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" t="s">
         <v>30</v>
       </c>
-      <c r="G15" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15">
+      <c r="B54" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" t="s">
+        <v>69</v>
+      </c>
+      <c r="D54" t="s">
+        <v>92</v>
+      </c>
+      <c r="E54" t="s">
+        <v>102</v>
+      </c>
+      <c r="F54" t="s">
+        <v>103</v>
+      </c>
+      <c r="G54" t="s">
+        <v>151</v>
+      </c>
+      <c r="H54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" t="s">
+        <v>31</v>
+      </c>
+      <c r="B55" t="s">
+        <v>62</v>
+      </c>
+      <c r="C55" t="s">
+        <v>69</v>
+      </c>
+      <c r="D55" t="s">
+        <v>93</v>
+      </c>
+      <c r="E55" t="s">
+        <v>101</v>
+      </c>
+      <c r="F55" t="s">
+        <v>101</v>
+      </c>
+      <c r="G55" t="s">
+        <v>152</v>
+      </c>
+      <c r="H55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" t="s">
+        <v>62</v>
+      </c>
+      <c r="C56" t="s">
+        <v>69</v>
+      </c>
+      <c r="D56" t="s">
+        <v>93</v>
+      </c>
+      <c r="E56" t="s">
+        <v>101</v>
+      </c>
+      <c r="F56" t="s">
+        <v>101</v>
+      </c>
+      <c r="G56" t="s">
+        <v>153</v>
+      </c>
+      <c r="H56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" t="s">
+        <v>32</v>
+      </c>
+      <c r="B57" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" t="s">
+        <v>69</v>
+      </c>
+      <c r="D57" t="s">
+        <v>94</v>
+      </c>
+      <c r="E57" t="s">
+        <v>102</v>
+      </c>
+      <c r="F57" t="s">
+        <v>102</v>
+      </c>
+      <c r="G57" t="s">
+        <v>154</v>
+      </c>
+      <c r="H57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" t="s">
+        <v>32</v>
+      </c>
+      <c r="B58" t="s">
+        <v>63</v>
+      </c>
+      <c r="C58" t="s">
+        <v>69</v>
+      </c>
+      <c r="D58" t="s">
+        <v>94</v>
+      </c>
+      <c r="E58" t="s">
+        <v>102</v>
+      </c>
+      <c r="F58" t="s">
+        <v>103</v>
+      </c>
+      <c r="G58" t="s">
+        <v>155</v>
+      </c>
+      <c r="H58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" t="s">
+        <v>33</v>
+      </c>
+      <c r="B59" t="s">
+        <v>64</v>
+      </c>
+      <c r="C59" t="s">
+        <v>69</v>
+      </c>
+      <c r="D59" t="s">
+        <v>95</v>
+      </c>
+      <c r="E59" t="s">
+        <v>102</v>
+      </c>
+      <c r="F59" t="s">
+        <v>103</v>
+      </c>
+      <c r="G59" t="s">
+        <v>156</v>
+      </c>
+      <c r="H59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" t="s">
+        <v>33</v>
+      </c>
+      <c r="B60" t="s">
+        <v>64</v>
+      </c>
+      <c r="C60" t="s">
+        <v>69</v>
+      </c>
+      <c r="D60" t="s">
+        <v>95</v>
+      </c>
+      <c r="E60" t="s">
+        <v>102</v>
+      </c>
+      <c r="F60" t="s">
+        <v>102</v>
+      </c>
+      <c r="G60" t="s">
+        <v>156</v>
+      </c>
+      <c r="H60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" t="s">
+        <v>34</v>
+      </c>
+      <c r="B61" t="s">
+        <v>65</v>
+      </c>
+      <c r="C61" t="s">
+        <v>69</v>
+      </c>
+      <c r="D61" t="s">
+        <v>96</v>
+      </c>
+      <c r="E61" t="s">
+        <v>101</v>
+      </c>
+      <c r="F61" t="s">
+        <v>101</v>
+      </c>
+      <c r="G61" t="s">
+        <v>157</v>
+      </c>
+      <c r="H61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" t="s">
+        <v>34</v>
+      </c>
+      <c r="B62" t="s">
+        <v>65</v>
+      </c>
+      <c r="C62" t="s">
+        <v>69</v>
+      </c>
+      <c r="D62" t="s">
+        <v>96</v>
+      </c>
+      <c r="E62" t="s">
+        <v>101</v>
+      </c>
+      <c r="F62" t="s">
+        <v>102</v>
+      </c>
+      <c r="G62" t="s">
+        <v>158</v>
+      </c>
+      <c r="H62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" t="s">
+        <v>34</v>
+      </c>
+      <c r="B63" t="s">
+        <v>65</v>
+      </c>
+      <c r="C63" t="s">
+        <v>69</v>
+      </c>
+      <c r="D63" t="s">
+        <v>96</v>
+      </c>
+      <c r="E63" t="s">
+        <v>101</v>
+      </c>
+      <c r="F63" t="s">
+        <v>103</v>
+      </c>
+      <c r="G63" t="s">
+        <v>159</v>
+      </c>
+      <c r="H63">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" t="s">
+        <v>35</v>
+      </c>
+      <c r="B64" t="s">
+        <v>42</v>
+      </c>
+      <c r="C64" t="s">
+        <v>69</v>
+      </c>
+      <c r="D64" t="s">
+        <v>97</v>
+      </c>
+      <c r="E64" t="s">
+        <v>102</v>
+      </c>
+      <c r="F64" t="s">
+        <v>102</v>
+      </c>
+      <c r="G64" t="s">
+        <v>160</v>
+      </c>
+      <c r="H64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>35</v>
+      </c>
+      <c r="B65" t="s">
+        <v>42</v>
+      </c>
+      <c r="C65" t="s">
+        <v>69</v>
+      </c>
+      <c r="D65" t="s">
+        <v>97</v>
+      </c>
+      <c r="E65" t="s">
+        <v>102</v>
+      </c>
+      <c r="F65" t="s">
+        <v>103</v>
+      </c>
+      <c r="G65" t="s">
+        <v>161</v>
+      </c>
+      <c r="H65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>36</v>
+      </c>
+      <c r="B66" t="s">
+        <v>66</v>
+      </c>
+      <c r="C66" t="s">
+        <v>69</v>
+      </c>
+      <c r="D66" t="s">
+        <v>98</v>
+      </c>
+      <c r="E66" t="s">
+        <v>102</v>
+      </c>
+      <c r="F66" t="s">
+        <v>102</v>
+      </c>
+      <c r="G66" t="s">
+        <v>162</v>
+      </c>
+      <c r="H66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" t="s">
+        <v>36</v>
+      </c>
+      <c r="B67" t="s">
+        <v>66</v>
+      </c>
+      <c r="C67" t="s">
+        <v>69</v>
+      </c>
+      <c r="D67" t="s">
+        <v>98</v>
+      </c>
+      <c r="E67" t="s">
+        <v>102</v>
+      </c>
+      <c r="F67" t="s">
+        <v>103</v>
+      </c>
+      <c r="G67" t="s">
+        <v>163</v>
+      </c>
+      <c r="H67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" t="s">
+        <v>37</v>
+      </c>
+      <c r="B68" t="s">
+        <v>67</v>
+      </c>
+      <c r="C68" t="s">
+        <v>69</v>
+      </c>
+      <c r="D68" t="s">
+        <v>99</v>
+      </c>
+      <c r="E68" t="s">
+        <v>102</v>
+      </c>
+      <c r="F68" t="s">
+        <v>102</v>
+      </c>
+      <c r="G68" t="s">
+        <v>164</v>
+      </c>
+      <c r="H68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" t="s">
+        <v>37</v>
+      </c>
+      <c r="B69" t="s">
+        <v>67</v>
+      </c>
+      <c r="C69" t="s">
+        <v>69</v>
+      </c>
+      <c r="D69" t="s">
+        <v>99</v>
+      </c>
+      <c r="E69" t="s">
+        <v>102</v>
+      </c>
+      <c r="F69" t="s">
+        <v>103</v>
+      </c>
+      <c r="G69" t="s">
+        <v>165</v>
+      </c>
+      <c r="H69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" t="s">
+        <v>38</v>
+      </c>
+      <c r="B70" t="s">
+        <v>68</v>
+      </c>
+      <c r="C70" t="s">
+        <v>69</v>
+      </c>
+      <c r="D70" t="s">
+        <v>100</v>
+      </c>
+      <c r="E70" t="s">
+        <v>102</v>
+      </c>
+      <c r="F70" t="s">
+        <v>102</v>
+      </c>
+      <c r="G70" t="s">
+        <v>166</v>
+      </c>
+      <c r="H70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" t="s">
+        <v>38</v>
+      </c>
+      <c r="B71" t="s">
+        <v>68</v>
+      </c>
+      <c r="C71" t="s">
+        <v>69</v>
+      </c>
+      <c r="D71" t="s">
+        <v>100</v>
+      </c>
+      <c r="E71" t="s">
+        <v>102</v>
+      </c>
+      <c r="F71" t="s">
+        <v>103</v>
+      </c>
+      <c r="G71" t="s">
+        <v>167</v>
+      </c>
+      <c r="H71">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add new email cleaning script and initialize Playwright Chrome profile directory mash salah yg ub assign
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="146">
   <si>
     <t>code</t>
   </si>
@@ -88,7 +88,37 @@
     <t>abbb91f7-66fb-497f-87e0-235b843068fd</t>
   </si>
   <si>
-    <t>BPR SYARIAH KHAIRAN INTI  &lt;AGUS SUPRIADI&gt;</t>
+    <t>64348838-c95b-4e73-8c90-1539e49a8fa6</t>
+  </si>
+  <si>
+    <t>0219fe15-1f5c-4cd7-96f0-734727640195</t>
+  </si>
+  <si>
+    <t>208ebcc6-9881-4752-a982-5d8825476be0</t>
+  </si>
+  <si>
+    <t>df965e5e-d457-436c-a65a-af7726c7ce2b</t>
+  </si>
+  <si>
+    <t>0c6fcc80-9ea0-43b2-8775-cb18edc33d25</t>
+  </si>
+  <si>
+    <t>b2cf42e6-965c-49fa-abac-9af54426d0cc</t>
+  </si>
+  <si>
+    <t>e0e3282e-4685-4ad8-b636-6449ef659410</t>
+  </si>
+  <si>
+    <t>9818074f-7f62-4f6f-8a12-7b9ec153718e</t>
+  </si>
+  <si>
+    <t>2676b7e4-6dca-4e7f-991e-6ae27b0b0c85</t>
+  </si>
+  <si>
+    <t>9b9e29d1-fc1e-4b2d-99d7-838fde85299c</t>
+  </si>
+  <si>
+    <t>PTBPRSYARIAHKHAIRANINTIAMANAH</t>
   </si>
   <si>
     <t>BPR MODERN EXPRESS PT</t>
@@ -136,12 +166,42 @@
     <t>JOB PERTAMINA - MEDCO E&amp;P TOMORI SULAWESI</t>
   </si>
   <si>
+    <t>INDONESIA TSINGSHAN STAINLESS STEEL</t>
+  </si>
+  <si>
+    <t>HUA CHIN ALUMINUM  INDONESIA</t>
+  </si>
+  <si>
+    <t>TIGA BAJI, PT</t>
+  </si>
+  <si>
+    <t>MCC15 ENGINEERING AND CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>BROLY NICKEL INDUSTRY</t>
+  </si>
+  <si>
+    <t>BANK SYARIAH INDONESIA, PT</t>
+  </si>
+  <si>
+    <t>HADJI KALLA</t>
+  </si>
+  <si>
+    <t>Detian Coking Indonesia</t>
+  </si>
+  <si>
+    <t>JEMBATAN MAS ENGINEERING</t>
+  </si>
+  <si>
+    <t>INDONESIA RUIPU NICKEL AND CROME ALLOY, PT</t>
+  </si>
+  <si>
+    <t>SUBMITTED RESPONDENT</t>
+  </si>
+  <si>
     <t>DRAFT</t>
   </si>
   <si>
-    <t>SUBMITTED RESPONDENT</t>
-  </si>
-  <si>
     <t>OPEN</t>
   </si>
   <si>
@@ -193,6 +253,36 @@
     <t>haris.ismail@job-tomori.com</t>
   </si>
   <si>
+    <t>secretariat@it-stainlesssteel.com</t>
+  </si>
+  <si>
+    <t>secretariathuachinind@gmail.com</t>
+  </si>
+  <si>
+    <t>aka-hamsah@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>mccmorowali@yahoo.com</t>
+  </si>
+  <si>
+    <t>hengjayasite@yahoo.com</t>
+  </si>
+  <si>
+    <t>sapriliya@bsm.co.id</t>
+  </si>
+  <si>
+    <t>nur.salam.coning@kallagroup.co.id</t>
+  </si>
+  <si>
+    <t>secretariat@detiancoking-ind.com</t>
+  </si>
+  <si>
+    <t>jembatanmas579@yahoo.com</t>
+  </si>
+  <si>
+    <t>smaalkhairatkolono@yahoo.co.id</t>
+  </si>
+  <si>
     <t>Permanent_fail</t>
   </si>
   <si>
@@ -202,6 +292,9 @@
     <t>Queued</t>
   </si>
   <si>
+    <t>11 Jun 2026, 14:00:36</t>
+  </si>
+  <si>
     <t>09 Jun 2026, 11:19:15</t>
   </si>
   <si>
@@ -302,6 +395,63 @@
   </si>
   <si>
     <t>02 Jun 2026, 05:51:24</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:23:23</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:57:25</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 22:48:15</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:04:32</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:47:52</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:55:13</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:52:30</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:00:02</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:38</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:57:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:49:47</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:57:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:45:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:43:12</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:08:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:11:39</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:16</t>
   </si>
 </sst>
 </file>
@@ -659,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -693,22 +843,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -719,22 +869,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="G3" t="s">
-        <v>63</v>
+        <v>93</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -745,22 +895,22 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F4" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G4" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -768,51 +918,51 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="G5" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -823,51 +973,51 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="G8" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -875,25 +1025,25 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -901,51 +1051,51 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G11" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -953,51 +1103,51 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F13" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1005,51 +1155,51 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F14" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G15" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1057,51 +1207,51 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G16" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G17" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1109,51 +1259,51 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G18" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G19" t="s">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1161,51 +1311,51 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F20" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G20" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="G21" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1213,51 +1363,51 @@
         <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="E22" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F22" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G22" t="s">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D23" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="E23" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F23" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="G23" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1265,25 +1415,25 @@
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D24" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F24" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G24" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1291,74 +1441,74 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D25" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E25" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F25" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G25" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="E26" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F26" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="G26" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="E27" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F27" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G27" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="H27">
         <v>1</v>
@@ -1369,25 +1519,25 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C28" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D28" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="E28" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F28" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1395,51 +1545,51 @@
         <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C29" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F29" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G29" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C30" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E30" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="F30" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G30" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1447,51 +1597,51 @@
         <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F31" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G31" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="H31">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D32" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="E32" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F32" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="G32" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1499,25 +1649,25 @@
         <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C33" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E33" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F33" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G33" t="s">
-        <v>91</v>
+        <v>121</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1525,51 +1675,51 @@
         <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C34" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D34" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E34" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F34" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G34" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="H34">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="E35" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F35" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="G35" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1577,25 +1727,25 @@
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C36" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D36" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="F36" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G36" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1603,25 +1753,623 @@
         <v>23</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D37" t="s">
+        <v>78</v>
+      </c>
+      <c r="E37" t="s">
+        <v>89</v>
+      </c>
+      <c r="F37" t="s">
+        <v>89</v>
+      </c>
+      <c r="G37" t="s">
+        <v>125</v>
+      </c>
+      <c r="H37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E38" t="s">
+        <v>89</v>
+      </c>
+      <c r="F38" t="s">
+        <v>89</v>
+      </c>
+      <c r="G38" t="s">
+        <v>126</v>
+      </c>
+      <c r="H38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" t="s">
+        <v>62</v>
+      </c>
+      <c r="D39" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39" t="s">
+        <v>90</v>
+      </c>
+      <c r="F39" t="s">
+        <v>91</v>
+      </c>
+      <c r="G39" t="s">
+        <v>127</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" t="s">
+        <v>90</v>
+      </c>
+      <c r="F40" t="s">
+        <v>90</v>
+      </c>
+      <c r="G40" t="s">
+        <v>127</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
+        <v>51</v>
+      </c>
+      <c r="C41" t="s">
+        <v>62</v>
+      </c>
+      <c r="D41" t="s">
+        <v>80</v>
+      </c>
+      <c r="E41" t="s">
+        <v>89</v>
+      </c>
+      <c r="F41" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" t="s">
+        <v>128</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42" t="s">
+        <v>62</v>
+      </c>
+      <c r="D42" t="s">
+        <v>80</v>
+      </c>
+      <c r="E42" t="s">
+        <v>89</v>
+      </c>
+      <c r="F42" t="s">
+        <v>90</v>
+      </c>
+      <c r="G42" t="s">
+        <v>129</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>51</v>
+      </c>
+      <c r="C43" t="s">
+        <v>62</v>
+      </c>
+      <c r="D43" t="s">
+        <v>80</v>
+      </c>
+      <c r="E43" t="s">
+        <v>89</v>
+      </c>
+      <c r="F43" t="s">
+        <v>91</v>
+      </c>
+      <c r="G43" t="s">
+        <v>129</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" t="s">
+        <v>81</v>
+      </c>
+      <c r="E44" t="s">
+        <v>89</v>
+      </c>
+      <c r="F44" t="s">
+        <v>89</v>
+      </c>
+      <c r="G44" t="s">
+        <v>130</v>
+      </c>
+      <c r="H44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" t="s">
+        <v>62</v>
+      </c>
+      <c r="D45" t="s">
+        <v>81</v>
+      </c>
+      <c r="E45" t="s">
+        <v>89</v>
+      </c>
+      <c r="F45" t="s">
+        <v>90</v>
+      </c>
+      <c r="G45" t="s">
+        <v>131</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" t="s">
+        <v>52</v>
+      </c>
+      <c r="C46" t="s">
+        <v>62</v>
+      </c>
+      <c r="D46" t="s">
+        <v>81</v>
+      </c>
+      <c r="E46" t="s">
+        <v>89</v>
+      </c>
+      <c r="F46" t="s">
+        <v>91</v>
+      </c>
+      <c r="G46" t="s">
+        <v>131</v>
+      </c>
+      <c r="H46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
+        <v>27</v>
+      </c>
+      <c r="B47" t="s">
+        <v>53</v>
+      </c>
+      <c r="C47" t="s">
+        <v>62</v>
+      </c>
+      <c r="D47" t="s">
+        <v>82</v>
+      </c>
+      <c r="E47" t="s">
+        <v>90</v>
+      </c>
+      <c r="F47" t="s">
+        <v>90</v>
+      </c>
+      <c r="G47" t="s">
+        <v>132</v>
+      </c>
+      <c r="H47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" t="s">
+        <v>62</v>
+      </c>
+      <c r="D48" t="s">
+        <v>82</v>
+      </c>
+      <c r="E48" t="s">
+        <v>90</v>
+      </c>
+      <c r="F48" t="s">
+        <v>91</v>
+      </c>
+      <c r="G48" t="s">
+        <v>133</v>
+      </c>
+      <c r="H48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" t="s">
+        <v>62</v>
+      </c>
+      <c r="D49" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" t="s">
+        <v>89</v>
+      </c>
+      <c r="F49" t="s">
+        <v>89</v>
+      </c>
+      <c r="G49" t="s">
+        <v>134</v>
+      </c>
+      <c r="H49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" t="s">
+        <v>62</v>
+      </c>
+      <c r="D50" t="s">
+        <v>83</v>
+      </c>
+      <c r="E50" t="s">
+        <v>89</v>
+      </c>
+      <c r="F50" t="s">
+        <v>90</v>
+      </c>
+      <c r="G50" t="s">
+        <v>135</v>
+      </c>
+      <c r="H50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" t="s">
+        <v>54</v>
+      </c>
+      <c r="C51" t="s">
+        <v>62</v>
+      </c>
+      <c r="D51" t="s">
+        <v>83</v>
+      </c>
+      <c r="E51" t="s">
+        <v>89</v>
+      </c>
+      <c r="F51" t="s">
+        <v>91</v>
+      </c>
+      <c r="G51" t="s">
+        <v>136</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" t="s">
+        <v>29</v>
+      </c>
+      <c r="B52" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" t="s">
+        <v>62</v>
+      </c>
+      <c r="D52" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52" t="s">
+        <v>90</v>
+      </c>
+      <c r="F52" t="s">
+        <v>90</v>
+      </c>
+      <c r="G52" t="s">
+        <v>137</v>
+      </c>
+      <c r="H52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" t="s">
+        <v>29</v>
+      </c>
+      <c r="B53" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" t="s">
+        <v>62</v>
+      </c>
+      <c r="D53" t="s">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>90</v>
+      </c>
+      <c r="F53" t="s">
+        <v>91</v>
+      </c>
+      <c r="G53" t="s">
+        <v>138</v>
+      </c>
+      <c r="H53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" t="s">
+        <v>30</v>
+      </c>
+      <c r="B54" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D54" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" t="s">
+        <v>89</v>
+      </c>
+      <c r="F54" t="s">
+        <v>89</v>
+      </c>
+      <c r="G54" t="s">
+        <v>139</v>
+      </c>
+      <c r="H54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" t="s">
+        <v>31</v>
+      </c>
+      <c r="B55" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55" t="s">
+        <v>62</v>
+      </c>
+      <c r="D55" t="s">
+        <v>86</v>
+      </c>
+      <c r="E55" t="s">
+        <v>90</v>
+      </c>
+      <c r="F55" t="s">
+        <v>90</v>
+      </c>
+      <c r="G55" t="s">
+        <v>140</v>
+      </c>
+      <c r="H55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" t="s">
+        <v>57</v>
+      </c>
+      <c r="C56" t="s">
+        <v>62</v>
+      </c>
+      <c r="D56" t="s">
+        <v>86</v>
+      </c>
+      <c r="E56" t="s">
+        <v>90</v>
+      </c>
+      <c r="F56" t="s">
+        <v>91</v>
+      </c>
+      <c r="G56" t="s">
+        <v>141</v>
+      </c>
+      <c r="H56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" t="s">
+        <v>32</v>
+      </c>
+      <c r="B57" t="s">
         <v>58</v>
       </c>
-      <c r="E37" t="s">
+      <c r="C57" t="s">
+        <v>62</v>
+      </c>
+      <c r="D57" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" t="s">
+        <v>89</v>
+      </c>
+      <c r="F57" t="s">
+        <v>89</v>
+      </c>
+      <c r="G57" t="s">
+        <v>142</v>
+      </c>
+      <c r="H57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" t="s">
+        <v>32</v>
+      </c>
+      <c r="B58" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58" t="s">
+        <v>62</v>
+      </c>
+      <c r="D58" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58" t="s">
+        <v>89</v>
+      </c>
+      <c r="F58" t="s">
+        <v>89</v>
+      </c>
+      <c r="G58" t="s">
+        <v>143</v>
+      </c>
+      <c r="H58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" t="s">
+        <v>33</v>
+      </c>
+      <c r="B59" t="s">
         <v>59</v>
       </c>
-      <c r="F37" t="s">
+      <c r="C59" t="s">
+        <v>62</v>
+      </c>
+      <c r="D59" t="s">
+        <v>88</v>
+      </c>
+      <c r="E59" t="s">
+        <v>90</v>
+      </c>
+      <c r="F59" t="s">
+        <v>90</v>
+      </c>
+      <c r="G59" t="s">
+        <v>144</v>
+      </c>
+      <c r="H59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" t="s">
+        <v>33</v>
+      </c>
+      <c r="B60" t="s">
         <v>59</v>
       </c>
-      <c r="G37" t="s">
-        <v>95</v>
-      </c>
-      <c r="H37">
-        <v>3</v>
+      <c r="C60" t="s">
+        <v>62</v>
+      </c>
+      <c r="D60" t="s">
+        <v>88</v>
+      </c>
+      <c r="E60" t="s">
+        <v>90</v>
+      </c>
+      <c r="F60" t="s">
+        <v>91</v>
+      </c>
+      <c r="G60" t="s">
+        <v>145</v>
+      </c>
+      <c r="H60">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update scraping scripts and session data while cleaning up browser profile cache files
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="64">
   <si>
     <t>code</t>
   </si>
@@ -49,6 +49,27 @@
     <t>ec2ea21f-b88a-400a-8f3d-a03562ff60ad</t>
   </si>
   <si>
+    <t>0d4bfa96-7cd5-47d9-b366-e133f6ea27c4</t>
+  </si>
+  <si>
+    <t>ca7ed898-5339-4d22-8a89-b89adc186705</t>
+  </si>
+  <si>
+    <t>c5b60633-13fc-4352-a09f-e6b11e93fe60</t>
+  </si>
+  <si>
+    <t>87ab3e43-e1be-4b02-af1e-14720ebfb03f</t>
+  </si>
+  <si>
+    <t>941bb532-7c5e-4c33-baca-ee0b2d06fb62</t>
+  </si>
+  <si>
+    <t>96d663ec-f298-4560-9b84-996b8de92249</t>
+  </si>
+  <si>
+    <t>bcd04260-5f2a-4732-99e6-e2a415b8b206</t>
+  </si>
+  <si>
     <t>PTBPRSYARIAHKHAIRANINTIAMANAH</t>
   </si>
   <si>
@@ -58,12 +79,36 @@
     <t>BRI UNIT SALAKAN</t>
   </si>
   <si>
+    <t>BANK DANAMON INDONESIA, PT TBK KCP LUWUK</t>
+  </si>
+  <si>
+    <t>BANK PERKREDITAN RAKYAT PALU LOKADANA UTAMA</t>
+  </si>
+  <si>
+    <t>BANK SAMPAH INDUK BERLIAN</t>
+  </si>
+  <si>
+    <t>CAHAYA BARU SENTOSA</t>
+  </si>
+  <si>
+    <t>ALL BERKEMBANG BERSAMA</t>
+  </si>
+  <si>
+    <t>TRAKINDO UTAMA, PT</t>
+  </si>
+  <si>
+    <t>BRI UNIT BUALEMO</t>
+  </si>
+  <si>
     <t>SUBMITTED RESPONDENT</t>
   </si>
   <si>
     <t>DRAFT</t>
   </si>
   <si>
+    <t>OPEN</t>
+  </si>
+  <si>
     <t>avatarcrue@gmail.com</t>
   </si>
   <si>
@@ -73,6 +118,27 @@
     <t>n5164@corp.bri.com</t>
   </si>
   <si>
+    <t>bankdanamon.admin@gmail.com</t>
+  </si>
+  <si>
+    <t>kc.luwuk@bprpalulokadanautama.com</t>
+  </si>
+  <si>
+    <t>anasholechah6196@gmail.com</t>
+  </si>
+  <si>
+    <t>cbs_luwuk@yahoo.com</t>
+  </si>
+  <si>
+    <t>allswalayan@ymail.com</t>
+  </si>
+  <si>
+    <t>info_trakindo@gmail.com</t>
+  </si>
+  <si>
+    <t>nbobs@corp.brico.id</t>
+  </si>
+  <si>
     <t>Permanent_fail</t>
   </si>
   <si>
@@ -101,6 +167,45 @@
   </si>
   <si>
     <t>02 Jun 2026, 09:36:44</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:00:04</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:07:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:38:30</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:38:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:23:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:23:53</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 03:53:26</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 03:51:54</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:33:23</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:32:41</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:39:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:39:23</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:50:12</t>
   </si>
 </sst>
 </file>
@@ -458,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -492,22 +597,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -518,22 +623,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -544,22 +649,22 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -570,22 +675,22 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -596,22 +701,22 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -622,22 +727,22 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -648,24 +753,414 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" t="s">
+        <v>56</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" t="s">
+        <v>42</v>
+      </c>
+      <c r="G16" t="s">
+        <v>57</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" t="s">
+        <v>58</v>
+      </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8">
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" t="s">
+        <v>42</v>
+      </c>
+      <c r="G18" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" t="s">
+        <v>42</v>
+      </c>
+      <c r="G20" t="s">
+        <v>61</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" t="s">
+        <v>62</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" t="s">
+        <v>42</v>
+      </c>
+      <c r="F22" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" t="s">
+        <v>63</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G23" t="s">
+        <v>63</v>
+      </c>
+      <c r="H23">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
perbaiki layout stats grid di ipad
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="74">
   <si>
     <t>code</t>
   </si>
@@ -64,6 +64,18 @@
     <t>941bb532-7c5e-4c33-baca-ee0b2d06fb62</t>
   </si>
   <si>
+    <t>96d663ec-f298-4560-9b84-996b8de92249</t>
+  </si>
+  <si>
+    <t>bcd04260-5f2a-4732-99e6-e2a415b8b206</t>
+  </si>
+  <si>
+    <t>19131aed-4f2e-465e-a7f6-9c0d50cbf975</t>
+  </si>
+  <si>
+    <t>5ed2770d-9be6-4fc1-bf70-0d4e10c482c8</t>
+  </si>
+  <si>
     <t>PTBPRSYARIAHKHAIRANINTIAMANAH</t>
   </si>
   <si>
@@ -88,6 +100,18 @@
     <t>ALL BERKEMBANG BERSAMA</t>
   </si>
   <si>
+    <t>TRAKINDO UTAMA, PT</t>
+  </si>
+  <si>
+    <t>BRI UNIT BUALEMO</t>
+  </si>
+  <si>
+    <t>BANK CENTRAL ASIA TBK. CABANG LUWUK</t>
+  </si>
+  <si>
+    <t>BANK PERKREDITAN RAKYAT MITRA NIAGA BANGGAI</t>
+  </si>
+  <si>
     <t>SUBMITTED RESPONDENT</t>
   </si>
   <si>
@@ -121,6 +145,18 @@
     <t>allswalayan@ymail.com</t>
   </si>
   <si>
+    <t>info_trakindo@gmail.com</t>
+  </si>
+  <si>
+    <t>nbobs@corp.brico.id</t>
+  </si>
+  <si>
+    <t>bca_luwuk_pajak@gmail.com</t>
+  </si>
+  <si>
+    <t>toili@mailnesia.com</t>
+  </si>
+  <si>
     <t>Permanent_fail</t>
   </si>
   <si>
@@ -179,6 +215,27 @@
   </si>
   <si>
     <t>02 Jun 2026, 04:32:41</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:39:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:39:23</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:50:12</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:02:57</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:34:59</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:34:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:11:11</t>
   </si>
 </sst>
 </file>
@@ -536,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -570,22 +627,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -596,22 +653,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -622,22 +679,22 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -648,22 +705,22 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -674,22 +731,22 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -700,22 +757,22 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -726,22 +783,22 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -752,22 +809,22 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -778,22 +835,22 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -804,22 +861,22 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G11" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -830,22 +887,22 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F12" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G12" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -856,22 +913,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -882,22 +939,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E14" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G14" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -908,22 +965,22 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -934,22 +991,22 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G16" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -960,22 +1017,22 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G17" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="H17">
         <v>2</v>
@@ -986,22 +1043,22 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F18" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G18" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1012,25 +1069,233 @@
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G19" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H19">
         <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" t="s">
+        <v>49</v>
+      </c>
+      <c r="G21" t="s">
+        <v>68</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" t="s">
+        <v>69</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" t="s">
+        <v>48</v>
+      </c>
+      <c r="G23" t="s">
+        <v>69</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" t="s">
+        <v>47</v>
+      </c>
+      <c r="F24" t="s">
+        <v>47</v>
+      </c>
+      <c r="G24" t="s">
+        <v>70</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" t="s">
+        <v>71</v>
+      </c>
+      <c r="H25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" t="s">
+        <v>49</v>
+      </c>
+      <c r="G26" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" t="s">
+        <v>47</v>
+      </c>
+      <c r="F27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27" t="s">
+        <v>73</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update IPAS data and append new entries to email history records
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="238">
   <si>
     <t>code</t>
   </si>
@@ -67,7 +67,7 @@
     <t>5ed2770d-9be6-4fc1-bf70-0d4e10c482c8</t>
   </si>
   <si>
-    <t>2b350499-a5b6-45ce-97b3-88359725419f</t>
+    <t>aed96e17-8337-406e-9f72-c02f709f865c</t>
   </si>
   <si>
     <t>ad55d177-41a1-444e-ae54-8c6807aee095</t>
@@ -127,6 +127,42 @@
     <t>df80536f-5125-46c8-aa0a-220b8d26441b</t>
   </si>
   <si>
+    <t>e674036e-bee0-47b7-bc94-a0c32bfa2d71</t>
+  </si>
+  <si>
+    <t>081008bc-6a02-4888-bfb2-2c1c805fa4ad</t>
+  </si>
+  <si>
+    <t>358e68c2-9ecd-47b3-85a5-e07045612b91</t>
+  </si>
+  <si>
+    <t>9e3fbec4-42cd-41c0-9b1d-f442487ed552</t>
+  </si>
+  <si>
+    <t>01b351f3-b52c-4516-a91c-00f58d08579d</t>
+  </si>
+  <si>
+    <t>7880f953-35e8-4387-aac5-b4a94b0c3c2e</t>
+  </si>
+  <si>
+    <t>74e56a04-fcd1-4332-ba6e-1bfb657dc781</t>
+  </si>
+  <si>
+    <t>d61d41d8-08d5-40a5-9a4b-ec2cda0629c1</t>
+  </si>
+  <si>
+    <t>66b93b8d-817c-4af4-9183-47792e43d54e</t>
+  </si>
+  <si>
+    <t>b6c21085-5e3c-4d3b-bcb0-1e48c3bbaca7</t>
+  </si>
+  <si>
+    <t>15f31e98-1701-4d23-8de8-7493899a44db</t>
+  </si>
+  <si>
+    <t>8d3e9626-0215-47a7-86cd-bf85990128c8</t>
+  </si>
+  <si>
     <t>BANK DANAMON INDONESIA, PT TBK KCP LUWUK</t>
   </si>
   <si>
@@ -214,6 +250,42 @@
     <t>BANK BPD</t>
   </si>
   <si>
+    <t>AKAR DAYA MANDIRI PT</t>
+  </si>
+  <si>
+    <t>BANK BPR PALU LOKADANA UTAMA CAB POSO, PT</t>
+  </si>
+  <si>
+    <t>AMRI MARGA JAYA, PT</t>
+  </si>
+  <si>
+    <t>PLTA Poso 1</t>
+  </si>
+  <si>
+    <t>KCP MANDIRI MITRA USAHA TENTENA</t>
+  </si>
+  <si>
+    <t>PNM MODAL MIKRO</t>
+  </si>
+  <si>
+    <t>Balindo Manunggal Bersama, PT</t>
+  </si>
+  <si>
+    <t>FIF, PT</t>
+  </si>
+  <si>
+    <t>SEKOLAH POLISI NEGARA</t>
+  </si>
+  <si>
+    <t>PDAM KAB DONGGALA</t>
+  </si>
+  <si>
+    <t>BPR PALU LOKADANA UTAMA KAS LABUAN</t>
+  </si>
+  <si>
+    <t>PT. BANK SULTENG KAS LABEAN</t>
+  </si>
+  <si>
     <t>OPEN</t>
   </si>
   <si>
@@ -313,6 +385,42 @@
     <t>bsposo@yahoo.com</t>
   </si>
   <si>
+    <t>akardayamandiri49@gmail.com</t>
+  </si>
+  <si>
+    <t>kc.poso@bprpalulokadanautama.com</t>
+  </si>
+  <si>
+    <t>pt.amrimargajaya@ymail.com</t>
+  </si>
+  <si>
+    <t>pltaposo2@posoenergy.com</t>
+  </si>
+  <si>
+    <t>kcpmandirimitrausaha@gmail.com</t>
+  </si>
+  <si>
+    <t>ulamposo@gmail.com</t>
+  </si>
+  <si>
+    <t>gracekayupa@gmail.com</t>
+  </si>
+  <si>
+    <t>dewiputrihilika90@gmail.com</t>
+  </si>
+  <si>
+    <t>kppnpalu651707@yahoo.com</t>
+  </si>
+  <si>
+    <t>pdam_donggala@gmail.com</t>
+  </si>
+  <si>
+    <t>bprlabuan@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>banksulteng_kaslabean@yahoo.com</t>
+  </si>
+  <si>
     <t>Permanent_fail</t>
   </si>
   <si>
@@ -322,6 +430,15 @@
     <t>Queued</t>
   </si>
   <si>
+    <t>Clicked</t>
+  </si>
+  <si>
+    <t>Opened</t>
+  </si>
+  <si>
+    <t>Delivered</t>
+  </si>
+  <si>
     <t>09 Jun 2026, 11:00:04</t>
   </si>
   <si>
@@ -512,6 +629,105 @@
   </si>
   <si>
     <t>02 Jun 2026, 08:52:14</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:17:21</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:59:00</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:58:55</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:13:28</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 00:37:51</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 00:37:47</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:08:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:07:16</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:57:14</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 22:47:26</t>
+  </si>
+  <si>
+    <t>26 May 2026, 08:34:35</t>
+  </si>
+  <si>
+    <t>26 May 2026, 07:30:38</t>
+  </si>
+  <si>
+    <t>26 May 2026, 07:30:35</t>
+  </si>
+  <si>
+    <t>31 May 2026, 12:04:58</t>
+  </si>
+  <si>
+    <t>31 May 2026, 12:04:55</t>
+  </si>
+  <si>
+    <t>31 May 2026, 12:04:51</t>
+  </si>
+  <si>
+    <t>26 May 2026, 11:40:36</t>
+  </si>
+  <si>
+    <t>26 May 2026, 11:27:53</t>
+  </si>
+  <si>
+    <t>26 May 2026, 11:27:52</t>
+  </si>
+  <si>
+    <t>26 May 2026, 09:13:56</t>
+  </si>
+  <si>
+    <t>26 May 2026, 08:30:14</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 13:44:06</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:54:52</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:53:32</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:53:24</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:30:55</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:29:47</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:31:35</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:02:07</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:30:02</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:29:34</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:12:10</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:11:35</t>
   </si>
 </sst>
 </file>
@@ -869,7 +1085,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -903,22 +1119,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -929,22 +1145,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G3" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -955,22 +1171,22 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -981,22 +1197,22 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1007,22 +1223,22 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H6">
         <v>2</v>
@@ -1033,22 +1249,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1059,22 +1275,22 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F8" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -1085,22 +1301,22 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="E9" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1111,22 +1327,22 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="E10" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F10" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -1137,22 +1353,22 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="E11" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F11" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G11" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1163,22 +1379,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="E12" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F12" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="H12">
         <v>2</v>
@@ -1189,22 +1405,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>151</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -1215,22 +1431,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F14" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G14" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="H14">
         <v>2</v>
@@ -1241,22 +1457,22 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E15" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1267,22 +1483,22 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E16" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G16" t="s">
-        <v>115</v>
+        <v>154</v>
       </c>
       <c r="H16">
         <v>2</v>
@@ -1293,22 +1509,22 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="E17" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G17" t="s">
-        <v>116</v>
+        <v>155</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1319,22 +1535,22 @@
         <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="E18" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G18" t="s">
-        <v>116</v>
+        <v>155</v>
       </c>
       <c r="H18">
         <v>2</v>
@@ -1345,22 +1561,22 @@
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F19" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1371,22 +1587,22 @@
         <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="E20" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F20" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>157</v>
       </c>
       <c r="H20">
         <v>2</v>
@@ -1397,22 +1613,22 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F21" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G21" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="H21">
         <v>3</v>
@@ -1423,22 +1639,22 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F22" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G22" t="s">
-        <v>120</v>
+        <v>159</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1449,22 +1665,22 @@
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F23" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G23" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -1475,22 +1691,22 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C24" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E24" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F24" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G24" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="H24">
         <v>2</v>
@@ -1501,22 +1717,22 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D25" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E25" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F25" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>162</v>
       </c>
       <c r="H25">
         <v>3</v>
@@ -1527,22 +1743,22 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G26" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1553,22 +1769,22 @@
         <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E27" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F27" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G27" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="H27">
         <v>2</v>
@@ -1579,22 +1795,22 @@
         <v>17</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E28" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F28" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G28" t="s">
-        <v>123</v>
+        <v>162</v>
       </c>
       <c r="H28">
         <v>3</v>
@@ -1605,22 +1821,22 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D29" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="E29" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F29" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G29" t="s">
-        <v>124</v>
+        <v>163</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -1631,22 +1847,22 @@
         <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E30" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F30" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G30" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -1657,22 +1873,22 @@
         <v>17</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D31" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E31" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F31" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G31" t="s">
-        <v>126</v>
+        <v>165</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -1683,22 +1899,22 @@
         <v>17</v>
       </c>
       <c r="B32" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D32" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E32" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F32" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G32" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -1709,22 +1925,22 @@
         <v>17</v>
       </c>
       <c r="B33" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E33" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F33" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G33" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="H33">
         <v>2</v>
@@ -1735,22 +1951,22 @@
         <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E34" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F34" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G34" t="s">
-        <v>123</v>
+        <v>162</v>
       </c>
       <c r="H34">
         <v>3</v>
@@ -1761,22 +1977,22 @@
         <v>17</v>
       </c>
       <c r="B35" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E35" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F35" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G35" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H35">
         <v>1</v>
@@ -1787,22 +2003,22 @@
         <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D36" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E36" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F36" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G36" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="H36">
         <v>2</v>
@@ -1813,22 +2029,22 @@
         <v>17</v>
       </c>
       <c r="B37" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E37" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G37" t="s">
-        <v>123</v>
+        <v>162</v>
       </c>
       <c r="H37">
         <v>3</v>
@@ -1839,22 +2055,22 @@
         <v>18</v>
       </c>
       <c r="B38" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D38" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F38" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G38" t="s">
-        <v>127</v>
+        <v>166</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -1865,22 +2081,22 @@
         <v>18</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D39" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="E39" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F39" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
-        <v>128</v>
+        <v>167</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -1891,22 +2107,22 @@
         <v>19</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C40" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D40" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="E40" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F40" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G40" t="s">
-        <v>129</v>
+        <v>168</v>
       </c>
       <c r="H40">
         <v>1</v>
@@ -1917,22 +2133,22 @@
         <v>19</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C41" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D41" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="E41" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F41" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G41" t="s">
-        <v>130</v>
+        <v>169</v>
       </c>
       <c r="H41">
         <v>2</v>
@@ -1943,22 +2159,22 @@
         <v>19</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C42" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D42" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="E42" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F42" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G42" t="s">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="H42">
         <v>3</v>
@@ -1969,22 +2185,22 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C43" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D43" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="E43" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F43" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G43" t="s">
-        <v>132</v>
+        <v>171</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -1995,22 +2211,22 @@
         <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C44" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="E44" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F44" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G44" t="s">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -2021,22 +2237,22 @@
         <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D45" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="E45" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F45" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G45" t="s">
-        <v>134</v>
+        <v>173</v>
       </c>
       <c r="H45">
         <v>3</v>
@@ -2047,22 +2263,22 @@
         <v>21</v>
       </c>
       <c r="B46" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E46" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F46" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G46" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -2073,22 +2289,22 @@
         <v>21</v>
       </c>
       <c r="B47" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="C47" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D47" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E47" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F47" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G47" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -2099,22 +2315,22 @@
         <v>22</v>
       </c>
       <c r="B48" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C48" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D48" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="E48" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F48" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G48" t="s">
-        <v>136</v>
+        <v>175</v>
       </c>
       <c r="H48">
         <v>1</v>
@@ -2125,22 +2341,22 @@
         <v>22</v>
       </c>
       <c r="B49" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C49" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D49" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="E49" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F49" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G49" t="s">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="H49">
         <v>2</v>
@@ -2151,22 +2367,22 @@
         <v>22</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C50" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D50" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="E50" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F50" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G50" t="s">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="H50">
         <v>3</v>
@@ -2177,22 +2393,22 @@
         <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="C51" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D51" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E51" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F51" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G51" t="s">
-        <v>138</v>
+        <v>177</v>
       </c>
       <c r="H51">
         <v>1</v>
@@ -2203,22 +2419,22 @@
         <v>23</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="C52" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D52" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E52" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F52" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G52" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -2229,22 +2445,22 @@
         <v>23</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="C53" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D53" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E53" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F53" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G53" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="H53">
         <v>3</v>
@@ -2255,22 +2471,22 @@
         <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="E54" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F54" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G54" t="s">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -2281,22 +2497,22 @@
         <v>24</v>
       </c>
       <c r="B55" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="C55" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D55" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="E55" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F55" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G55" t="s">
-        <v>141</v>
+        <v>180</v>
       </c>
       <c r="H55">
         <v>2</v>
@@ -2307,22 +2523,22 @@
         <v>25</v>
       </c>
       <c r="B56" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="C56" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D56" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E56" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F56" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G56" t="s">
-        <v>142</v>
+        <v>181</v>
       </c>
       <c r="H56">
         <v>1</v>
@@ -2333,22 +2549,22 @@
         <v>25</v>
       </c>
       <c r="B57" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="C57" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E57" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F57" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G57" t="s">
-        <v>143</v>
+        <v>182</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -2359,22 +2575,22 @@
         <v>25</v>
       </c>
       <c r="B58" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="C58" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D58" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E58" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F58" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G58" t="s">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="H58">
         <v>3</v>
@@ -2385,22 +2601,22 @@
         <v>26</v>
       </c>
       <c r="B59" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="C59" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D59" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="E59" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F59" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G59" t="s">
-        <v>145</v>
+        <v>184</v>
       </c>
       <c r="H59">
         <v>1</v>
@@ -2411,22 +2627,22 @@
         <v>26</v>
       </c>
       <c r="B60" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="C60" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="E60" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F60" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G60" t="s">
-        <v>146</v>
+        <v>185</v>
       </c>
       <c r="H60">
         <v>2</v>
@@ -2437,22 +2653,22 @@
         <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C61" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="E61" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F61" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G61" t="s">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -2463,22 +2679,22 @@
         <v>28</v>
       </c>
       <c r="B62" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C62" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="E62" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F62" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G62" t="s">
-        <v>148</v>
+        <v>187</v>
       </c>
       <c r="H62">
         <v>1</v>
@@ -2489,22 +2705,22 @@
         <v>28</v>
       </c>
       <c r="B63" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D63" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="E63" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F63" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G63" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="H63">
         <v>2</v>
@@ -2515,22 +2731,22 @@
         <v>29</v>
       </c>
       <c r="B64" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C64" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D64" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="E64" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F64" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G64" t="s">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="H64">
         <v>1</v>
@@ -2541,22 +2757,22 @@
         <v>29</v>
       </c>
       <c r="B65" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="E65" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F65" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G65" t="s">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="H65">
         <v>2</v>
@@ -2567,22 +2783,22 @@
         <v>30</v>
       </c>
       <c r="B66" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="C66" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E66" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F66" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G66" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="H66">
         <v>1</v>
@@ -2593,22 +2809,22 @@
         <v>30</v>
       </c>
       <c r="B67" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E67" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F67" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G67" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="H67">
         <v>2</v>
@@ -2619,22 +2835,22 @@
         <v>31</v>
       </c>
       <c r="B68" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C68" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E68" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F68" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G68" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="H68">
         <v>1</v>
@@ -2645,22 +2861,22 @@
         <v>31</v>
       </c>
       <c r="B69" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C69" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E69" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F69" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G69" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="H69">
         <v>2</v>
@@ -2671,22 +2887,22 @@
         <v>32</v>
       </c>
       <c r="B70" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C70" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E70" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F70" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G70" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -2697,22 +2913,22 @@
         <v>32</v>
       </c>
       <c r="B71" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C71" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D71" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E71" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F71" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G71" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="H71">
         <v>2</v>
@@ -2723,22 +2939,22 @@
         <v>32</v>
       </c>
       <c r="B72" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C72" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E72" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="F72" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G72" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="H72">
         <v>3</v>
@@ -2749,22 +2965,22 @@
         <v>9</v>
       </c>
       <c r="B73" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C73" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D73" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E73" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F73" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G73" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -2775,22 +2991,22 @@
         <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C74" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D74" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E74" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F74" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G74" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -2801,22 +3017,22 @@
         <v>9</v>
       </c>
       <c r="B75" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C75" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E75" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F75" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G75" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H75">
         <v>1</v>
@@ -2827,22 +3043,22 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C76" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E76" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F76" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G76" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H76">
         <v>2</v>
@@ -2853,22 +3069,22 @@
         <v>33</v>
       </c>
       <c r="B77" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="C77" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E77" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F77" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G77" t="s">
-        <v>158</v>
+        <v>197</v>
       </c>
       <c r="H77">
         <v>1</v>
@@ -2879,22 +3095,22 @@
         <v>33</v>
       </c>
       <c r="B78" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="C78" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E78" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F78" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G78" t="s">
-        <v>159</v>
+        <v>198</v>
       </c>
       <c r="H78">
         <v>2</v>
@@ -2905,22 +3121,22 @@
         <v>34</v>
       </c>
       <c r="B79" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C79" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E79" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F79" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G79" t="s">
-        <v>160</v>
+        <v>199</v>
       </c>
       <c r="H79">
         <v>1</v>
@@ -2931,22 +3147,22 @@
         <v>34</v>
       </c>
       <c r="B80" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C80" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E80" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F80" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G80" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="H80">
         <v>2</v>
@@ -2957,22 +3173,22 @@
         <v>35</v>
       </c>
       <c r="B81" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="C81" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E81" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F81" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G81" t="s">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="H81">
         <v>1</v>
@@ -2983,22 +3199,22 @@
         <v>35</v>
       </c>
       <c r="B82" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="C82" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D82" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E82" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F82" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G82" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="H82">
         <v>2</v>
@@ -3009,22 +3225,22 @@
         <v>36</v>
       </c>
       <c r="B83" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C83" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E83" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F83" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G83" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="H83">
         <v>1</v>
@@ -3035,24 +3251,1376 @@
         <v>36</v>
       </c>
       <c r="B84" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C84" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D84" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E84" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="F84" t="s">
+        <v>137</v>
+      </c>
+      <c r="G84" t="s">
+        <v>204</v>
+      </c>
+      <c r="H84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
+        <v>37</v>
+      </c>
+      <c r="B85" t="s">
+        <v>78</v>
+      </c>
+      <c r="C85" t="s">
+        <v>90</v>
+      </c>
+      <c r="D85" t="s">
+        <v>123</v>
+      </c>
+      <c r="E85" t="s">
+        <v>136</v>
+      </c>
+      <c r="F85" t="s">
+        <v>136</v>
+      </c>
+      <c r="G85" t="s">
+        <v>205</v>
+      </c>
+      <c r="H85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" t="s">
+        <v>37</v>
+      </c>
+      <c r="B86" t="s">
+        <v>78</v>
+      </c>
+      <c r="C86" t="s">
+        <v>90</v>
+      </c>
+      <c r="D86" t="s">
+        <v>123</v>
+      </c>
+      <c r="E86" t="s">
+        <v>136</v>
+      </c>
+      <c r="F86" t="s">
+        <v>137</v>
+      </c>
+      <c r="G86" t="s">
+        <v>205</v>
+      </c>
+      <c r="H86">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" t="s">
+        <v>17</v>
+      </c>
+      <c r="B87" t="s">
+        <v>58</v>
+      </c>
+      <c r="C87" t="s">
+        <v>90</v>
+      </c>
+      <c r="D87" t="s">
         <v>101</v>
       </c>
-      <c r="G84" t="s">
+      <c r="E87" t="s">
+        <v>135</v>
+      </c>
+      <c r="F87" t="s">
+        <v>135</v>
+      </c>
+      <c r="G87" t="s">
+        <v>160</v>
+      </c>
+      <c r="H87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" t="s">
+        <v>17</v>
+      </c>
+      <c r="B88" t="s">
+        <v>58</v>
+      </c>
+      <c r="C88" t="s">
+        <v>90</v>
+      </c>
+      <c r="D88" t="s">
+        <v>101</v>
+      </c>
+      <c r="E88" t="s">
+        <v>135</v>
+      </c>
+      <c r="F88" t="s">
+        <v>136</v>
+      </c>
+      <c r="G88" t="s">
+        <v>161</v>
+      </c>
+      <c r="H88">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" t="s">
+        <v>17</v>
+      </c>
+      <c r="B89" t="s">
+        <v>58</v>
+      </c>
+      <c r="C89" t="s">
+        <v>90</v>
+      </c>
+      <c r="D89" t="s">
+        <v>101</v>
+      </c>
+      <c r="E89" t="s">
+        <v>135</v>
+      </c>
+      <c r="F89" t="s">
+        <v>137</v>
+      </c>
+      <c r="G89" t="s">
+        <v>162</v>
+      </c>
+      <c r="H89">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" t="s">
+        <v>17</v>
+      </c>
+      <c r="B90" t="s">
+        <v>58</v>
+      </c>
+      <c r="C90" t="s">
+        <v>90</v>
+      </c>
+      <c r="D90" t="s">
+        <v>101</v>
+      </c>
+      <c r="E90" t="s">
+        <v>135</v>
+      </c>
+      <c r="F90" t="s">
+        <v>135</v>
+      </c>
+      <c r="G90" t="s">
+        <v>160</v>
+      </c>
+      <c r="H90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" t="s">
+        <v>17</v>
+      </c>
+      <c r="B91" t="s">
+        <v>58</v>
+      </c>
+      <c r="C91" t="s">
+        <v>90</v>
+      </c>
+      <c r="D91" t="s">
+        <v>101</v>
+      </c>
+      <c r="E91" t="s">
+        <v>135</v>
+      </c>
+      <c r="F91" t="s">
+        <v>136</v>
+      </c>
+      <c r="G91" t="s">
+        <v>161</v>
+      </c>
+      <c r="H91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" t="s">
+        <v>17</v>
+      </c>
+      <c r="B92" t="s">
+        <v>58</v>
+      </c>
+      <c r="C92" t="s">
+        <v>90</v>
+      </c>
+      <c r="D92" t="s">
+        <v>101</v>
+      </c>
+      <c r="E92" t="s">
+        <v>135</v>
+      </c>
+      <c r="F92" t="s">
+        <v>137</v>
+      </c>
+      <c r="G92" t="s">
+        <v>162</v>
+      </c>
+      <c r="H92">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93" t="s">
+        <v>17</v>
+      </c>
+      <c r="B93" t="s">
+        <v>58</v>
+      </c>
+      <c r="C93" t="s">
+        <v>90</v>
+      </c>
+      <c r="D93" t="s">
+        <v>102</v>
+      </c>
+      <c r="E93" t="s">
+        <v>135</v>
+      </c>
+      <c r="F93" t="s">
+        <v>135</v>
+      </c>
+      <c r="G93" t="s">
+        <v>163</v>
+      </c>
+      <c r="H93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" t="s">
+        <v>17</v>
+      </c>
+      <c r="B94" t="s">
+        <v>58</v>
+      </c>
+      <c r="C94" t="s">
+        <v>90</v>
+      </c>
+      <c r="D94" t="s">
+        <v>103</v>
+      </c>
+      <c r="E94" t="s">
+        <v>136</v>
+      </c>
+      <c r="F94" t="s">
+        <v>136</v>
+      </c>
+      <c r="G94" t="s">
+        <v>164</v>
+      </c>
+      <c r="H94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" t="s">
+        <v>17</v>
+      </c>
+      <c r="B95" t="s">
+        <v>58</v>
+      </c>
+      <c r="C95" t="s">
+        <v>90</v>
+      </c>
+      <c r="D95" t="s">
+        <v>103</v>
+      </c>
+      <c r="E95" t="s">
+        <v>136</v>
+      </c>
+      <c r="F95" t="s">
+        <v>137</v>
+      </c>
+      <c r="G95" t="s">
         <v>165</v>
       </c>
-      <c r="H84">
+      <c r="H95">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" t="s">
+        <v>17</v>
+      </c>
+      <c r="B96" t="s">
+        <v>58</v>
+      </c>
+      <c r="C96" t="s">
+        <v>90</v>
+      </c>
+      <c r="D96" t="s">
+        <v>101</v>
+      </c>
+      <c r="E96" t="s">
+        <v>135</v>
+      </c>
+      <c r="F96" t="s">
+        <v>135</v>
+      </c>
+      <c r="G96" t="s">
+        <v>160</v>
+      </c>
+      <c r="H96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97" t="s">
+        <v>17</v>
+      </c>
+      <c r="B97" t="s">
+        <v>58</v>
+      </c>
+      <c r="C97" t="s">
+        <v>90</v>
+      </c>
+      <c r="D97" t="s">
+        <v>101</v>
+      </c>
+      <c r="E97" t="s">
+        <v>135</v>
+      </c>
+      <c r="F97" t="s">
+        <v>136</v>
+      </c>
+      <c r="G97" t="s">
+        <v>161</v>
+      </c>
+      <c r="H97">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98" t="s">
+        <v>17</v>
+      </c>
+      <c r="B98" t="s">
+        <v>58</v>
+      </c>
+      <c r="C98" t="s">
+        <v>90</v>
+      </c>
+      <c r="D98" t="s">
+        <v>101</v>
+      </c>
+      <c r="E98" t="s">
+        <v>135</v>
+      </c>
+      <c r="F98" t="s">
+        <v>137</v>
+      </c>
+      <c r="G98" t="s">
+        <v>162</v>
+      </c>
+      <c r="H98">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
+      <c r="A99" t="s">
+        <v>17</v>
+      </c>
+      <c r="B99" t="s">
+        <v>58</v>
+      </c>
+      <c r="C99" t="s">
+        <v>90</v>
+      </c>
+      <c r="D99" t="s">
+        <v>101</v>
+      </c>
+      <c r="E99" t="s">
+        <v>135</v>
+      </c>
+      <c r="F99" t="s">
+        <v>135</v>
+      </c>
+      <c r="G99" t="s">
+        <v>160</v>
+      </c>
+      <c r="H99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
+      <c r="A100" t="s">
+        <v>17</v>
+      </c>
+      <c r="B100" t="s">
+        <v>58</v>
+      </c>
+      <c r="C100" t="s">
+        <v>90</v>
+      </c>
+      <c r="D100" t="s">
+        <v>101</v>
+      </c>
+      <c r="E100" t="s">
+        <v>135</v>
+      </c>
+      <c r="F100" t="s">
+        <v>136</v>
+      </c>
+      <c r="G100" t="s">
+        <v>161</v>
+      </c>
+      <c r="H100">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
+      <c r="A101" t="s">
+        <v>17</v>
+      </c>
+      <c r="B101" t="s">
+        <v>58</v>
+      </c>
+      <c r="C101" t="s">
+        <v>90</v>
+      </c>
+      <c r="D101" t="s">
+        <v>101</v>
+      </c>
+      <c r="E101" t="s">
+        <v>135</v>
+      </c>
+      <c r="F101" t="s">
+        <v>137</v>
+      </c>
+      <c r="G101" t="s">
+        <v>162</v>
+      </c>
+      <c r="H101">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
+      <c r="A102" t="s">
+        <v>38</v>
+      </c>
+      <c r="B102" t="s">
+        <v>79</v>
+      </c>
+      <c r="C102" t="s">
+        <v>90</v>
+      </c>
+      <c r="D102" t="s">
+        <v>124</v>
+      </c>
+      <c r="E102" t="s">
+        <v>136</v>
+      </c>
+      <c r="F102" t="s">
+        <v>136</v>
+      </c>
+      <c r="G102" t="s">
+        <v>206</v>
+      </c>
+      <c r="H102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
+      <c r="A103" t="s">
+        <v>38</v>
+      </c>
+      <c r="B103" t="s">
+        <v>79</v>
+      </c>
+      <c r="C103" t="s">
+        <v>90</v>
+      </c>
+      <c r="D103" t="s">
+        <v>124</v>
+      </c>
+      <c r="E103" t="s">
+        <v>136</v>
+      </c>
+      <c r="F103" t="s">
+        <v>137</v>
+      </c>
+      <c r="G103" t="s">
+        <v>207</v>
+      </c>
+      <c r="H103">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
+      <c r="A104" t="s">
+        <v>39</v>
+      </c>
+      <c r="B104" t="s">
+        <v>80</v>
+      </c>
+      <c r="C104" t="s">
+        <v>90</v>
+      </c>
+      <c r="D104" t="s">
+        <v>125</v>
+      </c>
+      <c r="E104" t="s">
+        <v>135</v>
+      </c>
+      <c r="F104" t="s">
+        <v>135</v>
+      </c>
+      <c r="G104" t="s">
+        <v>208</v>
+      </c>
+      <c r="H104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" t="s">
+        <v>39</v>
+      </c>
+      <c r="B105" t="s">
+        <v>80</v>
+      </c>
+      <c r="C105" t="s">
+        <v>90</v>
+      </c>
+      <c r="D105" t="s">
+        <v>125</v>
+      </c>
+      <c r="E105" t="s">
+        <v>135</v>
+      </c>
+      <c r="F105" t="s">
+        <v>136</v>
+      </c>
+      <c r="G105" t="s">
+        <v>209</v>
+      </c>
+      <c r="H105">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" t="s">
+        <v>39</v>
+      </c>
+      <c r="B106" t="s">
+        <v>80</v>
+      </c>
+      <c r="C106" t="s">
+        <v>90</v>
+      </c>
+      <c r="D106" t="s">
+        <v>125</v>
+      </c>
+      <c r="E106" t="s">
+        <v>135</v>
+      </c>
+      <c r="F106" t="s">
+        <v>137</v>
+      </c>
+      <c r="G106" t="s">
+        <v>210</v>
+      </c>
+      <c r="H106">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" t="s">
+        <v>40</v>
+      </c>
+      <c r="B107" t="s">
+        <v>81</v>
+      </c>
+      <c r="C107" t="s">
+        <v>90</v>
+      </c>
+      <c r="D107" t="s">
+        <v>126</v>
+      </c>
+      <c r="E107" t="s">
+        <v>136</v>
+      </c>
+      <c r="F107" t="s">
+        <v>136</v>
+      </c>
+      <c r="G107" t="s">
+        <v>211</v>
+      </c>
+      <c r="H107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
+      <c r="A108" t="s">
+        <v>40</v>
+      </c>
+      <c r="B108" t="s">
+        <v>81</v>
+      </c>
+      <c r="C108" t="s">
+        <v>90</v>
+      </c>
+      <c r="D108" t="s">
+        <v>126</v>
+      </c>
+      <c r="E108" t="s">
+        <v>136</v>
+      </c>
+      <c r="F108" t="s">
+        <v>137</v>
+      </c>
+      <c r="G108" t="s">
+        <v>212</v>
+      </c>
+      <c r="H108">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
+      <c r="A109" t="s">
+        <v>41</v>
+      </c>
+      <c r="B109" t="s">
+        <v>82</v>
+      </c>
+      <c r="C109" t="s">
+        <v>90</v>
+      </c>
+      <c r="D109" t="s">
+        <v>127</v>
+      </c>
+      <c r="E109" t="s">
+        <v>135</v>
+      </c>
+      <c r="F109" t="s">
+        <v>135</v>
+      </c>
+      <c r="G109" t="s">
+        <v>213</v>
+      </c>
+      <c r="H109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
+      <c r="A110" t="s">
+        <v>41</v>
+      </c>
+      <c r="B110" t="s">
+        <v>82</v>
+      </c>
+      <c r="C110" t="s">
+        <v>90</v>
+      </c>
+      <c r="D110" t="s">
+        <v>127</v>
+      </c>
+      <c r="E110" t="s">
+        <v>135</v>
+      </c>
+      <c r="F110" t="s">
+        <v>137</v>
+      </c>
+      <c r="G110" t="s">
+        <v>214</v>
+      </c>
+      <c r="H110">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
+      <c r="A111" t="s">
+        <v>41</v>
+      </c>
+      <c r="B111" t="s">
+        <v>82</v>
+      </c>
+      <c r="C111" t="s">
+        <v>90</v>
+      </c>
+      <c r="D111" t="s">
+        <v>127</v>
+      </c>
+      <c r="E111" t="s">
+        <v>135</v>
+      </c>
+      <c r="F111" t="s">
+        <v>136</v>
+      </c>
+      <c r="G111" t="s">
+        <v>214</v>
+      </c>
+      <c r="H111">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8">
+      <c r="A112" t="s">
+        <v>42</v>
+      </c>
+      <c r="B112" t="s">
+        <v>83</v>
+      </c>
+      <c r="C112" t="s">
+        <v>90</v>
+      </c>
+      <c r="D112" t="s">
+        <v>128</v>
+      </c>
+      <c r="E112" t="s">
+        <v>136</v>
+      </c>
+      <c r="F112" t="s">
+        <v>136</v>
+      </c>
+      <c r="G112" t="s">
+        <v>215</v>
+      </c>
+      <c r="H112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8">
+      <c r="A113" t="s">
+        <v>42</v>
+      </c>
+      <c r="B113" t="s">
+        <v>83</v>
+      </c>
+      <c r="C113" t="s">
+        <v>90</v>
+      </c>
+      <c r="D113" t="s">
+        <v>128</v>
+      </c>
+      <c r="E113" t="s">
+        <v>136</v>
+      </c>
+      <c r="F113" t="s">
+        <v>137</v>
+      </c>
+      <c r="G113" t="s">
+        <v>215</v>
+      </c>
+      <c r="H113">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8">
+      <c r="A114" t="s">
+        <v>43</v>
+      </c>
+      <c r="B114" t="s">
+        <v>84</v>
+      </c>
+      <c r="C114" t="s">
+        <v>90</v>
+      </c>
+      <c r="D114" t="s">
+        <v>129</v>
+      </c>
+      <c r="E114" t="s">
+        <v>136</v>
+      </c>
+      <c r="F114" t="s">
+        <v>136</v>
+      </c>
+      <c r="G114" t="s">
+        <v>216</v>
+      </c>
+      <c r="H114">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8">
+      <c r="A115" t="s">
+        <v>43</v>
+      </c>
+      <c r="B115" t="s">
+        <v>84</v>
+      </c>
+      <c r="C115" t="s">
+        <v>90</v>
+      </c>
+      <c r="D115" t="s">
+        <v>129</v>
+      </c>
+      <c r="E115" t="s">
+        <v>136</v>
+      </c>
+      <c r="F115" t="s">
+        <v>137</v>
+      </c>
+      <c r="G115" t="s">
+        <v>217</v>
+      </c>
+      <c r="H115">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8">
+      <c r="A116" t="s">
+        <v>44</v>
+      </c>
+      <c r="B116" t="s">
+        <v>85</v>
+      </c>
+      <c r="C116" t="s">
+        <v>90</v>
+      </c>
+      <c r="D116" t="s">
+        <v>130</v>
+      </c>
+      <c r="E116" t="s">
+        <v>136</v>
+      </c>
+      <c r="F116" t="s">
+        <v>138</v>
+      </c>
+      <c r="G116" t="s">
+        <v>218</v>
+      </c>
+      <c r="H116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8">
+      <c r="A117" t="s">
+        <v>44</v>
+      </c>
+      <c r="B117" t="s">
+        <v>85</v>
+      </c>
+      <c r="C117" t="s">
+        <v>90</v>
+      </c>
+      <c r="D117" t="s">
+        <v>130</v>
+      </c>
+      <c r="E117" t="s">
+        <v>136</v>
+      </c>
+      <c r="F117" t="s">
+        <v>139</v>
+      </c>
+      <c r="G117" t="s">
+        <v>219</v>
+      </c>
+      <c r="H117">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8">
+      <c r="A118" t="s">
+        <v>44</v>
+      </c>
+      <c r="B118" t="s">
+        <v>85</v>
+      </c>
+      <c r="C118" t="s">
+        <v>90</v>
+      </c>
+      <c r="D118" t="s">
+        <v>130</v>
+      </c>
+      <c r="E118" t="s">
+        <v>136</v>
+      </c>
+      <c r="F118" t="s">
+        <v>139</v>
+      </c>
+      <c r="G118" t="s">
+        <v>220</v>
+      </c>
+      <c r="H118">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8">
+      <c r="A119" t="s">
+        <v>44</v>
+      </c>
+      <c r="B119" t="s">
+        <v>85</v>
+      </c>
+      <c r="C119" t="s">
+        <v>90</v>
+      </c>
+      <c r="D119" t="s">
+        <v>130</v>
+      </c>
+      <c r="E119" t="s">
+        <v>136</v>
+      </c>
+      <c r="F119" t="s">
+        <v>139</v>
+      </c>
+      <c r="G119" t="s">
+        <v>221</v>
+      </c>
+      <c r="H119">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8">
+      <c r="A120" t="s">
+        <v>44</v>
+      </c>
+      <c r="B120" t="s">
+        <v>85</v>
+      </c>
+      <c r="C120" t="s">
+        <v>90</v>
+      </c>
+      <c r="D120" t="s">
+        <v>130</v>
+      </c>
+      <c r="E120" t="s">
+        <v>136</v>
+      </c>
+      <c r="F120" t="s">
+        <v>140</v>
+      </c>
+      <c r="G120" t="s">
+        <v>222</v>
+      </c>
+      <c r="H120">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8">
+      <c r="A121" t="s">
+        <v>44</v>
+      </c>
+      <c r="B121" t="s">
+        <v>85</v>
+      </c>
+      <c r="C121" t="s">
+        <v>90</v>
+      </c>
+      <c r="D121" t="s">
+        <v>130</v>
+      </c>
+      <c r="E121" t="s">
+        <v>136</v>
+      </c>
+      <c r="F121" t="s">
+        <v>137</v>
+      </c>
+      <c r="G121" t="s">
+        <v>223</v>
+      </c>
+      <c r="H121">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8">
+      <c r="A122" t="s">
+        <v>44</v>
+      </c>
+      <c r="B122" t="s">
+        <v>85</v>
+      </c>
+      <c r="C122" t="s">
+        <v>90</v>
+      </c>
+      <c r="D122" t="s">
+        <v>130</v>
+      </c>
+      <c r="E122" t="s">
+        <v>136</v>
+      </c>
+      <c r="F122" t="s">
+        <v>136</v>
+      </c>
+      <c r="G122" t="s">
+        <v>224</v>
+      </c>
+      <c r="H122">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8">
+      <c r="A123" t="s">
+        <v>44</v>
+      </c>
+      <c r="B123" t="s">
+        <v>85</v>
+      </c>
+      <c r="C123" t="s">
+        <v>90</v>
+      </c>
+      <c r="D123" t="s">
+        <v>130</v>
+      </c>
+      <c r="E123" t="s">
+        <v>136</v>
+      </c>
+      <c r="F123" t="s">
+        <v>137</v>
+      </c>
+      <c r="G123" t="s">
+        <v>225</v>
+      </c>
+      <c r="H123">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8">
+      <c r="A124" t="s">
+        <v>44</v>
+      </c>
+      <c r="B124" t="s">
+        <v>85</v>
+      </c>
+      <c r="C124" t="s">
+        <v>90</v>
+      </c>
+      <c r="D124" t="s">
+        <v>130</v>
+      </c>
+      <c r="E124" t="s">
+        <v>136</v>
+      </c>
+      <c r="F124" t="s">
+        <v>139</v>
+      </c>
+      <c r="G124" t="s">
+        <v>226</v>
+      </c>
+      <c r="H124">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8">
+      <c r="A125" t="s">
+        <v>44</v>
+      </c>
+      <c r="B125" t="s">
+        <v>85</v>
+      </c>
+      <c r="C125" t="s">
+        <v>90</v>
+      </c>
+      <c r="D125" t="s">
+        <v>130</v>
+      </c>
+      <c r="E125" t="s">
+        <v>136</v>
+      </c>
+      <c r="F125" t="s">
+        <v>139</v>
+      </c>
+      <c r="G125" t="s">
+        <v>227</v>
+      </c>
+      <c r="H125">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8">
+      <c r="A126" t="s">
+        <v>44</v>
+      </c>
+      <c r="B126" t="s">
+        <v>85</v>
+      </c>
+      <c r="C126" t="s">
+        <v>90</v>
+      </c>
+      <c r="D126" t="s">
+        <v>130</v>
+      </c>
+      <c r="E126" t="s">
+        <v>136</v>
+      </c>
+      <c r="F126" t="s">
+        <v>140</v>
+      </c>
+      <c r="G126" t="s">
+        <v>228</v>
+      </c>
+      <c r="H126">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8">
+      <c r="A127" t="s">
+        <v>44</v>
+      </c>
+      <c r="B127" t="s">
+        <v>85</v>
+      </c>
+      <c r="C127" t="s">
+        <v>90</v>
+      </c>
+      <c r="D127" t="s">
+        <v>130</v>
+      </c>
+      <c r="E127" t="s">
+        <v>136</v>
+      </c>
+      <c r="F127" t="s">
+        <v>137</v>
+      </c>
+      <c r="G127" t="s">
+        <v>229</v>
+      </c>
+      <c r="H127">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8">
+      <c r="A128" t="s">
+        <v>45</v>
+      </c>
+      <c r="B128" t="s">
+        <v>86</v>
+      </c>
+      <c r="C128" t="s">
+        <v>90</v>
+      </c>
+      <c r="D128" t="s">
+        <v>131</v>
+      </c>
+      <c r="E128" t="s">
+        <v>136</v>
+      </c>
+      <c r="F128" t="s">
+        <v>136</v>
+      </c>
+      <c r="G128" t="s">
+        <v>230</v>
+      </c>
+      <c r="H128">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8">
+      <c r="A129" t="s">
+        <v>45</v>
+      </c>
+      <c r="B129" t="s">
+        <v>86</v>
+      </c>
+      <c r="C129" t="s">
+        <v>90</v>
+      </c>
+      <c r="D129" t="s">
+        <v>131</v>
+      </c>
+      <c r="E129" t="s">
+        <v>136</v>
+      </c>
+      <c r="F129" t="s">
+        <v>137</v>
+      </c>
+      <c r="G129" t="s">
+        <v>231</v>
+      </c>
+      <c r="H129">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8">
+      <c r="A130" t="s">
+        <v>46</v>
+      </c>
+      <c r="B130" t="s">
+        <v>87</v>
+      </c>
+      <c r="C130" t="s">
+        <v>90</v>
+      </c>
+      <c r="D130" t="s">
+        <v>132</v>
+      </c>
+      <c r="E130" t="s">
+        <v>136</v>
+      </c>
+      <c r="F130" t="s">
+        <v>137</v>
+      </c>
+      <c r="G130" t="s">
+        <v>232</v>
+      </c>
+      <c r="H130">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8">
+      <c r="A131" t="s">
+        <v>46</v>
+      </c>
+      <c r="B131" t="s">
+        <v>87</v>
+      </c>
+      <c r="C131" t="s">
+        <v>90</v>
+      </c>
+      <c r="D131" t="s">
+        <v>132</v>
+      </c>
+      <c r="E131" t="s">
+        <v>136</v>
+      </c>
+      <c r="F131" t="s">
+        <v>136</v>
+      </c>
+      <c r="G131" t="s">
+        <v>232</v>
+      </c>
+      <c r="H131">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8">
+      <c r="A132" t="s">
+        <v>47</v>
+      </c>
+      <c r="B132" t="s">
+        <v>88</v>
+      </c>
+      <c r="C132" t="s">
+        <v>90</v>
+      </c>
+      <c r="D132" t="s">
+        <v>133</v>
+      </c>
+      <c r="E132" t="s">
+        <v>135</v>
+      </c>
+      <c r="F132" t="s">
+        <v>135</v>
+      </c>
+      <c r="G132" t="s">
+        <v>233</v>
+      </c>
+      <c r="H132">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8">
+      <c r="A133" t="s">
+        <v>47</v>
+      </c>
+      <c r="B133" t="s">
+        <v>88</v>
+      </c>
+      <c r="C133" t="s">
+        <v>90</v>
+      </c>
+      <c r="D133" t="s">
+        <v>133</v>
+      </c>
+      <c r="E133" t="s">
+        <v>135</v>
+      </c>
+      <c r="F133" t="s">
+        <v>136</v>
+      </c>
+      <c r="G133" t="s">
+        <v>234</v>
+      </c>
+      <c r="H133">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8">
+      <c r="A134" t="s">
+        <v>47</v>
+      </c>
+      <c r="B134" t="s">
+        <v>88</v>
+      </c>
+      <c r="C134" t="s">
+        <v>90</v>
+      </c>
+      <c r="D134" t="s">
+        <v>133</v>
+      </c>
+      <c r="E134" t="s">
+        <v>135</v>
+      </c>
+      <c r="F134" t="s">
+        <v>137</v>
+      </c>
+      <c r="G134" t="s">
+        <v>235</v>
+      </c>
+      <c r="H134">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8">
+      <c r="A135" t="s">
+        <v>48</v>
+      </c>
+      <c r="B135" t="s">
+        <v>89</v>
+      </c>
+      <c r="C135" t="s">
+        <v>90</v>
+      </c>
+      <c r="D135" t="s">
+        <v>134</v>
+      </c>
+      <c r="E135" t="s">
+        <v>136</v>
+      </c>
+      <c r="F135" t="s">
+        <v>136</v>
+      </c>
+      <c r="G135" t="s">
+        <v>236</v>
+      </c>
+      <c r="H135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8">
+      <c r="A136" t="s">
+        <v>48</v>
+      </c>
+      <c r="B136" t="s">
+        <v>89</v>
+      </c>
+      <c r="C136" t="s">
+        <v>90</v>
+      </c>
+      <c r="D136" t="s">
+        <v>134</v>
+      </c>
+      <c r="E136" t="s">
+        <v>136</v>
+      </c>
+      <c r="F136" t="s">
+        <v>137</v>
+      </c>
+      <c r="G136" t="s">
+        <v>237</v>
+      </c>
+      <c r="H136">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update email survey tracking data and timestamps
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="251">
   <si>
     <t>code</t>
   </si>
@@ -40,6 +40,15 @@
     <t>order</t>
   </si>
   <si>
+    <t>ec2ea21f-b88a-400a-8f3d-a03562ff60ad</t>
+  </si>
+  <si>
+    <t>4b3d4210-f21f-43bc-90cb-365395f8d755</t>
+  </si>
+  <si>
+    <t>81b140d6-80f9-436f-81e4-bbfc8ae820d3</t>
+  </si>
+  <si>
     <t>0d4bfa96-7cd5-47d9-b366-e133f6ea27c4</t>
   </si>
   <si>
@@ -160,7 +169,13 @@
     <t>15f31e98-1701-4d23-8de8-7493899a44db</t>
   </si>
   <si>
-    <t>8d3e9626-0215-47a7-86cd-bf85990128c8</t>
+    <t>BRI UNIT SALAKAN</t>
+  </si>
+  <si>
+    <t>PTBPRSYARIAHKHAIRANINTIAMANAH</t>
+  </si>
+  <si>
+    <t>BPR MODERN EXPRESS PT</t>
   </si>
   <si>
     <t>BANK DANAMON INDONESIA, PT TBK KCP LUWUK</t>
@@ -283,12 +298,24 @@
     <t>BPR PALU LOKADANA UTAMA KAS LABUAN</t>
   </si>
   <si>
-    <t>PT. BANK SULTENG KAS LABEAN</t>
+    <t>DRAFT</t>
+  </si>
+  <si>
+    <t>SUBMITTED RESPONDENT</t>
   </si>
   <si>
     <t>OPEN</t>
   </si>
   <si>
+    <t>n5164@corp.bri.com</t>
+  </si>
+  <si>
+    <t>avatarcrue@gmail.com</t>
+  </si>
+  <si>
+    <t>bpr.381@lakadana.com</t>
+  </si>
+  <si>
     <t>bankdanamon.admin@gmail.com</t>
   </si>
   <si>
@@ -418,15 +445,12 @@
     <t>bprlabuan@yahoo.co.id</t>
   </si>
   <si>
-    <t>banksulteng_kaslabean@yahoo.com</t>
+    <t>Bounced</t>
   </si>
   <si>
     <t>Permanent_fail</t>
   </si>
   <si>
-    <t>Bounced</t>
-  </si>
-  <si>
     <t>Queued</t>
   </si>
   <si>
@@ -439,6 +463,27 @@
     <t>Delivered</t>
   </si>
   <si>
+    <t>02 Jun 2026, 09:36:45</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:36:44</t>
+  </si>
+  <si>
+    <t>11 Jun 2026, 14:00:36</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:19:15</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:35:03</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:35:02</t>
+  </si>
+  <si>
+    <t>11 Jun 2026, 10:53:00</t>
+  </si>
+  <si>
     <t>09 Jun 2026, 11:00:04</t>
   </si>
   <si>
@@ -722,12 +767,6 @@
   </si>
   <si>
     <t>01 Jun 2026, 23:29:34</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 04:12:10</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 04:11:35</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1119,22 +1158,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G2" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -1145,22 +1184,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G3" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -1168,28 +1207,28 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1197,25 +1236,25 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G5" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1223,25 +1262,25 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G6" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1249,74 +1288,74 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G7" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F8" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G8" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F9" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G9" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1324,25 +1363,25 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D10" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F10" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G10" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -1353,51 +1392,51 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G11" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E12" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F12" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G12" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1405,25 +1444,25 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E13" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F13" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G13" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1431,51 +1470,51 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E14" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F14" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G14" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F15" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G15" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1483,51 +1522,51 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F16" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G16" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D17" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E17" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F17" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G17" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1535,51 +1574,51 @@
         <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D18" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G18" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D19" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E19" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F19" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G19" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1587,25 +1626,25 @@
         <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E20" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F20" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G20" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1613,25 +1652,25 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D21" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E21" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F21" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G21" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1639,22 +1678,22 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E22" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F22" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G22" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1662,28 +1701,28 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E23" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F23" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G23" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1691,25 +1730,25 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E24" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G24" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1717,48 +1756,48 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E25" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F25" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G25" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E26" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F26" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G26" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1766,25 +1805,25 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F27" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G27" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="H27">
         <v>2</v>
@@ -1792,25 +1831,25 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D28" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E28" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F28" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G28" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="H28">
         <v>3</v>
@@ -1818,25 +1857,25 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C29" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E29" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F29" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G29" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -1844,25 +1883,25 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E30" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F30" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G30" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -1870,25 +1909,25 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C31" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E31" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F31" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G31" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -1896,288 +1935,288 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C32" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E32" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F32" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G32" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C33" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D33" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E33" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F33" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G33" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C34" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D34" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E34" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F34" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G34" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="H34">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D35" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E35" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F35" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G35" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D36" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E36" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F36" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G36" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C37" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D37" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E37" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F37" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G37" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D38" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E38" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F38" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G38" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="H38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D39" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="E39" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G39" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F40" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G40" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="H40">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C41" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F41" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G41" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H41">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D42" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F42" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G42" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="H42">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2185,25 +2224,25 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E43" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F43" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G43" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2211,51 +2250,51 @@
         <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D44" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E44" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F44" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G44" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H44">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B45" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C45" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D45" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E45" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F45" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G45" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="H45">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2263,51 +2302,51 @@
         <v>21</v>
       </c>
       <c r="B46" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D46" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="E46" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F46" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G46" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="H46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B47" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D47" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="E47" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F47" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G47" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2315,25 +2354,25 @@
         <v>22</v>
       </c>
       <c r="B48" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C48" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D48" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E48" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F48" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G48" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2341,51 +2380,51 @@
         <v>22</v>
       </c>
       <c r="B49" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C49" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E49" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F49" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G49" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B50" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C50" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E50" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F50" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G50" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2393,25 +2432,25 @@
         <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C51" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D51" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E51" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F51" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G51" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="H51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2419,51 +2458,51 @@
         <v>23</v>
       </c>
       <c r="B52" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C52" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D52" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E52" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G52" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="H52">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B53" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C53" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D53" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="E53" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F53" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G53" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2471,51 +2510,51 @@
         <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D54" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E54" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F54" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G54" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B55" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C55" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D55" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E55" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F55" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G55" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="H55">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2523,25 +2562,25 @@
         <v>25</v>
       </c>
       <c r="B56" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C56" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D56" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E56" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F56" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G56" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="H56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2549,51 +2588,51 @@
         <v>25</v>
       </c>
       <c r="B57" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D57" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E57" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F57" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G57" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B58" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C58" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D58" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="E58" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F58" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G58" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2601,25 +2640,25 @@
         <v>26</v>
       </c>
       <c r="B59" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C59" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D59" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E59" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F59" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G59" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2627,25 +2666,25 @@
         <v>26</v>
       </c>
       <c r="B60" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C60" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D60" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E60" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F60" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G60" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="H60">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2653,22 +2692,22 @@
         <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C61" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D61" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E61" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F61" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G61" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -2676,28 +2715,28 @@
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B62" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D62" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E62" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F62" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G62" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2705,100 +2744,100 @@
         <v>28</v>
       </c>
       <c r="B63" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C63" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D63" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E63" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F63" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G63" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="H63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B64" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C64" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D64" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E64" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F64" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G64" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="H64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C65" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D65" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E65" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F65" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G65" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="H65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B66" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C66" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D66" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E66" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F66" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G66" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="H66">
         <v>1</v>
@@ -2806,25 +2845,25 @@
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B67" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D67" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E67" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F67" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G67" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="H67">
         <v>2</v>
@@ -2832,25 +2871,25 @@
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D68" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E68" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F68" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G68" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="H68">
         <v>1</v>
@@ -2861,51 +2900,51 @@
         <v>31</v>
       </c>
       <c r="B69" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D69" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E69" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F69" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G69" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B70" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C70" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D70" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E70" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F70" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G70" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2913,25 +2952,25 @@
         <v>32</v>
       </c>
       <c r="B71" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C71" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D71" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E71" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F71" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G71" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="H71">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2939,48 +2978,48 @@
         <v>32</v>
       </c>
       <c r="B72" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C72" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D72" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E72" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F72" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G72" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="H72">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="B73" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D73" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="E73" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F73" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G73" t="s">
-        <v>143</v>
+        <v>206</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -2988,25 +3027,25 @@
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="B74" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C74" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D74" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="E74" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F74" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G74" t="s">
-        <v>144</v>
+        <v>207</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -3014,25 +3053,25 @@
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B75" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C75" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D75" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="E75" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F75" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G75" t="s">
-        <v>145</v>
+        <v>208</v>
       </c>
       <c r="H75">
         <v>1</v>
@@ -3040,25 +3079,25 @@
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B76" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C76" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D76" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="E76" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F76" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G76" t="s">
-        <v>146</v>
+        <v>208</v>
       </c>
       <c r="H76">
         <v>2</v>
@@ -3066,25 +3105,25 @@
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B77" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C77" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D77" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="E77" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F77" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G77" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="H77">
         <v>1</v>
@@ -3092,25 +3131,25 @@
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B78" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C78" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D78" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="E78" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F78" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G78" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="H78">
         <v>2</v>
@@ -3118,132 +3157,132 @@
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B79" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C79" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D79" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="E79" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F79" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G79" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C80" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D80" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="E80" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F80" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G80" t="s">
-        <v>200</v>
+        <v>158</v>
       </c>
       <c r="H80">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="C81" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D81" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="E81" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F81" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G81" t="s">
-        <v>201</v>
+        <v>159</v>
       </c>
       <c r="H81">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="C82" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D82" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="E82" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F82" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G82" t="s">
-        <v>202</v>
+        <v>160</v>
       </c>
       <c r="H82">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="C83" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D83" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="E83" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F83" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G83" t="s">
-        <v>203</v>
+        <v>161</v>
       </c>
       <c r="H83">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -3251,51 +3290,51 @@
         <v>36</v>
       </c>
       <c r="B84" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D84" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E84" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F84" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G84" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="H84">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B85" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C85" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D85" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E85" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F85" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G85" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="H85">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -3303,126 +3342,126 @@
         <v>37</v>
       </c>
       <c r="B86" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C86" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D86" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E86" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F86" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G86" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="H86">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B87" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="C87" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E87" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F87" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G87" t="s">
-        <v>160</v>
+        <v>215</v>
       </c>
       <c r="H87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B88" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="C88" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D88" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="E88" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F88" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G88" t="s">
-        <v>161</v>
+        <v>216</v>
       </c>
       <c r="H88">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B89" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="C89" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D89" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="E89" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F89" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G89" t="s">
-        <v>162</v>
+        <v>217</v>
       </c>
       <c r="H89">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B90" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="C90" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D90" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="E90" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F90" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G90" t="s">
-        <v>160</v>
+        <v>218</v>
       </c>
       <c r="H90">
         <v>1</v>
@@ -3430,25 +3469,25 @@
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="C91" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D91" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="E91" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F91" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G91" t="s">
-        <v>161</v>
+        <v>219</v>
       </c>
       <c r="H91">
         <v>2</v>
@@ -3456,77 +3495,77 @@
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="B92" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="C92" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D92" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
       <c r="E92" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F92" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G92" t="s">
-        <v>162</v>
+        <v>220</v>
       </c>
       <c r="H92">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="B93" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="C93" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D93" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="E93" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F93" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G93" t="s">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="H93">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B94" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C94" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E94" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F94" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G94" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="H94">
         <v>1</v>
@@ -3534,25 +3573,25 @@
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B95" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C95" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D95" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E95" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F95" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G95" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="H95">
         <v>2</v>
@@ -3560,340 +3599,340 @@
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B96" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C96" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D96" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E96" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F96" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G96" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="H96">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B97" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C97" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D97" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E97" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F97" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G97" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="H97">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B98" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C98" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D98" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E98" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F98" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G98" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="H98">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B99" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C99" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D99" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E99" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F99" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G99" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="H99">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B100" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C100" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D100" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E100" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F100" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G100" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="H100">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B101" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C101" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D101" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E101" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F101" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G101" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="H101">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B102" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C102" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D102" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="E102" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F102" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G102" t="s">
-        <v>206</v>
+        <v>180</v>
       </c>
       <c r="H102">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B103" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C103" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D103" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="E103" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F103" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G103" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
       <c r="H103">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="B104" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="C104" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D104" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="E104" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F104" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G104" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H104">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="B105" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="C105" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D105" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="E105" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F105" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G105" t="s">
-        <v>209</v>
+        <v>177</v>
       </c>
       <c r="H105">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="B106" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="C106" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D106" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="E106" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F106" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="G106" t="s">
-        <v>210</v>
+        <v>175</v>
       </c>
       <c r="H106">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B107" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C107" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D107" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E107" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F107" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G107" t="s">
-        <v>211</v>
+        <v>176</v>
       </c>
       <c r="H107">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B108" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C108" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D108" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E108" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F108" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G108" t="s">
-        <v>212</v>
+        <v>177</v>
       </c>
       <c r="H108">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -3901,22 +3940,22 @@
         <v>41</v>
       </c>
       <c r="B109" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C109" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D109" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E109" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F109" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G109" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="H109">
         <v>1</v>
@@ -3927,22 +3966,22 @@
         <v>41</v>
       </c>
       <c r="B110" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C110" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D110" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E110" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F110" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G110" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="H110">
         <v>2</v>
@@ -3950,28 +3989,28 @@
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B111" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C111" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D111" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="E111" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F111" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G111" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="H111">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -3979,25 +4018,25 @@
         <v>42</v>
       </c>
       <c r="B112" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C112" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D112" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E112" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F112" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G112" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="H112">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -4005,25 +4044,25 @@
         <v>42</v>
       </c>
       <c r="B113" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C113" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D113" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E113" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F113" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G113" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="H113">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -4031,22 +4070,22 @@
         <v>43</v>
       </c>
       <c r="B114" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C114" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D114" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="E114" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F114" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G114" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="H114">
         <v>1</v>
@@ -4057,22 +4096,22 @@
         <v>43</v>
       </c>
       <c r="B115" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C115" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D115" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="E115" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F115" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G115" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="H115">
         <v>2</v>
@@ -4083,22 +4122,22 @@
         <v>44</v>
       </c>
       <c r="B116" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C116" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D116" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E116" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F116" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G116" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="H116">
         <v>1</v>
@@ -4109,22 +4148,22 @@
         <v>44</v>
       </c>
       <c r="B117" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C117" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D117" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E117" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F117" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="G117" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="H117">
         <v>2</v>
@@ -4135,22 +4174,22 @@
         <v>44</v>
       </c>
       <c r="B118" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C118" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D118" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E118" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F118" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G118" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="H118">
         <v>3</v>
@@ -4158,340 +4197,340 @@
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B119" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C119" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D119" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E119" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F119" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G119" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="H119">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B120" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C120" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D120" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E120" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F120" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="G120" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="H120">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:8">
       <c r="A121" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B121" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C121" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D121" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E121" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F121" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G121" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H121">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:8">
       <c r="A122" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B122" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C122" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D122" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E122" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F122" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G122" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="H122">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" spans="1:8">
       <c r="A123" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B123" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C123" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D123" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E123" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F123" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G123" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="H123">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:8">
       <c r="A124" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B124" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C124" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D124" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E124" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F124" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="G124" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H124">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B125" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C125" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D125" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E125" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F125" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="G125" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="H125">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="A126" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B126" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C126" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D126" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E126" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F126" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="G126" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="H126">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:8">
       <c r="A127" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B127" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C127" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D127" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E127" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F127" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G127" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="H127">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128" spans="1:8">
       <c r="A128" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B128" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C128" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D128" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E128" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F128" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G128" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="H128">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="129" spans="1:8">
       <c r="A129" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B129" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C129" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D129" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E129" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F129" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="G129" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="H129">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="130" spans="1:8">
       <c r="A130" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B130" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C130" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D130" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="E130" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F130" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G130" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="H130">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B131" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C131" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D131" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="E131" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F131" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="G131" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="H131">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="132" spans="1:8">
@@ -4499,25 +4538,25 @@
         <v>47</v>
       </c>
       <c r="B132" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C132" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D132" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E132" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F132" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="G132" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="H132">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -4525,25 +4564,25 @@
         <v>47</v>
       </c>
       <c r="B133" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C133" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D133" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E133" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F133" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="G133" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="H133">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="134" spans="1:8">
@@ -4551,25 +4590,25 @@
         <v>47</v>
       </c>
       <c r="B134" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C134" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D134" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E134" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F134" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G134" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="H134">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="135" spans="1:8">
@@ -4577,22 +4616,22 @@
         <v>48</v>
       </c>
       <c r="B135" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C135" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D135" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="E135" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F135" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G135" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="H135">
         <v>1</v>
@@ -4603,25 +4642,155 @@
         <v>48</v>
       </c>
       <c r="B136" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C136" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D136" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="E136" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F136" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G136" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="H136">
         <v>2</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8">
+      <c r="A137" t="s">
+        <v>49</v>
+      </c>
+      <c r="B137" t="s">
+        <v>92</v>
+      </c>
+      <c r="C137" t="s">
+        <v>96</v>
+      </c>
+      <c r="D137" t="s">
+        <v>141</v>
+      </c>
+      <c r="E137" t="s">
+        <v>143</v>
+      </c>
+      <c r="F137" t="s">
+        <v>145</v>
+      </c>
+      <c r="G137" t="s">
+        <v>247</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8">
+      <c r="A138" t="s">
+        <v>49</v>
+      </c>
+      <c r="B138" t="s">
+        <v>92</v>
+      </c>
+      <c r="C138" t="s">
+        <v>96</v>
+      </c>
+      <c r="D138" t="s">
+        <v>141</v>
+      </c>
+      <c r="E138" t="s">
+        <v>143</v>
+      </c>
+      <c r="F138" t="s">
+        <v>143</v>
+      </c>
+      <c r="G138" t="s">
+        <v>247</v>
+      </c>
+      <c r="H138">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8">
+      <c r="A139" t="s">
+        <v>50</v>
+      </c>
+      <c r="B139" t="s">
+        <v>93</v>
+      </c>
+      <c r="C139" t="s">
+        <v>96</v>
+      </c>
+      <c r="D139" t="s">
+        <v>142</v>
+      </c>
+      <c r="E139" t="s">
+        <v>144</v>
+      </c>
+      <c r="F139" t="s">
+        <v>144</v>
+      </c>
+      <c r="G139" t="s">
+        <v>248</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8">
+      <c r="A140" t="s">
+        <v>50</v>
+      </c>
+      <c r="B140" t="s">
+        <v>93</v>
+      </c>
+      <c r="C140" t="s">
+        <v>96</v>
+      </c>
+      <c r="D140" t="s">
+        <v>142</v>
+      </c>
+      <c r="E140" t="s">
+        <v>144</v>
+      </c>
+      <c r="F140" t="s">
+        <v>143</v>
+      </c>
+      <c r="G140" t="s">
+        <v>249</v>
+      </c>
+      <c r="H140">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8">
+      <c r="A141" t="s">
+        <v>50</v>
+      </c>
+      <c r="B141" t="s">
+        <v>93</v>
+      </c>
+      <c r="C141" t="s">
+        <v>96</v>
+      </c>
+      <c r="D141" t="s">
+        <v>142</v>
+      </c>
+      <c r="E141" t="s">
+        <v>144</v>
+      </c>
+      <c r="F141" t="s">
+        <v>145</v>
+      </c>
+      <c r="G141" t="s">
+        <v>250</v>
+      </c>
+      <c r="H141">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update sync progress UI with doughnut gauge chart and append email history records
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="124">
   <si>
     <t>code</t>
   </si>
@@ -82,6 +82,24 @@
     <t>ad55d177-41a1-444e-ae54-8c6807aee095</t>
   </si>
   <si>
+    <t>2155505c-bb3d-48ec-ba48-ac98edbdca95</t>
+  </si>
+  <si>
+    <t>abbb91f7-66fb-497f-87e0-235b843068fd</t>
+  </si>
+  <si>
+    <t>64348838-c95b-4e73-8c90-1539e49a8fa6</t>
+  </si>
+  <si>
+    <t>0219fe15-1f5c-4cd7-96f0-734727640195</t>
+  </si>
+  <si>
+    <t>208ebcc6-9881-4752-a982-5d8825476be0</t>
+  </si>
+  <si>
+    <t>df965e5e-d457-436c-a65a-af7726c7ce2b</t>
+  </si>
+  <si>
     <t>BRI UNIT SALAKAN</t>
   </si>
   <si>
@@ -124,6 +142,24 @@
     <t>TOTALINDO BANGGAI PERKASA</t>
   </si>
   <si>
+    <t>REKAYASA INDUSTRI PT</t>
+  </si>
+  <si>
+    <t>JOB PERTAMINA - MEDCO E&amp;P TOMORI SULAWESI</t>
+  </si>
+  <si>
+    <t>INDONESIA TSINGSHAN STAINLESS STEEL</t>
+  </si>
+  <si>
+    <t>HUA CHIN ALUMINUM  INDONESIA</t>
+  </si>
+  <si>
+    <t>TIGA BAJI, PT</t>
+  </si>
+  <si>
+    <t>MCC15 ENGINEERING AND CONSTRUCTION</t>
+  </si>
+  <si>
     <t>DRAFT</t>
   </si>
   <si>
@@ -184,6 +220,24 @@
     <t>totalindobatbperkasa@gmail.com</t>
   </si>
   <si>
+    <t>wandysendjaja@yahoo.com</t>
+  </si>
+  <si>
+    <t>haris.ismail@job-tomori.com</t>
+  </si>
+  <si>
+    <t>secretariat@it-stainlesssteel.com</t>
+  </si>
+  <si>
+    <t>secretariathuachinind@gmail.com</t>
+  </si>
+  <si>
+    <t>aka-hamsah@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>mccmorowali@yahoo.com</t>
+  </si>
+  <si>
     <t>Bounced</t>
   </si>
   <si>
@@ -293,6 +347,45 @@
   </si>
   <si>
     <t>02 Jun 2026, 05:57:20</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:05:04</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:49:00</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:48:57</t>
+  </si>
+  <si>
+    <t>18 May 2026, 12:37:49</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 09:53:25</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 05:51:24</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 02:23:23</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 10:57:25</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 22:48:15</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:04:32</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:47:52</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:55:13</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:52:30</t>
   </si>
 </sst>
 </file>
@@ -650,7 +743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -684,22 +777,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -710,22 +803,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -736,22 +829,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -762,22 +855,22 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -788,22 +881,22 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G6" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="H6">
         <v>3</v>
@@ -814,22 +907,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G7" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="H7">
         <v>4</v>
@@ -840,22 +933,22 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G8" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -866,22 +959,22 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G9" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -892,22 +985,22 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G10" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -918,22 +1011,22 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -944,22 +1037,22 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G12" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -970,22 +1063,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G13" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -996,22 +1089,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1022,22 +1115,22 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -1048,22 +1141,22 @@
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G16" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1074,22 +1167,22 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="H17">
         <v>2</v>
@@ -1100,22 +1193,22 @@
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F18" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1126,22 +1219,22 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F19" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H19">
         <v>2</v>
@@ -1152,22 +1245,22 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E20" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F20" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G20" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1178,22 +1271,22 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F21" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H21">
         <v>2</v>
@@ -1204,22 +1297,22 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C22" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="E22" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F22" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1230,22 +1323,22 @@
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D23" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F23" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="H23">
         <v>2</v>
@@ -1256,22 +1349,22 @@
         <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="E24" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F24" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G24" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -1282,22 +1375,22 @@
         <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="E25" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F25" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="H25">
         <v>2</v>
@@ -1308,22 +1401,22 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D26" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F26" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G26" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1334,22 +1427,22 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E27" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F27" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G27" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="H27">
         <v>2</v>
@@ -1360,22 +1453,22 @@
         <v>17</v>
       </c>
       <c r="B28" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E28" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F28" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G28" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -1386,22 +1479,22 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E29" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F29" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G29" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="H29">
         <v>2</v>
@@ -1412,22 +1505,22 @@
         <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C30" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D30" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E30" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F30" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G30" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -1438,22 +1531,22 @@
         <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D31" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G31" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -1464,22 +1557,22 @@
         <v>18</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D32" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E32" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F32" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G32" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="H32">
         <v>3</v>
@@ -1490,22 +1583,22 @@
         <v>19</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="E33" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F33" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G33" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -1516,22 +1609,22 @@
         <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D34" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E34" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F34" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G34" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -1542,22 +1635,22 @@
         <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D35" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E35" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F35" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G35" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1568,22 +1661,22 @@
         <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D36" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E36" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F36" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G36" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H36">
         <v>3</v>
@@ -1594,22 +1687,22 @@
         <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D37" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E37" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F37" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G37" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H37">
         <v>1</v>
@@ -1620,22 +1713,22 @@
         <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D38" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E38" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F38" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G38" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H38">
         <v>2</v>
@@ -1646,22 +1739,22 @@
         <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D39" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E39" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G39" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H39">
         <v>3</v>
@@ -1672,22 +1765,22 @@
         <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D40" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E40" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F40" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G40" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="H40">
         <v>1</v>
@@ -1698,22 +1791,22 @@
         <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C41" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D41" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E41" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F41" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G41" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="H41">
         <v>1</v>
@@ -1724,22 +1817,22 @@
         <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D42" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F42" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G42" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -1750,22 +1843,22 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D43" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E43" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F43" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G43" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -1776,22 +1869,22 @@
         <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D44" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E44" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F44" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G44" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -1802,22 +1895,22 @@
         <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D45" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E45" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F45" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G45" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H45">
         <v>3</v>
@@ -1828,22 +1921,22 @@
         <v>20</v>
       </c>
       <c r="B46" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D46" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E46" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F46" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G46" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -1854,22 +1947,22 @@
         <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C47" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D47" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E47" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F47" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G47" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -1880,22 +1973,22 @@
         <v>20</v>
       </c>
       <c r="B48" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D48" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E48" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F48" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G48" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H48">
         <v>3</v>
@@ -1906,22 +1999,22 @@
         <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C49" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D49" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E49" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F49" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G49" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H49">
         <v>1</v>
@@ -1932,22 +2025,22 @@
         <v>20</v>
       </c>
       <c r="B50" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C50" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D50" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E50" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F50" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G50" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H50">
         <v>2</v>
@@ -1958,22 +2051,22 @@
         <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D51" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E51" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F51" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G51" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H51">
         <v>3</v>
@@ -1984,22 +2077,22 @@
         <v>20</v>
       </c>
       <c r="B52" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C52" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D52" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E52" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F52" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G52" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -2010,22 +2103,22 @@
         <v>20</v>
       </c>
       <c r="B53" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D53" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E53" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F53" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G53" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -2036,22 +2129,22 @@
         <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D54" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E54" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F54" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G54" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H54">
         <v>3</v>
@@ -2062,22 +2155,22 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D55" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E55" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F55" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G55" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="H55">
         <v>1</v>
@@ -2088,22 +2181,22 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D56" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E56" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F56" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G56" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="H56">
         <v>1</v>
@@ -2114,22 +2207,22 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D57" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E57" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F57" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G57" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -2140,22 +2233,22 @@
         <v>20</v>
       </c>
       <c r="B58" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D58" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E58" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F58" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G58" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H58">
         <v>1</v>
@@ -2166,22 +2259,22 @@
         <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C59" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D59" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E59" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F59" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G59" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H59">
         <v>2</v>
@@ -2192,22 +2285,22 @@
         <v>20</v>
       </c>
       <c r="B60" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C60" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D60" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E60" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F60" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G60" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H60">
         <v>3</v>
@@ -2218,22 +2311,22 @@
         <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D61" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E61" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F61" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G61" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -2244,22 +2337,22 @@
         <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D62" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E62" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F62" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G62" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H62">
         <v>2</v>
@@ -2270,22 +2363,22 @@
         <v>20</v>
       </c>
       <c r="B63" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D63" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E63" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F63" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G63" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H63">
         <v>3</v>
@@ -2296,22 +2389,22 @@
         <v>20</v>
       </c>
       <c r="B64" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C64" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D64" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E64" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F64" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G64" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H64">
         <v>1</v>
@@ -2322,22 +2415,22 @@
         <v>20</v>
       </c>
       <c r="B65" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C65" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D65" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E65" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F65" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G65" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H65">
         <v>2</v>
@@ -2348,22 +2441,22 @@
         <v>20</v>
       </c>
       <c r="B66" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D66" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E66" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F66" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G66" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H66">
         <v>3</v>
@@ -2374,22 +2467,22 @@
         <v>20</v>
       </c>
       <c r="B67" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C67" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E67" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F67" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G67" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H67">
         <v>1</v>
@@ -2400,22 +2493,22 @@
         <v>20</v>
       </c>
       <c r="B68" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C68" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D68" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E68" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F68" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G68" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H68">
         <v>2</v>
@@ -2426,22 +2519,22 @@
         <v>20</v>
       </c>
       <c r="B69" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D69" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E69" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F69" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G69" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H69">
         <v>3</v>
@@ -2452,22 +2545,22 @@
         <v>20</v>
       </c>
       <c r="B70" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D70" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E70" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F70" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G70" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -2478,22 +2571,22 @@
         <v>20</v>
       </c>
       <c r="B71" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D71" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E71" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F71" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G71" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="H71">
         <v>1</v>
@@ -2504,22 +2597,22 @@
         <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D72" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E72" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F72" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G72" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -2530,22 +2623,22 @@
         <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D73" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E73" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F73" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G73" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -2556,22 +2649,22 @@
         <v>20</v>
       </c>
       <c r="B74" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D74" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E74" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F74" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G74" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -2582,22 +2675,22 @@
         <v>20</v>
       </c>
       <c r="B75" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D75" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E75" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F75" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G75" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H75">
         <v>3</v>
@@ -2608,22 +2701,22 @@
         <v>20</v>
       </c>
       <c r="B76" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D76" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E76" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F76" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G76" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H76">
         <v>1</v>
@@ -2634,22 +2727,22 @@
         <v>20</v>
       </c>
       <c r="B77" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D77" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E77" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F77" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G77" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H77">
         <v>2</v>
@@ -2660,22 +2753,22 @@
         <v>20</v>
       </c>
       <c r="B78" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D78" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E78" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F78" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G78" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H78">
         <v>3</v>
@@ -2686,22 +2779,22 @@
         <v>20</v>
       </c>
       <c r="B79" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D79" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E79" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F79" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G79" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H79">
         <v>1</v>
@@ -2712,22 +2805,22 @@
         <v>20</v>
       </c>
       <c r="B80" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D80" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E80" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F80" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G80" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H80">
         <v>2</v>
@@ -2738,22 +2831,22 @@
         <v>20</v>
       </c>
       <c r="B81" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D81" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E81" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F81" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G81" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H81">
         <v>3</v>
@@ -2764,22 +2857,22 @@
         <v>20</v>
       </c>
       <c r="B82" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D82" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E82" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F82" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G82" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H82">
         <v>1</v>
@@ -2790,22 +2883,22 @@
         <v>20</v>
       </c>
       <c r="B83" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D83" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E83" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F83" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G83" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H83">
         <v>2</v>
@@ -2816,22 +2909,22 @@
         <v>20</v>
       </c>
       <c r="B84" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D84" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E84" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F84" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G84" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H84">
         <v>3</v>
@@ -2842,22 +2935,22 @@
         <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C85" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D85" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E85" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F85" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G85" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="H85">
         <v>1</v>
@@ -2868,22 +2961,22 @@
         <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D86" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E86" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F86" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G86" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="H86">
         <v>1</v>
@@ -2894,22 +2987,22 @@
         <v>20</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D87" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E87" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F87" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G87" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="H87">
         <v>2</v>
@@ -2920,22 +3013,22 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D88" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E88" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F88" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G88" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H88">
         <v>1</v>
@@ -2946,22 +3039,22 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C89" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D89" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E89" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F89" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G89" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H89">
         <v>2</v>
@@ -2972,22 +3065,22 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D90" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E90" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F90" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G90" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H90">
         <v>3</v>
@@ -2998,22 +3091,22 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D91" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E91" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F91" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G91" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="H91">
         <v>1</v>
@@ -3024,22 +3117,22 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D92" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E92" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F92" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G92" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H92">
         <v>2</v>
@@ -3050,22 +3143,22 @@
         <v>20</v>
       </c>
       <c r="B93" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D93" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E93" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F93" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G93" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H93">
         <v>3</v>
@@ -3076,22 +3169,22 @@
         <v>21</v>
       </c>
       <c r="B94" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D94" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E94" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F94" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G94" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="H94">
         <v>1</v>
@@ -3102,24 +3195,440 @@
         <v>21</v>
       </c>
       <c r="B95" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D95" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E95" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="F95" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G95" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="H95">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" t="s">
+        <v>22</v>
+      </c>
+      <c r="B96" t="s">
+        <v>42</v>
+      </c>
+      <c r="C96" t="s">
+        <v>50</v>
+      </c>
+      <c r="D96" t="s">
+        <v>68</v>
+      </c>
+      <c r="E96" t="s">
+        <v>75</v>
+      </c>
+      <c r="F96" t="s">
+        <v>75</v>
+      </c>
+      <c r="G96" t="s">
+        <v>111</v>
+      </c>
+      <c r="H96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97" t="s">
+        <v>22</v>
+      </c>
+      <c r="B97" t="s">
+        <v>42</v>
+      </c>
+      <c r="C97" t="s">
+        <v>50</v>
+      </c>
+      <c r="D97" t="s">
+        <v>68</v>
+      </c>
+      <c r="E97" t="s">
+        <v>75</v>
+      </c>
+      <c r="F97" t="s">
+        <v>74</v>
+      </c>
+      <c r="G97" t="s">
+        <v>112</v>
+      </c>
+      <c r="H97">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98" t="s">
+        <v>22</v>
+      </c>
+      <c r="B98" t="s">
+        <v>42</v>
+      </c>
+      <c r="C98" t="s">
+        <v>50</v>
+      </c>
+      <c r="D98" t="s">
+        <v>68</v>
+      </c>
+      <c r="E98" t="s">
+        <v>75</v>
+      </c>
+      <c r="F98" t="s">
+        <v>76</v>
+      </c>
+      <c r="G98" t="s">
+        <v>113</v>
+      </c>
+      <c r="H98">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
+      <c r="A99" t="s">
+        <v>23</v>
+      </c>
+      <c r="B99" t="s">
+        <v>43</v>
+      </c>
+      <c r="C99" t="s">
+        <v>50</v>
+      </c>
+      <c r="D99" t="s">
+        <v>69</v>
+      </c>
+      <c r="E99" t="s">
+        <v>75</v>
+      </c>
+      <c r="F99" t="s">
+        <v>75</v>
+      </c>
+      <c r="G99" t="s">
+        <v>114</v>
+      </c>
+      <c r="H99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
+      <c r="A100" t="s">
+        <v>23</v>
+      </c>
+      <c r="B100" t="s">
+        <v>43</v>
+      </c>
+      <c r="C100" t="s">
+        <v>50</v>
+      </c>
+      <c r="D100" t="s">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>75</v>
+      </c>
+      <c r="F100" t="s">
+        <v>75</v>
+      </c>
+      <c r="G100" t="s">
+        <v>115</v>
+      </c>
+      <c r="H100">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
+      <c r="A101" t="s">
+        <v>23</v>
+      </c>
+      <c r="B101" t="s">
+        <v>43</v>
+      </c>
+      <c r="C101" t="s">
+        <v>50</v>
+      </c>
+      <c r="D101" t="s">
+        <v>69</v>
+      </c>
+      <c r="E101" t="s">
+        <v>75</v>
+      </c>
+      <c r="F101" t="s">
+        <v>75</v>
+      </c>
+      <c r="G101" t="s">
+        <v>116</v>
+      </c>
+      <c r="H101">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
+      <c r="A102" t="s">
+        <v>24</v>
+      </c>
+      <c r="B102" t="s">
+        <v>44</v>
+      </c>
+      <c r="C102" t="s">
+        <v>50</v>
+      </c>
+      <c r="D102" t="s">
+        <v>70</v>
+      </c>
+      <c r="E102" t="s">
+        <v>74</v>
+      </c>
+      <c r="F102" t="s">
+        <v>76</v>
+      </c>
+      <c r="G102" t="s">
+        <v>117</v>
+      </c>
+      <c r="H102">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
+      <c r="A103" t="s">
+        <v>24</v>
+      </c>
+      <c r="B103" t="s">
+        <v>44</v>
+      </c>
+      <c r="C103" t="s">
+        <v>50</v>
+      </c>
+      <c r="D103" t="s">
+        <v>70</v>
+      </c>
+      <c r="E103" t="s">
+        <v>74</v>
+      </c>
+      <c r="F103" t="s">
+        <v>74</v>
+      </c>
+      <c r="G103" t="s">
+        <v>117</v>
+      </c>
+      <c r="H103">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
+      <c r="A104" t="s">
+        <v>25</v>
+      </c>
+      <c r="B104" t="s">
+        <v>45</v>
+      </c>
+      <c r="C104" t="s">
+        <v>50</v>
+      </c>
+      <c r="D104" t="s">
+        <v>71</v>
+      </c>
+      <c r="E104" t="s">
+        <v>75</v>
+      </c>
+      <c r="F104" t="s">
+        <v>75</v>
+      </c>
+      <c r="G104" t="s">
+        <v>118</v>
+      </c>
+      <c r="H104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" t="s">
+        <v>25</v>
+      </c>
+      <c r="B105" t="s">
+        <v>45</v>
+      </c>
+      <c r="C105" t="s">
+        <v>50</v>
+      </c>
+      <c r="D105" t="s">
+        <v>71</v>
+      </c>
+      <c r="E105" t="s">
+        <v>75</v>
+      </c>
+      <c r="F105" t="s">
+        <v>74</v>
+      </c>
+      <c r="G105" t="s">
+        <v>119</v>
+      </c>
+      <c r="H105">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" t="s">
+        <v>25</v>
+      </c>
+      <c r="B106" t="s">
+        <v>45</v>
+      </c>
+      <c r="C106" t="s">
+        <v>50</v>
+      </c>
+      <c r="D106" t="s">
+        <v>71</v>
+      </c>
+      <c r="E106" t="s">
+        <v>75</v>
+      </c>
+      <c r="F106" t="s">
+        <v>76</v>
+      </c>
+      <c r="G106" t="s">
+        <v>119</v>
+      </c>
+      <c r="H106">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" t="s">
+        <v>26</v>
+      </c>
+      <c r="B107" t="s">
+        <v>46</v>
+      </c>
+      <c r="C107" t="s">
+        <v>50</v>
+      </c>
+      <c r="D107" t="s">
+        <v>72</v>
+      </c>
+      <c r="E107" t="s">
+        <v>75</v>
+      </c>
+      <c r="F107" t="s">
+        <v>75</v>
+      </c>
+      <c r="G107" t="s">
+        <v>120</v>
+      </c>
+      <c r="H107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
+      <c r="A108" t="s">
+        <v>26</v>
+      </c>
+      <c r="B108" t="s">
+        <v>46</v>
+      </c>
+      <c r="C108" t="s">
+        <v>50</v>
+      </c>
+      <c r="D108" t="s">
+        <v>72</v>
+      </c>
+      <c r="E108" t="s">
+        <v>75</v>
+      </c>
+      <c r="F108" t="s">
+        <v>74</v>
+      </c>
+      <c r="G108" t="s">
+        <v>121</v>
+      </c>
+      <c r="H108">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
+      <c r="A109" t="s">
+        <v>26</v>
+      </c>
+      <c r="B109" t="s">
+        <v>46</v>
+      </c>
+      <c r="C109" t="s">
+        <v>50</v>
+      </c>
+      <c r="D109" t="s">
+        <v>72</v>
+      </c>
+      <c r="E109" t="s">
+        <v>75</v>
+      </c>
+      <c r="F109" t="s">
+        <v>76</v>
+      </c>
+      <c r="G109" t="s">
+        <v>121</v>
+      </c>
+      <c r="H109">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
+      <c r="A110" t="s">
+        <v>27</v>
+      </c>
+      <c r="B110" t="s">
+        <v>47</v>
+      </c>
+      <c r="C110" t="s">
+        <v>50</v>
+      </c>
+      <c r="D110" t="s">
+        <v>73</v>
+      </c>
+      <c r="E110" t="s">
+        <v>74</v>
+      </c>
+      <c r="F110" t="s">
+        <v>74</v>
+      </c>
+      <c r="G110" t="s">
+        <v>122</v>
+      </c>
+      <c r="H110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
+      <c r="A111" t="s">
+        <v>27</v>
+      </c>
+      <c r="B111" t="s">
+        <v>47</v>
+      </c>
+      <c r="C111" t="s">
+        <v>50</v>
+      </c>
+      <c r="D111" t="s">
+        <v>73</v>
+      </c>
+      <c r="E111" t="s">
+        <v>74</v>
+      </c>
+      <c r="F111" t="s">
+        <v>76</v>
+      </c>
+      <c r="G111" t="s">
+        <v>123</v>
+      </c>
+      <c r="H111">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update dashboard UI and rename assign status for all businesses
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="188">
   <si>
     <t>code</t>
   </si>
@@ -100,6 +100,45 @@
     <t>df965e5e-d457-436c-a65a-af7726c7ce2b</t>
   </si>
   <si>
+    <t>0c6fcc80-9ea0-43b2-8775-cb18edc33d25</t>
+  </si>
+  <si>
+    <t>b2cf42e6-965c-49fa-abac-9af54426d0cc</t>
+  </si>
+  <si>
+    <t>e0e3282e-4685-4ad8-b636-6449ef659410</t>
+  </si>
+  <si>
+    <t>9818074f-7f62-4f6f-8a12-7b9ec153718e</t>
+  </si>
+  <si>
+    <t>2676b7e4-6dca-4e7f-991e-6ae27b0b0c85</t>
+  </si>
+  <si>
+    <t>9b9e29d1-fc1e-4b2d-99d7-838fde85299c</t>
+  </si>
+  <si>
+    <t>e807b2d0-c9e8-4158-bc0a-301bcc232add</t>
+  </si>
+  <si>
+    <t>22df9424-5a77-4276-ab7d-9c4bc6b29108</t>
+  </si>
+  <si>
+    <t>b58860b3-d502-48de-bf29-ebc5b51b0389</t>
+  </si>
+  <si>
+    <t>cf953441-4548-4748-b059-68c60a1c9312</t>
+  </si>
+  <si>
+    <t>befe39ef-4187-40aa-9e99-fef88d32baa1</t>
+  </si>
+  <si>
+    <t>df80536f-5125-46c8-aa0a-220b8d26441b</t>
+  </si>
+  <si>
+    <t>e674036e-bee0-47b7-bc94-a0c32bfa2d71</t>
+  </si>
+  <si>
     <t>BRI UNIT SALAKAN</t>
   </si>
   <si>
@@ -160,6 +199,45 @@
     <t>MCC15 ENGINEERING AND CONSTRUCTION</t>
   </si>
   <si>
+    <t>BROLY NICKEL INDUSTRY</t>
+  </si>
+  <si>
+    <t>BANK SYARIAH INDONESIA, PT</t>
+  </si>
+  <si>
+    <t>HADJI KALLA</t>
+  </si>
+  <si>
+    <t>Detian Coking Indonesia</t>
+  </si>
+  <si>
+    <t>JEMBATAN MAS ENGINEERING</t>
+  </si>
+  <si>
+    <t>INDONESIA RUIPU NICKEL AND CROME ALLOY, PT</t>
+  </si>
+  <si>
+    <t>THE SIXTH CHEMICAL ENGINEERING CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>KENCANA BUMI MINERAL</t>
+  </si>
+  <si>
+    <t>CIPTA MANDIRI MOROWALI</t>
+  </si>
+  <si>
+    <t>INDONESIA GUANG CHING NICKEL AND STAINLESS STEEL INDUSTRY TKA</t>
+  </si>
+  <si>
+    <t>KINRUI NEW ENERGY TECHNOLOGIES  INDONESIA</t>
+  </si>
+  <si>
+    <t>BANK BPD</t>
+  </si>
+  <si>
+    <t>AKAR DAYA MANDIRI PT</t>
+  </si>
+  <si>
     <t>DRAFT</t>
   </si>
   <si>
@@ -238,6 +316,45 @@
     <t>mccmorowali@yahoo.com</t>
   </si>
   <si>
+    <t>hengjayasite@yahoo.com</t>
+  </si>
+  <si>
+    <t>sapriliya@bsm.co.id</t>
+  </si>
+  <si>
+    <t>nur.salam.coning@kallagroup.co.id</t>
+  </si>
+  <si>
+    <t>secretariat@detiancoking-ind.com</t>
+  </si>
+  <si>
+    <t>jembatanmas579@yahoo.com</t>
+  </si>
+  <si>
+    <t>smaalkhairatkolono@yahoo.co.id</t>
+  </si>
+  <si>
+    <t>sobeh@ppc-adulsory.com</t>
+  </si>
+  <si>
+    <t>acctaxkbm@yahoo.com</t>
+  </si>
+  <si>
+    <t>ciptamandiri@yahoo.com</t>
+  </si>
+  <si>
+    <t>rukun@bd.em.com</t>
+  </si>
+  <si>
+    <t>secretariatkinrui@gmail.com</t>
+  </si>
+  <si>
+    <t>bsposo@yahoo.com</t>
+  </si>
+  <si>
+    <t>akardayamandiri49@gmail.com</t>
+  </si>
+  <si>
     <t>Bounced</t>
   </si>
   <si>
@@ -386,6 +503,81 @@
   </si>
   <si>
     <t>02 Jun 2026, 08:52:30</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:00:02</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:38</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:06:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:57:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 11:49:47</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:57:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:45:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:43:12</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:08:56</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:11:39</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 04:58:16</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:22:02</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:06:55</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:52:15</t>
+  </si>
+  <si>
+    <t>01 Jun 2026, 23:52:11</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:29:20</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:28:43</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:54:53</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:54:49</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:59:29</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 06:59:25</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:52:48</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 08:52:14</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:17:21</t>
   </si>
 </sst>
 </file>
@@ -743,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -777,22 +969,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
+        <v>116</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -803,22 +995,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -829,22 +1021,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -855,22 +1047,22 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G5" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -881,22 +1073,22 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="H6">
         <v>3</v>
@@ -907,22 +1099,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G7" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="H7">
         <v>4</v>
@@ -933,22 +1125,22 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -959,22 +1151,22 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G9" t="s">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -985,22 +1177,22 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G10" t="s">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -1011,22 +1203,22 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G11" t="s">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -1037,22 +1229,22 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F12" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G12" t="s">
-        <v>86</v>
+        <v>125</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -1063,22 +1255,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F13" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>87</v>
+        <v>126</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -1089,22 +1281,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G14" t="s">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1115,22 +1307,22 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G15" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -1141,22 +1333,22 @@
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F16" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>86</v>
+        <v>125</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1167,22 +1359,22 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E17" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F17" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>87</v>
+        <v>126</v>
       </c>
       <c r="H17">
         <v>2</v>
@@ -1193,22 +1385,22 @@
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1219,22 +1411,22 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F19" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G19" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="H19">
         <v>2</v>
@@ -1245,22 +1437,22 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G20" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1271,22 +1463,22 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D21" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="E21" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G21" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="H21">
         <v>2</v>
@@ -1297,22 +1489,22 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="E22" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G22" t="s">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1323,22 +1515,22 @@
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D23" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G23" t="s">
-        <v>93</v>
+        <v>132</v>
       </c>
       <c r="H23">
         <v>2</v>
@@ -1349,22 +1541,22 @@
         <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F24" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G24" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -1375,22 +1567,22 @@
         <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C25" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="E25" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G25" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
       <c r="H25">
         <v>2</v>
@@ -1401,22 +1593,22 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="E26" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F26" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G26" t="s">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1427,22 +1619,22 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D27" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="E27" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G27" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="H27">
         <v>2</v>
@@ -1453,22 +1645,22 @@
         <v>17</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D28" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="E28" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F28" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G28" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -1479,22 +1671,22 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D29" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="E29" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F29" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G29" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="H29">
         <v>2</v>
@@ -1505,22 +1697,22 @@
         <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F30" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G30" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -1531,22 +1723,22 @@
         <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D31" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E31" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F31" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G31" t="s">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -1557,22 +1749,22 @@
         <v>18</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C32" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E32" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G32" t="s">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="H32">
         <v>3</v>
@@ -1583,22 +1775,22 @@
         <v>19</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C33" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D33" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="E33" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G33" t="s">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -1609,22 +1801,22 @@
         <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C34" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D34" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E34" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G34" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -1635,22 +1827,22 @@
         <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C35" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D35" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E35" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F35" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G35" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1661,22 +1853,22 @@
         <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C36" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D36" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F36" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G36" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H36">
         <v>3</v>
@@ -1687,22 +1879,22 @@
         <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C37" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D37" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F37" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G37" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H37">
         <v>1</v>
@@ -1713,22 +1905,22 @@
         <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C38" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D38" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F38" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G38" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H38">
         <v>2</v>
@@ -1739,22 +1931,22 @@
         <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C39" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D39" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E39" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F39" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G39" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H39">
         <v>3</v>
@@ -1765,22 +1957,22 @@
         <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C40" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D40" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="E40" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F40" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G40" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H40">
         <v>1</v>
@@ -1791,22 +1983,22 @@
         <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C41" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D41" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E41" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F41" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G41" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H41">
         <v>1</v>
@@ -1817,22 +2009,22 @@
         <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C42" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D42" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E42" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F42" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G42" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -1843,22 +2035,22 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C43" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D43" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E43" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F43" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G43" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -1869,22 +2061,22 @@
         <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C44" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D44" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E44" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F44" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G44" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -1895,22 +2087,22 @@
         <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C45" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E45" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F45" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G45" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H45">
         <v>3</v>
@@ -1921,22 +2113,22 @@
         <v>20</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C46" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E46" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F46" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G46" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -1947,22 +2139,22 @@
         <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C47" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E47" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F47" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G47" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -1973,22 +2165,22 @@
         <v>20</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C48" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E48" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F48" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G48" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H48">
         <v>3</v>
@@ -1999,22 +2191,22 @@
         <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C49" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D49" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E49" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F49" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G49" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H49">
         <v>1</v>
@@ -2025,22 +2217,22 @@
         <v>20</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C50" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D50" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E50" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F50" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G50" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H50">
         <v>2</v>
@@ -2051,22 +2243,22 @@
         <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C51" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D51" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E51" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F51" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G51" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H51">
         <v>3</v>
@@ -2077,22 +2269,22 @@
         <v>20</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D52" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E52" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F52" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G52" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -2103,22 +2295,22 @@
         <v>20</v>
       </c>
       <c r="B53" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D53" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E53" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F53" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G53" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -2129,22 +2321,22 @@
         <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C54" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D54" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E54" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F54" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G54" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H54">
         <v>3</v>
@@ -2155,22 +2347,22 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C55" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D55" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="E55" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F55" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G55" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H55">
         <v>1</v>
@@ -2181,22 +2373,22 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C56" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D56" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E56" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F56" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G56" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H56">
         <v>1</v>
@@ -2207,22 +2399,22 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C57" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D57" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E57" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F57" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G57" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -2233,22 +2425,22 @@
         <v>20</v>
       </c>
       <c r="B58" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C58" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D58" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E58" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F58" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G58" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H58">
         <v>1</v>
@@ -2259,22 +2451,22 @@
         <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C59" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D59" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E59" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F59" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G59" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H59">
         <v>2</v>
@@ -2285,22 +2477,22 @@
         <v>20</v>
       </c>
       <c r="B60" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C60" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D60" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E60" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F60" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G60" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H60">
         <v>3</v>
@@ -2311,22 +2503,22 @@
         <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C61" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D61" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E61" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F61" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G61" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -2337,22 +2529,22 @@
         <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C62" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D62" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E62" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F62" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G62" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H62">
         <v>2</v>
@@ -2363,22 +2555,22 @@
         <v>20</v>
       </c>
       <c r="B63" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C63" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D63" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E63" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F63" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G63" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H63">
         <v>3</v>
@@ -2389,22 +2581,22 @@
         <v>20</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C64" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D64" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E64" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F64" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G64" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H64">
         <v>1</v>
@@ -2415,22 +2607,22 @@
         <v>20</v>
       </c>
       <c r="B65" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C65" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D65" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E65" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F65" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G65" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H65">
         <v>2</v>
@@ -2441,22 +2633,22 @@
         <v>20</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C66" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D66" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E66" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F66" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G66" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H66">
         <v>3</v>
@@ -2467,22 +2659,22 @@
         <v>20</v>
       </c>
       <c r="B67" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C67" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D67" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E67" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F67" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G67" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H67">
         <v>1</v>
@@ -2493,22 +2685,22 @@
         <v>20</v>
       </c>
       <c r="B68" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C68" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D68" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E68" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F68" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G68" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H68">
         <v>2</v>
@@ -2519,22 +2711,22 @@
         <v>20</v>
       </c>
       <c r="B69" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C69" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D69" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E69" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F69" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G69" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H69">
         <v>3</v>
@@ -2545,22 +2737,22 @@
         <v>20</v>
       </c>
       <c r="B70" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C70" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D70" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="E70" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F70" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G70" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -2571,22 +2763,22 @@
         <v>20</v>
       </c>
       <c r="B71" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C71" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D71" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E71" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F71" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G71" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H71">
         <v>1</v>
@@ -2597,22 +2789,22 @@
         <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C72" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D72" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E72" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F72" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G72" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -2623,22 +2815,22 @@
         <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C73" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D73" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E73" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F73" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G73" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -2649,22 +2841,22 @@
         <v>20</v>
       </c>
       <c r="B74" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C74" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D74" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E74" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F74" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G74" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -2675,22 +2867,22 @@
         <v>20</v>
       </c>
       <c r="B75" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C75" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D75" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E75" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F75" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G75" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H75">
         <v>3</v>
@@ -2701,22 +2893,22 @@
         <v>20</v>
       </c>
       <c r="B76" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C76" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D76" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E76" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F76" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G76" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H76">
         <v>1</v>
@@ -2727,22 +2919,22 @@
         <v>20</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C77" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D77" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E77" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F77" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G77" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H77">
         <v>2</v>
@@ -2753,22 +2945,22 @@
         <v>20</v>
       </c>
       <c r="B78" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C78" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D78" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E78" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F78" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G78" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H78">
         <v>3</v>
@@ -2779,22 +2971,22 @@
         <v>20</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C79" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D79" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E79" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F79" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G79" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H79">
         <v>1</v>
@@ -2805,22 +2997,22 @@
         <v>20</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C80" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D80" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E80" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F80" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G80" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H80">
         <v>2</v>
@@ -2831,22 +3023,22 @@
         <v>20</v>
       </c>
       <c r="B81" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C81" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D81" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E81" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F81" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G81" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H81">
         <v>3</v>
@@ -2857,22 +3049,22 @@
         <v>20</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C82" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D82" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E82" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F82" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G82" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H82">
         <v>1</v>
@@ -2883,22 +3075,22 @@
         <v>20</v>
       </c>
       <c r="B83" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C83" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D83" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E83" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F83" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G83" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H83">
         <v>2</v>
@@ -2909,22 +3101,22 @@
         <v>20</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C84" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D84" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E84" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F84" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G84" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H84">
         <v>3</v>
@@ -2935,22 +3127,22 @@
         <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C85" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D85" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="E85" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F85" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G85" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="H85">
         <v>1</v>
@@ -2961,22 +3153,22 @@
         <v>20</v>
       </c>
       <c r="B86" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C86" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D86" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E86" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F86" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G86" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="H86">
         <v>1</v>
@@ -2987,22 +3179,22 @@
         <v>20</v>
       </c>
       <c r="B87" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C87" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D87" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E87" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F87" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G87" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="H87">
         <v>2</v>
@@ -3013,22 +3205,22 @@
         <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C88" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D88" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E88" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F88" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G88" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H88">
         <v>1</v>
@@ -3039,22 +3231,22 @@
         <v>20</v>
       </c>
       <c r="B89" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C89" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D89" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E89" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F89" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G89" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H89">
         <v>2</v>
@@ -3065,22 +3257,22 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C90" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D90" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E90" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F90" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G90" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H90">
         <v>3</v>
@@ -3091,22 +3283,22 @@
         <v>20</v>
       </c>
       <c r="B91" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C91" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D91" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E91" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F91" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G91" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="H91">
         <v>1</v>
@@ -3117,22 +3309,22 @@
         <v>20</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C92" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D92" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E92" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F92" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G92" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="H92">
         <v>2</v>
@@ -3143,22 +3335,22 @@
         <v>20</v>
       </c>
       <c r="B93" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C93" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D93" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="E93" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F93" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G93" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="H93">
         <v>3</v>
@@ -3169,22 +3361,22 @@
         <v>21</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C94" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D94" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="E94" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F94" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G94" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="H94">
         <v>1</v>
@@ -3195,22 +3387,22 @@
         <v>21</v>
       </c>
       <c r="B95" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C95" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D95" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="E95" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F95" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G95" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="H95">
         <v>2</v>
@@ -3221,22 +3413,22 @@
         <v>22</v>
       </c>
       <c r="B96" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C96" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D96" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="E96" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F96" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G96" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="H96">
         <v>1</v>
@@ -3247,22 +3439,22 @@
         <v>22</v>
       </c>
       <c r="B97" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C97" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D97" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="E97" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F97" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G97" t="s">
-        <v>112</v>
+        <v>151</v>
       </c>
       <c r="H97">
         <v>2</v>
@@ -3273,22 +3465,22 @@
         <v>22</v>
       </c>
       <c r="B98" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C98" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D98" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="E98" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F98" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G98" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="H98">
         <v>3</v>
@@ -3299,22 +3491,22 @@
         <v>23</v>
       </c>
       <c r="B99" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C99" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D99" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E99" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F99" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G99" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="H99">
         <v>1</v>
@@ -3325,22 +3517,22 @@
         <v>23</v>
       </c>
       <c r="B100" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C100" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D100" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E100" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F100" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G100" t="s">
-        <v>115</v>
+        <v>154</v>
       </c>
       <c r="H100">
         <v>2</v>
@@ -3351,22 +3543,22 @@
         <v>23</v>
       </c>
       <c r="B101" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C101" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D101" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E101" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F101" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G101" t="s">
-        <v>116</v>
+        <v>155</v>
       </c>
       <c r="H101">
         <v>3</v>
@@ -3377,22 +3569,22 @@
         <v>24</v>
       </c>
       <c r="B102" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C102" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D102" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="E102" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F102" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G102" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="H102">
         <v>1</v>
@@ -3403,22 +3595,22 @@
         <v>24</v>
       </c>
       <c r="B103" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C103" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D103" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="E103" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F103" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G103" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="H103">
         <v>2</v>
@@ -3429,22 +3621,22 @@
         <v>25</v>
       </c>
       <c r="B104" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C104" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D104" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="E104" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F104" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G104" t="s">
-        <v>118</v>
+        <v>157</v>
       </c>
       <c r="H104">
         <v>1</v>
@@ -3455,22 +3647,22 @@
         <v>25</v>
       </c>
       <c r="B105" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C105" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D105" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="E105" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F105" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G105" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="H105">
         <v>2</v>
@@ -3481,22 +3673,22 @@
         <v>25</v>
       </c>
       <c r="B106" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C106" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D106" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="E106" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F106" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G106" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="H106">
         <v>3</v>
@@ -3507,22 +3699,22 @@
         <v>26</v>
       </c>
       <c r="B107" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C107" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D107" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="E107" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F107" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="G107" t="s">
-        <v>120</v>
+        <v>159</v>
       </c>
       <c r="H107">
         <v>1</v>
@@ -3533,22 +3725,22 @@
         <v>26</v>
       </c>
       <c r="B108" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C108" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D108" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="E108" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F108" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G108" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H108">
         <v>2</v>
@@ -3559,22 +3751,22 @@
         <v>26</v>
       </c>
       <c r="B109" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C109" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D109" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="E109" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F109" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="G109" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="H109">
         <v>3</v>
@@ -3585,22 +3777,22 @@
         <v>27</v>
       </c>
       <c r="B110" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C110" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D110" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="E110" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="F110" t="s">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="G110" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="H110">
         <v>1</v>
@@ -3611,24 +3803,934 @@
         <v>27</v>
       </c>
       <c r="B111" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C111" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D111" t="s">
+        <v>99</v>
+      </c>
+      <c r="E111" t="s">
+        <v>113</v>
+      </c>
+      <c r="F111" t="s">
+        <v>115</v>
+      </c>
+      <c r="G111" t="s">
+        <v>162</v>
+      </c>
+      <c r="H111">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8">
+      <c r="A112" t="s">
+        <v>28</v>
+      </c>
+      <c r="B112" t="s">
+        <v>61</v>
+      </c>
+      <c r="C112" t="s">
+        <v>76</v>
+      </c>
+      <c r="D112" t="s">
+        <v>100</v>
+      </c>
+      <c r="E112" t="s">
+        <v>114</v>
+      </c>
+      <c r="F112" t="s">
+        <v>114</v>
+      </c>
+      <c r="G112" t="s">
+        <v>163</v>
+      </c>
+      <c r="H112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8">
+      <c r="A113" t="s">
+        <v>28</v>
+      </c>
+      <c r="B113" t="s">
+        <v>61</v>
+      </c>
+      <c r="C113" t="s">
+        <v>76</v>
+      </c>
+      <c r="D113" t="s">
+        <v>100</v>
+      </c>
+      <c r="E113" t="s">
+        <v>114</v>
+      </c>
+      <c r="F113" t="s">
+        <v>113</v>
+      </c>
+      <c r="G113" t="s">
+        <v>164</v>
+      </c>
+      <c r="H113">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8">
+      <c r="A114" t="s">
+        <v>28</v>
+      </c>
+      <c r="B114" t="s">
+        <v>61</v>
+      </c>
+      <c r="C114" t="s">
+        <v>76</v>
+      </c>
+      <c r="D114" t="s">
+        <v>100</v>
+      </c>
+      <c r="E114" t="s">
+        <v>114</v>
+      </c>
+      <c r="F114" t="s">
+        <v>115</v>
+      </c>
+      <c r="G114" t="s">
+        <v>165</v>
+      </c>
+      <c r="H114">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8">
+      <c r="A115" t="s">
+        <v>29</v>
+      </c>
+      <c r="B115" t="s">
+        <v>62</v>
+      </c>
+      <c r="C115" t="s">
+        <v>76</v>
+      </c>
+      <c r="D115" t="s">
+        <v>101</v>
+      </c>
+      <c r="E115" t="s">
+        <v>113</v>
+      </c>
+      <c r="F115" t="s">
+        <v>113</v>
+      </c>
+      <c r="G115" t="s">
+        <v>166</v>
+      </c>
+      <c r="H115">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8">
+      <c r="A116" t="s">
+        <v>29</v>
+      </c>
+      <c r="B116" t="s">
+        <v>62</v>
+      </c>
+      <c r="C116" t="s">
+        <v>76</v>
+      </c>
+      <c r="D116" t="s">
+        <v>101</v>
+      </c>
+      <c r="E116" t="s">
+        <v>113</v>
+      </c>
+      <c r="F116" t="s">
+        <v>115</v>
+      </c>
+      <c r="G116" t="s">
+        <v>167</v>
+      </c>
+      <c r="H116">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8">
+      <c r="A117" t="s">
+        <v>30</v>
+      </c>
+      <c r="B117" t="s">
+        <v>63</v>
+      </c>
+      <c r="C117" t="s">
+        <v>76</v>
+      </c>
+      <c r="D117" t="s">
+        <v>102</v>
+      </c>
+      <c r="E117" t="s">
+        <v>114</v>
+      </c>
+      <c r="F117" t="s">
+        <v>114</v>
+      </c>
+      <c r="G117" t="s">
+        <v>168</v>
+      </c>
+      <c r="H117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8">
+      <c r="A118" t="s">
+        <v>31</v>
+      </c>
+      <c r="B118" t="s">
+        <v>64</v>
+      </c>
+      <c r="C118" t="s">
+        <v>76</v>
+      </c>
+      <c r="D118" t="s">
+        <v>103</v>
+      </c>
+      <c r="E118" t="s">
+        <v>113</v>
+      </c>
+      <c r="F118" t="s">
+        <v>113</v>
+      </c>
+      <c r="G118" t="s">
+        <v>169</v>
+      </c>
+      <c r="H118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8">
+      <c r="A119" t="s">
+        <v>31</v>
+      </c>
+      <c r="B119" t="s">
+        <v>64</v>
+      </c>
+      <c r="C119" t="s">
+        <v>76</v>
+      </c>
+      <c r="D119" t="s">
+        <v>103</v>
+      </c>
+      <c r="E119" t="s">
+        <v>113</v>
+      </c>
+      <c r="F119" t="s">
+        <v>115</v>
+      </c>
+      <c r="G119" t="s">
+        <v>170</v>
+      </c>
+      <c r="H119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8">
+      <c r="A120" t="s">
+        <v>32</v>
+      </c>
+      <c r="B120" t="s">
+        <v>65</v>
+      </c>
+      <c r="C120" t="s">
+        <v>76</v>
+      </c>
+      <c r="D120" t="s">
+        <v>104</v>
+      </c>
+      <c r="E120" t="s">
+        <v>114</v>
+      </c>
+      <c r="F120" t="s">
+        <v>114</v>
+      </c>
+      <c r="G120" t="s">
+        <v>171</v>
+      </c>
+      <c r="H120">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8">
+      <c r="A121" t="s">
+        <v>32</v>
+      </c>
+      <c r="B121" t="s">
+        <v>65</v>
+      </c>
+      <c r="C121" t="s">
+        <v>76</v>
+      </c>
+      <c r="D121" t="s">
+        <v>104</v>
+      </c>
+      <c r="E121" t="s">
+        <v>114</v>
+      </c>
+      <c r="F121" t="s">
+        <v>114</v>
+      </c>
+      <c r="G121" t="s">
+        <v>172</v>
+      </c>
+      <c r="H121">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8">
+      <c r="A122" t="s">
+        <v>33</v>
+      </c>
+      <c r="B122" t="s">
+        <v>66</v>
+      </c>
+      <c r="C122" t="s">
+        <v>76</v>
+      </c>
+      <c r="D122" t="s">
+        <v>105</v>
+      </c>
+      <c r="E122" t="s">
+        <v>113</v>
+      </c>
+      <c r="F122" t="s">
+        <v>113</v>
+      </c>
+      <c r="G122" t="s">
+        <v>173</v>
+      </c>
+      <c r="H122">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8">
+      <c r="A123" t="s">
+        <v>33</v>
+      </c>
+      <c r="B123" t="s">
+        <v>66</v>
+      </c>
+      <c r="C123" t="s">
+        <v>76</v>
+      </c>
+      <c r="D123" t="s">
+        <v>105</v>
+      </c>
+      <c r="E123" t="s">
+        <v>113</v>
+      </c>
+      <c r="F123" t="s">
+        <v>115</v>
+      </c>
+      <c r="G123" t="s">
+        <v>174</v>
+      </c>
+      <c r="H123">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8">
+      <c r="A124" t="s">
+        <v>34</v>
+      </c>
+      <c r="B124" t="s">
+        <v>67</v>
+      </c>
+      <c r="C124" t="s">
+        <v>76</v>
+      </c>
+      <c r="D124" t="s">
+        <v>106</v>
+      </c>
+      <c r="E124" t="s">
+        <v>113</v>
+      </c>
+      <c r="F124" t="s">
+        <v>115</v>
+      </c>
+      <c r="G124" t="s">
+        <v>175</v>
+      </c>
+      <c r="H124">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8">
+      <c r="A125" t="s">
+        <v>34</v>
+      </c>
+      <c r="B125" t="s">
+        <v>67</v>
+      </c>
+      <c r="C125" t="s">
+        <v>76</v>
+      </c>
+      <c r="D125" t="s">
+        <v>106</v>
+      </c>
+      <c r="E125" t="s">
+        <v>113</v>
+      </c>
+      <c r="F125" t="s">
+        <v>113</v>
+      </c>
+      <c r="G125" t="s">
+        <v>175</v>
+      </c>
+      <c r="H125">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8">
+      <c r="A126" t="s">
+        <v>35</v>
+      </c>
+      <c r="B126" t="s">
+        <v>68</v>
+      </c>
+      <c r="C126" t="s">
+        <v>76</v>
+      </c>
+      <c r="D126" t="s">
+        <v>107</v>
+      </c>
+      <c r="E126" t="s">
+        <v>114</v>
+      </c>
+      <c r="F126" t="s">
+        <v>114</v>
+      </c>
+      <c r="G126" t="s">
+        <v>176</v>
+      </c>
+      <c r="H126">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8">
+      <c r="A127" t="s">
+        <v>35</v>
+      </c>
+      <c r="B127" t="s">
+        <v>68</v>
+      </c>
+      <c r="C127" t="s">
+        <v>76</v>
+      </c>
+      <c r="D127" t="s">
+        <v>107</v>
+      </c>
+      <c r="E127" t="s">
+        <v>114</v>
+      </c>
+      <c r="F127" t="s">
+        <v>113</v>
+      </c>
+      <c r="G127" t="s">
+        <v>177</v>
+      </c>
+      <c r="H127">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8">
+      <c r="A128" t="s">
+        <v>35</v>
+      </c>
+      <c r="B128" t="s">
+        <v>68</v>
+      </c>
+      <c r="C128" t="s">
+        <v>76</v>
+      </c>
+      <c r="D128" t="s">
+        <v>107</v>
+      </c>
+      <c r="E128" t="s">
+        <v>114</v>
+      </c>
+      <c r="F128" t="s">
+        <v>115</v>
+      </c>
+      <c r="G128" t="s">
+        <v>178</v>
+      </c>
+      <c r="H128">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8">
+      <c r="A129" t="s">
+        <v>12</v>
+      </c>
+      <c r="B129" t="s">
+        <v>45</v>
+      </c>
+      <c r="C129" t="s">
+        <v>76</v>
+      </c>
+      <c r="D129" t="s">
+        <v>81</v>
+      </c>
+      <c r="E129" t="s">
+        <v>113</v>
+      </c>
+      <c r="F129" t="s">
+        <v>113</v>
+      </c>
+      <c r="G129" t="s">
+        <v>125</v>
+      </c>
+      <c r="H129">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8">
+      <c r="A130" t="s">
+        <v>12</v>
+      </c>
+      <c r="B130" t="s">
+        <v>45</v>
+      </c>
+      <c r="C130" t="s">
+        <v>76</v>
+      </c>
+      <c r="D130" t="s">
+        <v>81</v>
+      </c>
+      <c r="E130" t="s">
+        <v>113</v>
+      </c>
+      <c r="F130" t="s">
+        <v>115</v>
+      </c>
+      <c r="G130" t="s">
+        <v>126</v>
+      </c>
+      <c r="H130">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8">
+      <c r="A131" t="s">
+        <v>12</v>
+      </c>
+      <c r="B131" t="s">
+        <v>45</v>
+      </c>
+      <c r="C131" t="s">
+        <v>76</v>
+      </c>
+      <c r="D131" t="s">
+        <v>82</v>
+      </c>
+      <c r="E131" t="s">
+        <v>113</v>
+      </c>
+      <c r="F131" t="s">
+        <v>113</v>
+      </c>
+      <c r="G131" t="s">
+        <v>127</v>
+      </c>
+      <c r="H131">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8">
+      <c r="A132" t="s">
+        <v>12</v>
+      </c>
+      <c r="B132" t="s">
+        <v>45</v>
+      </c>
+      <c r="C132" t="s">
+        <v>76</v>
+      </c>
+      <c r="D132" t="s">
+        <v>82</v>
+      </c>
+      <c r="E132" t="s">
+        <v>113</v>
+      </c>
+      <c r="F132" t="s">
+        <v>115</v>
+      </c>
+      <c r="G132" t="s">
+        <v>128</v>
+      </c>
+      <c r="H132">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8">
+      <c r="A133" t="s">
+        <v>12</v>
+      </c>
+      <c r="B133" t="s">
+        <v>45</v>
+      </c>
+      <c r="C133" t="s">
+        <v>76</v>
+      </c>
+      <c r="D133" t="s">
+        <v>81</v>
+      </c>
+      <c r="E133" t="s">
+        <v>113</v>
+      </c>
+      <c r="F133" t="s">
+        <v>113</v>
+      </c>
+      <c r="G133" t="s">
+        <v>125</v>
+      </c>
+      <c r="H133">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8">
+      <c r="A134" t="s">
+        <v>12</v>
+      </c>
+      <c r="B134" t="s">
+        <v>45</v>
+      </c>
+      <c r="C134" t="s">
+        <v>76</v>
+      </c>
+      <c r="D134" t="s">
+        <v>81</v>
+      </c>
+      <c r="E134" t="s">
+        <v>113</v>
+      </c>
+      <c r="F134" t="s">
+        <v>115</v>
+      </c>
+      <c r="G134" t="s">
+        <v>126</v>
+      </c>
+      <c r="H134">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8">
+      <c r="A135" t="s">
+        <v>12</v>
+      </c>
+      <c r="B135" t="s">
+        <v>45</v>
+      </c>
+      <c r="C135" t="s">
+        <v>76</v>
+      </c>
+      <c r="D135" t="s">
+        <v>82</v>
+      </c>
+      <c r="E135" t="s">
+        <v>113</v>
+      </c>
+      <c r="F135" t="s">
+        <v>113</v>
+      </c>
+      <c r="G135" t="s">
+        <v>127</v>
+      </c>
+      <c r="H135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8">
+      <c r="A136" t="s">
+        <v>12</v>
+      </c>
+      <c r="B136" t="s">
+        <v>45</v>
+      </c>
+      <c r="C136" t="s">
+        <v>76</v>
+      </c>
+      <c r="D136" t="s">
+        <v>82</v>
+      </c>
+      <c r="E136" t="s">
+        <v>113</v>
+      </c>
+      <c r="F136" t="s">
+        <v>115</v>
+      </c>
+      <c r="G136" t="s">
+        <v>128</v>
+      </c>
+      <c r="H136">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8">
+      <c r="A137" t="s">
+        <v>36</v>
+      </c>
+      <c r="B137" t="s">
+        <v>69</v>
+      </c>
+      <c r="C137" t="s">
+        <v>76</v>
+      </c>
+      <c r="D137" t="s">
+        <v>108</v>
+      </c>
+      <c r="E137" t="s">
+        <v>113</v>
+      </c>
+      <c r="F137" t="s">
+        <v>113</v>
+      </c>
+      <c r="G137" t="s">
+        <v>179</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8">
+      <c r="A138" t="s">
+        <v>36</v>
+      </c>
+      <c r="B138" t="s">
+        <v>69</v>
+      </c>
+      <c r="C138" t="s">
+        <v>76</v>
+      </c>
+      <c r="D138" t="s">
+        <v>108</v>
+      </c>
+      <c r="E138" t="s">
+        <v>113</v>
+      </c>
+      <c r="F138" t="s">
+        <v>115</v>
+      </c>
+      <c r="G138" t="s">
+        <v>180</v>
+      </c>
+      <c r="H138">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8">
+      <c r="A139" t="s">
+        <v>37</v>
+      </c>
+      <c r="B139" t="s">
+        <v>70</v>
+      </c>
+      <c r="C139" t="s">
+        <v>76</v>
+      </c>
+      <c r="D139" t="s">
+        <v>109</v>
+      </c>
+      <c r="E139" t="s">
+        <v>113</v>
+      </c>
+      <c r="F139" t="s">
+        <v>113</v>
+      </c>
+      <c r="G139" t="s">
+        <v>181</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8">
+      <c r="A140" t="s">
+        <v>37</v>
+      </c>
+      <c r="B140" t="s">
+        <v>70</v>
+      </c>
+      <c r="C140" t="s">
+        <v>76</v>
+      </c>
+      <c r="D140" t="s">
+        <v>109</v>
+      </c>
+      <c r="E140" t="s">
+        <v>113</v>
+      </c>
+      <c r="F140" t="s">
+        <v>115</v>
+      </c>
+      <c r="G140" t="s">
+        <v>182</v>
+      </c>
+      <c r="H140">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8">
+      <c r="A141" t="s">
+        <v>38</v>
+      </c>
+      <c r="B141" t="s">
+        <v>71</v>
+      </c>
+      <c r="C141" t="s">
+        <v>76</v>
+      </c>
+      <c r="D141" t="s">
+        <v>110</v>
+      </c>
+      <c r="E141" t="s">
+        <v>113</v>
+      </c>
+      <c r="F141" t="s">
+        <v>113</v>
+      </c>
+      <c r="G141" t="s">
+        <v>183</v>
+      </c>
+      <c r="H141">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8">
+      <c r="A142" t="s">
+        <v>38</v>
+      </c>
+      <c r="B142" t="s">
+        <v>71</v>
+      </c>
+      <c r="C142" t="s">
+        <v>76</v>
+      </c>
+      <c r="D142" t="s">
+        <v>110</v>
+      </c>
+      <c r="E142" t="s">
+        <v>113</v>
+      </c>
+      <c r="F142" t="s">
+        <v>115</v>
+      </c>
+      <c r="G142" t="s">
+        <v>184</v>
+      </c>
+      <c r="H142">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8">
+      <c r="A143" t="s">
+        <v>39</v>
+      </c>
+      <c r="B143" t="s">
+        <v>72</v>
+      </c>
+      <c r="C143" t="s">
+        <v>76</v>
+      </c>
+      <c r="D143" t="s">
+        <v>111</v>
+      </c>
+      <c r="E143" t="s">
+        <v>113</v>
+      </c>
+      <c r="F143" t="s">
+        <v>113</v>
+      </c>
+      <c r="G143" t="s">
+        <v>185</v>
+      </c>
+      <c r="H143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8">
+      <c r="A144" t="s">
+        <v>39</v>
+      </c>
+      <c r="B144" t="s">
+        <v>72</v>
+      </c>
+      <c r="C144" t="s">
+        <v>76</v>
+      </c>
+      <c r="D144" t="s">
+        <v>111</v>
+      </c>
+      <c r="E144" t="s">
+        <v>113</v>
+      </c>
+      <c r="F144" t="s">
+        <v>115</v>
+      </c>
+      <c r="G144" t="s">
+        <v>186</v>
+      </c>
+      <c r="H144">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8">
+      <c r="A145" t="s">
+        <v>40</v>
+      </c>
+      <c r="B145" t="s">
         <v>73</v>
       </c>
-      <c r="E111" t="s">
-        <v>74</v>
-      </c>
-      <c r="F111" t="s">
-        <v>76</v>
-      </c>
-      <c r="G111" t="s">
-        <v>123</v>
-      </c>
-      <c r="H111">
+      <c r="C145" t="s">
+        <v>76</v>
+      </c>
+      <c r="D145" t="s">
+        <v>112</v>
+      </c>
+      <c r="E145" t="s">
+        <v>113</v>
+      </c>
+      <c r="F145" t="s">
+        <v>113</v>
+      </c>
+      <c r="G145" t="s">
+        <v>187</v>
+      </c>
+      <c r="H145">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8">
+      <c r="A146" t="s">
+        <v>40</v>
+      </c>
+      <c r="B146" t="s">
+        <v>73</v>
+      </c>
+      <c r="C146" t="s">
+        <v>76</v>
+      </c>
+      <c r="D146" t="s">
+        <v>112</v>
+      </c>
+      <c r="E146" t="s">
+        <v>113</v>
+      </c>
+      <c r="F146" t="s">
+        <v>115</v>
+      </c>
+      <c r="G146" t="s">
+        <v>187</v>
+      </c>
+      <c r="H146">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update email history logs and sync browser profile cache data
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -169,6 +169,12 @@
     <t>01b351f3-b52c-4516-a91c-00f58d08579d</t>
   </si>
   <si>
+    <t>b6c21085-5e3c-4d3b-bcb0-1e48c3bbaca7</t>
+  </si>
+  <si>
+    <t>eeee3ec7-6e8b-4ba0-86e1-e4a35de9cc96</t>
+  </si>
+  <si>
     <t>66b93b8d-817c-4af4-9183-47792e43d54e</t>
   </si>
   <si>
@@ -178,12 +184,6 @@
     <t>15f31e98-1701-4d23-8de8-7493899a44db</t>
   </si>
   <si>
-    <t>eeee3ec7-6e8b-4ba0-86e1-e4a35de9cc96</t>
-  </si>
-  <si>
-    <t>b6c21085-5e3c-4d3b-bcb0-1e48c3bbaca7</t>
-  </si>
-  <si>
     <t>f455e248-e952-4fc6-9076-0237c90636fd</t>
   </si>
   <si>
@@ -550,6 +550,12 @@
     <t>KCP MANDIRI MITRA USAHA TENTENA</t>
   </si>
   <si>
+    <t>PDAM KAB DONGGALA</t>
+  </si>
+  <si>
+    <t>ASTUN HI. ARSYAD</t>
+  </si>
+  <si>
     <t>SEKOLAH POLISI NEGARA</t>
   </si>
   <si>
@@ -559,12 +565,6 @@
     <t>BPR PALU LOKADANA UTAMA KAS LABUAN</t>
   </si>
   <si>
-    <t>ASTUN HI. ARSYAD</t>
-  </si>
-  <si>
-    <t>PDAM KAB DONGGALA</t>
-  </si>
-  <si>
     <t>KOPERASI KONSUMEN DHARMA MARITIM TOLITOLI</t>
   </si>
   <si>
@@ -931,6 +931,12 @@
     <t>kcpmandirimitrausaha@gmail.com</t>
   </si>
   <si>
+    <t>pdam_donggala@gmail.com</t>
+  </si>
+  <si>
+    <t>astunhiarsyad28@gmail.com</t>
+  </si>
+  <si>
     <t>kppnpalu651707@yahoo.com</t>
   </si>
   <si>
@@ -940,12 +946,6 @@
     <t>bprlabuan@yahoo.co.id</t>
   </si>
   <si>
-    <t>astunhiarsyad28@gmail.com</t>
-  </si>
-  <si>
-    <t>pdam_donggala@gmail.com</t>
-  </si>
-  <si>
     <t>koperasi_maritim@yahoo.com</t>
   </si>
   <si>
@@ -1480,6 +1480,15 @@
     <t>01 Jun 2026, 22:47:26</t>
   </si>
   <si>
+    <t>02 Jun 2026, 06:31:35</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:45:54</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 09:45:51</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 02:30:55</t>
   </si>
   <si>
@@ -1499,15 +1508,6 @@
   </si>
   <si>
     <t>01 Jun 2026, 23:29:34</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 09:45:54</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 09:45:51</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 06:31:35</t>
   </si>
   <si>
     <t>02 Jun 2026, 10:08:22</t>
@@ -5810,7 +5810,7 @@
         <v>388</v>
       </c>
       <c r="F114" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G114" t="s">
         <v>488</v>
@@ -5839,10 +5839,10 @@
         <v>388</v>
       </c>
       <c r="F115" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G115" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="H115">
         <v>2</v>
@@ -5871,7 +5871,7 @@
         <v>388</v>
       </c>
       <c r="G116" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="H116">
         <v>1</v>
@@ -5900,7 +5900,7 @@
         <v>390</v>
       </c>
       <c r="G117" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H117">
         <v>2</v>
@@ -5923,13 +5923,13 @@
         <v>307</v>
       </c>
       <c r="E118" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F118" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G118" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H118">
         <v>1</v>
@@ -5952,13 +5952,13 @@
         <v>307</v>
       </c>
       <c r="E119" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F119" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G119" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H119">
         <v>2</v>
@@ -5969,28 +5969,28 @@
     </row>
     <row r="120" spans="1:9">
       <c r="A120" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B120" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C120" t="s">
         <v>262</v>
       </c>
       <c r="D120" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E120" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F120" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G120" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H120">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I120" t="s">
         <v>705</v>
@@ -6013,13 +6013,13 @@
         <v>388</v>
       </c>
       <c r="F121" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G121" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="H121">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I121" t="s">
         <v>705</v>
@@ -6027,28 +6027,28 @@
     </row>
     <row r="122" spans="1:9">
       <c r="A122" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B122" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C122" t="s">
         <v>262</v>
       </c>
       <c r="D122" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E122" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F122" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G122" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H122">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I122" t="s">
         <v>705</v>
@@ -6068,16 +6068,16 @@
         <v>309</v>
       </c>
       <c r="E123" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F123" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G123" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="H123">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I123" t="s">
         <v>705</v>
@@ -6097,16 +6097,16 @@
         <v>309</v>
       </c>
       <c r="E124" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F124" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G124" t="s">
         <v>497</v>
       </c>
       <c r="H124">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I124" t="s">
         <v>705</v>

</xml_diff>

<commit_message>
perbaiki tampilan kotak kotak
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3097" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3121" uniqueCount="714">
   <si>
     <t>code</t>
   </si>
@@ -2513,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I387"/>
+  <dimension ref="A1:I390"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -13739,6 +13739,93 @@
         <v>713</v>
       </c>
     </row>
+    <row r="388" spans="1:9">
+      <c r="A388" t="s">
+        <v>92</v>
+      </c>
+      <c r="B388" t="s">
+        <v>218</v>
+      </c>
+      <c r="C388" t="s">
+        <v>261</v>
+      </c>
+      <c r="D388" t="s">
+        <v>346</v>
+      </c>
+      <c r="E388" t="s">
+        <v>389</v>
+      </c>
+      <c r="F388" t="s">
+        <v>389</v>
+      </c>
+      <c r="G388" t="s">
+        <v>604</v>
+      </c>
+      <c r="H388">
+        <v>1</v>
+      </c>
+      <c r="I388" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="389" spans="1:9">
+      <c r="A389" t="s">
+        <v>92</v>
+      </c>
+      <c r="B389" t="s">
+        <v>218</v>
+      </c>
+      <c r="C389" t="s">
+        <v>261</v>
+      </c>
+      <c r="D389" t="s">
+        <v>346</v>
+      </c>
+      <c r="E389" t="s">
+        <v>389</v>
+      </c>
+      <c r="F389" t="s">
+        <v>388</v>
+      </c>
+      <c r="G389" t="s">
+        <v>605</v>
+      </c>
+      <c r="H389">
+        <v>2</v>
+      </c>
+      <c r="I389" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="390" spans="1:9">
+      <c r="A390" t="s">
+        <v>92</v>
+      </c>
+      <c r="B390" t="s">
+        <v>218</v>
+      </c>
+      <c r="C390" t="s">
+        <v>261</v>
+      </c>
+      <c r="D390" t="s">
+        <v>346</v>
+      </c>
+      <c r="E390" t="s">
+        <v>389</v>
+      </c>
+      <c r="F390" t="s">
+        <v>390</v>
+      </c>
+      <c r="G390" t="s">
+        <v>606</v>
+      </c>
+      <c r="H390">
+        <v>3</v>
+      </c>
+      <c r="I390" t="s">
+        <v>713</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement granular assignment tracking and add supporting utility scripts for data processing
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -52,6 +52,9 @@
     <t>81b140d6-80f9-436f-81e4-bbfc8ae820d3</t>
   </si>
   <si>
+    <t>ca7ed898-5339-4d22-8a89-b89adc186705</t>
+  </si>
+  <si>
     <t>5ed2770d-9be6-4fc1-bf70-0d4e10c482c8</t>
   </si>
   <si>
@@ -85,9 +88,6 @@
     <t>87ab3e43-e1be-4b02-af1e-14720ebfb03f</t>
   </si>
   <si>
-    <t>ca7ed898-5339-4d22-8a89-b89adc186705</t>
-  </si>
-  <si>
     <t>0d4bfa96-7cd5-47d9-b366-e133f6ea27c4</t>
   </si>
   <si>
@@ -439,6 +439,9 @@
     <t>BPR MODERN EXPRESS PT</t>
   </si>
   <si>
+    <t>BANK PERKREDITAN RAKYAT PALU LOKADANA UTAMA</t>
+  </si>
+  <si>
     <t>BANK PERKREDITAN RAKYAT MITRA NIAGA BANGGAI</t>
   </si>
   <si>
@@ -472,9 +475,6 @@
     <t>CAHAYA BARU SENTOSA</t>
   </si>
   <si>
-    <t>BANK PERKREDITAN RAKYAT PALU LOKADANA UTAMA</t>
-  </si>
-  <si>
     <t>BANK DANAMON INDONESIA, PT TBK KCP LUWUK</t>
   </si>
   <si>
@@ -814,6 +814,12 @@
     <t>bpr.381@lakadana.com</t>
   </si>
   <si>
+    <t>kc.luwuk@bprpalulokadanautama.com</t>
+  </si>
+  <si>
+    <t>kc.morowali@bprpalulokadanautama.com</t>
+  </si>
+  <si>
     <t>toili@mailnesia.com</t>
   </si>
   <si>
@@ -847,12 +853,6 @@
     <t>cbs_luwuk@yahoo.com</t>
   </si>
   <si>
-    <t>kc.luwuk@bprpalulokadanautama.com</t>
-  </si>
-  <si>
-    <t>kc.morowali@bprpalulokadanautama.com</t>
-  </si>
-  <si>
     <t>bankdanamon.admin@gmail.com</t>
   </si>
   <si>
@@ -1219,6 +1219,18 @@
     <t>11 Jun 2026, 10:53:00</t>
   </si>
   <si>
+    <t>02 Jun 2026, 07:38:30</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:38:27</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:55:41</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 07:55:37</t>
+  </si>
+  <si>
     <t>02 Jun 2026, 02:11:11</t>
   </si>
   <si>
@@ -1289,18 +1301,6 @@
   </si>
   <si>
     <t>02 Jun 2026, 03:51:54</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 07:38:30</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 07:38:27</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 07:55:41</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 07:55:37</t>
   </si>
   <si>
     <t>09 Jun 2026, 11:00:04</t>
@@ -2965,10 +2965,10 @@
         <v>266</v>
       </c>
       <c r="E16" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F16" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G16" t="s">
         <v>401</v>
@@ -2982,28 +2982,28 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" t="s">
         <v>261</v>
       </c>
       <c r="D17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E17" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G17" t="s">
         <v>402</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" t="s">
         <v>702</v>
@@ -3011,10 +3011,10 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C18" t="s">
         <v>261</v>
@@ -3023,7 +3023,7 @@
         <v>267</v>
       </c>
       <c r="E18" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F18" t="s">
         <v>388</v>
@@ -3032,7 +3032,7 @@
         <v>403</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I18" t="s">
         <v>702</v>
@@ -3040,10 +3040,10 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C19" t="s">
         <v>261</v>
@@ -3052,7 +3052,7 @@
         <v>267</v>
       </c>
       <c r="E19" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F19" t="s">
         <v>390</v>
@@ -3061,7 +3061,7 @@
         <v>404</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19" t="s">
         <v>702</v>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C20" t="s">
         <v>261</v>
@@ -3107,19 +3107,19 @@
         <v>261</v>
       </c>
       <c r="D21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E21" t="s">
         <v>389</v>
       </c>
       <c r="F21" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G21" t="s">
         <v>406</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" t="s">
         <v>702</v>
@@ -3136,19 +3136,19 @@
         <v>261</v>
       </c>
       <c r="D22" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E22" t="s">
         <v>389</v>
       </c>
       <c r="F22" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G22" t="s">
         <v>407</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="s">
         <v>702</v>
@@ -3156,10 +3156,10 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C23" t="s">
         <v>261</v>
@@ -3168,16 +3168,16 @@
         <v>269</v>
       </c>
       <c r="E23" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F23" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G23" t="s">
         <v>408</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I23" t="s">
         <v>702</v>
@@ -3194,19 +3194,19 @@
         <v>261</v>
       </c>
       <c r="D24" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E24" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F24" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G24" t="s">
         <v>409</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" t="s">
         <v>702</v>
@@ -3214,10 +3214,10 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
         <v>261</v>
@@ -3226,16 +3226,16 @@
         <v>270</v>
       </c>
       <c r="E25" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G25" t="s">
         <v>410</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" t="s">
         <v>702</v>
@@ -3243,10 +3243,10 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C26" t="s">
         <v>261</v>
@@ -3255,16 +3255,16 @@
         <v>270</v>
       </c>
       <c r="E26" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F26" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G26" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" t="s">
         <v>702</v>
@@ -3272,10 +3272,10 @@
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C27" t="s">
         <v>261</v>
@@ -3284,13 +3284,13 @@
         <v>271</v>
       </c>
       <c r="E27" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F27" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G27" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="H27">
         <v>1</v>
@@ -3301,10 +3301,10 @@
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C28" t="s">
         <v>261</v>
@@ -3313,13 +3313,13 @@
         <v>271</v>
       </c>
       <c r="E28" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F28" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G28" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="H28">
         <v>2</v>
@@ -3339,19 +3339,19 @@
         <v>261</v>
       </c>
       <c r="D29" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E29" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F29" t="s">
         <v>390</v>
       </c>
       <c r="G29" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I29" t="s">
         <v>702</v>
@@ -3359,10 +3359,10 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C30" t="s">
         <v>261</v>
@@ -3380,7 +3380,7 @@
         <v>414</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" t="s">
         <v>702</v>
@@ -3397,19 +3397,19 @@
         <v>261</v>
       </c>
       <c r="D31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E31" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F31" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G31" t="s">
         <v>415</v>
       </c>
       <c r="H31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I31" t="s">
         <v>702</v>
@@ -3417,10 +3417,10 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B32" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C32" t="s">
         <v>261</v>
@@ -3432,13 +3432,13 @@
         <v>389</v>
       </c>
       <c r="F32" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G32" t="s">
         <v>416</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I32" t="s">
         <v>702</v>
@@ -3446,10 +3446,10 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B33" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C33" t="s">
         <v>261</v>
@@ -3461,13 +3461,13 @@
         <v>389</v>
       </c>
       <c r="F33" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G33" t="s">
         <v>417</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I33" t="s">
         <v>702</v>
@@ -3484,19 +3484,19 @@
         <v>261</v>
       </c>
       <c r="D34" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E34" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F34" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G34" t="s">
         <v>418</v>
       </c>
       <c r="H34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I34" t="s">
         <v>702</v>
@@ -3504,10 +3504,10 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C35" t="s">
         <v>261</v>
@@ -3519,13 +3519,13 @@
         <v>388</v>
       </c>
       <c r="F35" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G35" t="s">
         <v>419</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I35" t="s">
         <v>702</v>
@@ -3542,19 +3542,19 @@
         <v>261</v>
       </c>
       <c r="D36" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E36" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F36" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G36" t="s">
         <v>420</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36" t="s">
         <v>702</v>
@@ -3562,10 +3562,10 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C37" t="s">
         <v>261</v>
@@ -3574,16 +3574,16 @@
         <v>275</v>
       </c>
       <c r="E37" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F37" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G37" t="s">
         <v>421</v>
       </c>
       <c r="H37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I37" t="s">
         <v>702</v>
@@ -3591,10 +3591,10 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C38" t="s">
         <v>261</v>
@@ -3603,16 +3603,16 @@
         <v>275</v>
       </c>
       <c r="E38" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F38" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G38" t="s">
         <v>422</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I38" t="s">
         <v>702</v>
@@ -3620,10 +3620,10 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C39" t="s">
         <v>261</v>
@@ -3649,10 +3649,10 @@
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C40" t="s">
         <v>261</v>
@@ -3678,10 +3678,10 @@
     </row>
     <row r="41" spans="1:9">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C41" t="s">
         <v>261</v>
@@ -3707,10 +3707,10 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B42" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C42" t="s">
         <v>261</v>
@@ -3942,13 +3942,13 @@
         <v>26</v>
       </c>
       <c r="B50" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C50" t="s">
         <v>261</v>
       </c>
       <c r="D50" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="E50" t="s">
         <v>388</v>
@@ -3957,7 +3957,7 @@
         <v>390</v>
       </c>
       <c r="G50" t="s">
-        <v>428</v>
+        <v>404</v>
       </c>
       <c r="H50">
         <v>2</v>
@@ -3971,13 +3971,13 @@
         <v>26</v>
       </c>
       <c r="B51" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C51" t="s">
         <v>261</v>
       </c>
       <c r="D51" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="E51" t="s">
         <v>388</v>
@@ -3986,7 +3986,7 @@
         <v>388</v>
       </c>
       <c r="G51" t="s">
-        <v>425</v>
+        <v>401</v>
       </c>
       <c r="H51">
         <v>1</v>
@@ -4000,13 +4000,13 @@
         <v>26</v>
       </c>
       <c r="B52" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C52" t="s">
         <v>261</v>
       </c>
       <c r="D52" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="E52" t="s">
         <v>388</v>
@@ -4015,7 +4015,7 @@
         <v>390</v>
       </c>
       <c r="G52" t="s">
-        <v>426</v>
+        <v>402</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -4029,13 +4029,13 @@
         <v>26</v>
       </c>
       <c r="B53" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C53" t="s">
         <v>261</v>
       </c>
       <c r="D53" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="E53" t="s">
         <v>388</v>
@@ -4044,7 +4044,7 @@
         <v>388</v>
       </c>
       <c r="G53" t="s">
-        <v>427</v>
+        <v>403</v>
       </c>
       <c r="H53">
         <v>1</v>
@@ -5160,7 +5160,7 @@
         <v>44</v>
       </c>
       <c r="B92" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C92" t="s">
         <v>261</v>
@@ -7248,7 +7248,7 @@
         <v>65</v>
       </c>
       <c r="B164" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C164" t="s">
         <v>261</v>
@@ -7277,7 +7277,7 @@
         <v>65</v>
       </c>
       <c r="B165" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C165" t="s">
         <v>261</v>
@@ -7306,7 +7306,7 @@
         <v>65</v>
       </c>
       <c r="B166" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C166" t="s">
         <v>261</v>
@@ -7335,13 +7335,13 @@
         <v>65</v>
       </c>
       <c r="B167" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C167" t="s">
         <v>261</v>
       </c>
       <c r="D167" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E167" t="s">
         <v>389</v>
@@ -7350,7 +7350,7 @@
         <v>388</v>
       </c>
       <c r="G167" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H167">
         <v>2</v>
@@ -7364,13 +7364,13 @@
         <v>65</v>
       </c>
       <c r="B168" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C168" t="s">
         <v>261</v>
       </c>
       <c r="D168" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E168" t="s">
         <v>389</v>
@@ -7379,7 +7379,7 @@
         <v>390</v>
       </c>
       <c r="G168" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="H168">
         <v>3</v>
@@ -7393,13 +7393,13 @@
         <v>65</v>
       </c>
       <c r="B169" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C169" t="s">
         <v>261</v>
       </c>
       <c r="D169" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E169" t="s">
         <v>389</v>
@@ -7408,7 +7408,7 @@
         <v>389</v>
       </c>
       <c r="G169" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="H169">
         <v>1</v>
@@ -10424,7 +10424,7 @@
         <v>389</v>
       </c>
       <c r="G273" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="H273">
         <v>1</v>
@@ -10888,7 +10888,7 @@
         <v>388</v>
       </c>
       <c r="G289" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="H289">
         <v>1</v>
@@ -10917,7 +10917,7 @@
         <v>390</v>
       </c>
       <c r="G290" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="H290">
         <v>2</v>
@@ -13222,7 +13222,7 @@
         <v>131</v>
       </c>
       <c r="B370" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C370" t="s">
         <v>261</v>
@@ -13251,7 +13251,7 @@
         <v>131</v>
       </c>
       <c r="B371" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C371" t="s">
         <v>261</v>
@@ -13280,7 +13280,7 @@
         <v>131</v>
       </c>
       <c r="B372" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C372" t="s">
         <v>261</v>
@@ -13309,13 +13309,13 @@
         <v>131</v>
       </c>
       <c r="B373" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C373" t="s">
         <v>261</v>
       </c>
       <c r="D373" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E373" t="s">
         <v>389</v>
@@ -13324,7 +13324,7 @@
         <v>389</v>
       </c>
       <c r="G373" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="H373">
         <v>1</v>
@@ -13338,13 +13338,13 @@
         <v>131</v>
       </c>
       <c r="B374" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C374" t="s">
         <v>261</v>
       </c>
       <c r="D374" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E374" t="s">
         <v>389</v>
@@ -13353,7 +13353,7 @@
         <v>388</v>
       </c>
       <c r="G374" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H374">
         <v>2</v>
@@ -13367,13 +13367,13 @@
         <v>131</v>
       </c>
       <c r="B375" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C375" t="s">
         <v>261</v>
       </c>
       <c r="D375" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E375" t="s">
         <v>389</v>
@@ -13382,7 +13382,7 @@
         <v>390</v>
       </c>
       <c r="G375" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="H375">
         <v>3</v>

</xml_diff>

<commit_message>
feat: add multiple scratch utility scripts and update submission tracking data and application logic
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -199,18 +199,18 @@
     <t>11fd6f69-871d-4258-81f6-e2145ee9f73a</t>
   </si>
   <si>
+    <t>7caf507f-ded1-4591-bf6a-60996f83c71b</t>
+  </si>
+  <si>
+    <t>3266144a-e1e8-481f-a863-d9ee0ed1a652</t>
+  </si>
+  <si>
+    <t>75b6fc99-ef00-42bd-8f54-fcab0ac2a238</t>
+  </si>
+  <si>
     <t>a9979a0c-403c-4acf-bb30-3023bbfba8b5</t>
   </si>
   <si>
-    <t>75b6fc99-ef00-42bd-8f54-fcab0ac2a238</t>
-  </si>
-  <si>
-    <t>3266144a-e1e8-481f-a863-d9ee0ed1a652</t>
-  </si>
-  <si>
-    <t>7caf507f-ded1-4591-bf6a-60996f83c71b</t>
-  </si>
-  <si>
     <t>8a32e430-23b2-46ff-8b68-7dd7afb33862</t>
   </si>
   <si>
@@ -580,18 +580,18 @@
     <t>BANK PEREKONOMIAN RAKYAT (BPR) MODERN EXPRESS CABANG TOLTIOLI</t>
   </si>
   <si>
+    <t>BANK MANDIRI (PERSERO) TBK KCP BUOL, PT</t>
+  </si>
+  <si>
+    <t>BANK BRI UNIT DIAPATIH</t>
+  </si>
+  <si>
+    <t>PT BANK NEGARA INDONESIA (PERSERO) TBK</t>
+  </si>
+  <si>
     <t>BANK PEREKONOMIAN RAKYAT MODERN EXPRESS</t>
   </si>
   <si>
-    <t>PT BANK NEGARA INDONESIA (PERSERO) TBK</t>
-  </si>
-  <si>
-    <t>BANK BRI UNIT DIAPATIH</t>
-  </si>
-  <si>
-    <t>BANK MANDIRI (PERSERO) TBK KCP BUOL, PT</t>
-  </si>
-  <si>
     <t>BRI UNIT TINOMBO</t>
   </si>
   <si>
@@ -961,18 +961,18 @@
     <t>kc.tolitoli@bprpalulokadanautama.com</t>
   </si>
   <si>
+    <t>nyoalvaro@gmail.com</t>
+  </si>
+  <si>
+    <t>yohanesyafetsulung@gmail.com</t>
+  </si>
+  <si>
+    <t>ynataliaw@gmail.com</t>
+  </si>
+  <si>
     <t>fandhymadjid96@gmail.com</t>
   </si>
   <si>
-    <t>ynataliaw@gmail.com</t>
-  </si>
-  <si>
-    <t>yohanesyafetsulung@gmail.com</t>
-  </si>
-  <si>
-    <t>nyoalvaro@gmail.com</t>
-  </si>
-  <si>
     <t>kaslambunu@yahoo.co.id</t>
   </si>
   <si>
@@ -1543,6 +1543,42 @@
     <t>01 Jun 2026, 23:16:27</t>
   </si>
   <si>
+    <t>19 May 2026, 11:14:38</t>
+  </si>
+  <si>
+    <t>19 May 2026, 11:14:34</t>
+  </si>
+  <si>
+    <t>21 May 2026, 08:24:52</t>
+  </si>
+  <si>
+    <t>21 May 2026, 08:24:48</t>
+  </si>
+  <si>
+    <t>09 Jun 2026, 11:12:55</t>
+  </si>
+  <si>
+    <t>02 Jun 2026, 00:32:29</t>
+  </si>
+  <si>
+    <t>20 May 2026, 11:03:26</t>
+  </si>
+  <si>
+    <t>20 May 2026, 11:03:04</t>
+  </si>
+  <si>
+    <t>20 May 2026, 11:02:47</t>
+  </si>
+  <si>
+    <t>20 May 2026, 11:02:44</t>
+  </si>
+  <si>
+    <t>10 Jun 2026, 15:04:30</t>
+  </si>
+  <si>
+    <t>10 Jun 2026, 14:33:40</t>
+  </si>
+  <si>
     <t>20 May 2026, 14:15:07</t>
   </si>
   <si>
@@ -1571,42 +1607,6 @@
   </si>
   <si>
     <t>02 Jun 2026, 11:49:04</t>
-  </si>
-  <si>
-    <t>20 May 2026, 11:03:26</t>
-  </si>
-  <si>
-    <t>20 May 2026, 11:03:04</t>
-  </si>
-  <si>
-    <t>20 May 2026, 11:02:47</t>
-  </si>
-  <si>
-    <t>20 May 2026, 11:02:44</t>
-  </si>
-  <si>
-    <t>19 May 2026, 11:14:34</t>
-  </si>
-  <si>
-    <t>10 Jun 2026, 15:04:30</t>
-  </si>
-  <si>
-    <t>10 Jun 2026, 14:33:40</t>
-  </si>
-  <si>
-    <t>21 May 2026, 08:24:52</t>
-  </si>
-  <si>
-    <t>21 May 2026, 08:24:48</t>
-  </si>
-  <si>
-    <t>09 Jun 2026, 11:12:55</t>
-  </si>
-  <si>
-    <t>02 Jun 2026, 00:32:29</t>
-  </si>
-  <si>
-    <t>19 May 2026, 11:14:38</t>
   </si>
   <si>
     <t>02 Jun 2026, 04:02:15</t>
@@ -6497,7 +6497,7 @@
         <v>188</v>
       </c>
       <c r="C138" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D138" t="s">
         <v>315</v>
@@ -6506,7 +6506,7 @@
         <v>388</v>
       </c>
       <c r="F138" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="G138" t="s">
         <v>509</v>
@@ -6526,7 +6526,7 @@
         <v>188</v>
       </c>
       <c r="C139" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D139" t="s">
         <v>315</v>
@@ -6535,7 +6535,7 @@
         <v>388</v>
       </c>
       <c r="F139" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G139" t="s">
         <v>510</v>
@@ -6549,28 +6549,28 @@
     </row>
     <row r="140" spans="1:9">
       <c r="A140" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B140" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C140" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D140" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E140" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F140" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="G140" t="s">
         <v>511</v>
       </c>
       <c r="H140">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I140" t="s">
         <v>707</v>
@@ -6578,28 +6578,28 @@
     </row>
     <row r="141" spans="1:9">
       <c r="A141" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B141" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C141" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D141" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E141" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F141" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="G141" t="s">
         <v>512</v>
       </c>
       <c r="H141">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I141" t="s">
         <v>707</v>
@@ -6607,28 +6607,28 @@
     </row>
     <row r="142" spans="1:9">
       <c r="A142" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B142" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C142" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D142" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E142" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F142" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="G142" t="s">
         <v>513</v>
       </c>
       <c r="H142">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I142" t="s">
         <v>707</v>
@@ -6636,28 +6636,28 @@
     </row>
     <row r="143" spans="1:9">
       <c r="A143" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B143" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C143" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D143" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E143" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F143" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="G143" t="s">
         <v>514</v>
       </c>
       <c r="H143">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I143" t="s">
         <v>707</v>
@@ -6665,28 +6665,28 @@
     </row>
     <row r="144" spans="1:9">
       <c r="A144" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B144" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C144" t="s">
         <v>262</v>
       </c>
       <c r="D144" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E144" t="s">
         <v>388</v>
       </c>
       <c r="F144" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="G144" t="s">
         <v>515</v>
       </c>
       <c r="H144">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I144" t="s">
         <v>707</v>
@@ -6694,28 +6694,28 @@
     </row>
     <row r="145" spans="1:9">
       <c r="A145" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B145" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C145" t="s">
         <v>262</v>
       </c>
       <c r="D145" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E145" t="s">
         <v>388</v>
       </c>
       <c r="F145" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G145" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="H145">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I145" t="s">
         <v>707</v>
@@ -6723,28 +6723,28 @@
     </row>
     <row r="146" spans="1:9">
       <c r="A146" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B146" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C146" t="s">
         <v>262</v>
       </c>
       <c r="D146" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E146" t="s">
         <v>388</v>
       </c>
       <c r="F146" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="G146" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="H146">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I146" t="s">
         <v>707</v>
@@ -6752,16 +6752,16 @@
     </row>
     <row r="147" spans="1:9">
       <c r="A147" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B147" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C147" t="s">
         <v>262</v>
       </c>
       <c r="D147" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E147" t="s">
         <v>388</v>
@@ -6770,10 +6770,10 @@
         <v>390</v>
       </c>
       <c r="G147" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="H147">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I147" t="s">
         <v>707</v>
@@ -6781,28 +6781,28 @@
     </row>
     <row r="148" spans="1:9">
       <c r="A148" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B148" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C148" t="s">
         <v>262</v>
       </c>
       <c r="D148" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E148" t="s">
         <v>388</v>
       </c>
       <c r="F148" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="G148" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="H148">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I148" t="s">
         <v>707</v>
@@ -6810,28 +6810,28 @@
     </row>
     <row r="149" spans="1:9">
       <c r="A149" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B149" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C149" t="s">
         <v>262</v>
       </c>
       <c r="D149" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E149" t="s">
         <v>388</v>
       </c>
       <c r="F149" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="G149" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="H149">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I149" t="s">
         <v>707</v>
@@ -6839,28 +6839,28 @@
     </row>
     <row r="150" spans="1:9">
       <c r="A150" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B150" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C150" t="s">
         <v>262</v>
       </c>
       <c r="D150" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E150" t="s">
         <v>388</v>
       </c>
       <c r="F150" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G150" t="s">
         <v>519</v>
       </c>
       <c r="H150">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I150" t="s">
         <v>707</v>
@@ -6868,16 +6868,16 @@
     </row>
     <row r="151" spans="1:9">
       <c r="A151" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B151" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C151" t="s">
         <v>262</v>
       </c>
       <c r="D151" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E151" t="s">
         <v>388</v>
@@ -6889,7 +6889,7 @@
         <v>520</v>
       </c>
       <c r="H151">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I151" t="s">
         <v>707</v>
@@ -6897,28 +6897,28 @@
     </row>
     <row r="152" spans="1:9">
       <c r="A152" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B152" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C152" t="s">
         <v>262</v>
       </c>
       <c r="D152" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E152" t="s">
         <v>388</v>
       </c>
       <c r="F152" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="G152" t="s">
         <v>521</v>
       </c>
       <c r="H152">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I152" t="s">
         <v>707</v>
@@ -6926,28 +6926,28 @@
     </row>
     <row r="153" spans="1:9">
       <c r="A153" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B153" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C153" t="s">
         <v>262</v>
       </c>
       <c r="D153" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E153" t="s">
         <v>388</v>
       </c>
       <c r="F153" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G153" t="s">
         <v>522</v>
       </c>
       <c r="H153">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I153" t="s">
         <v>707</v>
@@ -6955,28 +6955,28 @@
     </row>
     <row r="154" spans="1:9">
       <c r="A154" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B154" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C154" t="s">
         <v>262</v>
       </c>
       <c r="D154" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E154" t="s">
         <v>388</v>
       </c>
       <c r="F154" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G154" t="s">
         <v>523</v>
       </c>
       <c r="H154">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I154" t="s">
         <v>707</v>
@@ -6984,28 +6984,28 @@
     </row>
     <row r="155" spans="1:9">
       <c r="A155" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B155" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C155" t="s">
         <v>262</v>
       </c>
       <c r="D155" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E155" t="s">
         <v>388</v>
       </c>
       <c r="F155" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="G155" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="H155">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I155" t="s">
         <v>707</v>
@@ -7013,28 +7013,28 @@
     </row>
     <row r="156" spans="1:9">
       <c r="A156" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B156" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C156" t="s">
         <v>262</v>
       </c>
       <c r="D156" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E156" t="s">
         <v>388</v>
       </c>
       <c r="F156" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="G156" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="H156">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I156" t="s">
         <v>707</v>
@@ -7042,16 +7042,16 @@
     </row>
     <row r="157" spans="1:9">
       <c r="A157" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B157" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C157" t="s">
         <v>262</v>
       </c>
       <c r="D157" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E157" t="s">
         <v>388</v>
@@ -7060,10 +7060,10 @@
         <v>392</v>
       </c>
       <c r="G157" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="H157">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I157" t="s">
         <v>707</v>
@@ -7071,28 +7071,28 @@
     </row>
     <row r="158" spans="1:9">
       <c r="A158" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B158" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C158" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D158" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E158" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F158" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="G158" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H158">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I158" t="s">
         <v>707</v>
@@ -7100,19 +7100,19 @@
     </row>
     <row r="159" spans="1:9">
       <c r="A159" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B159" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C159" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D159" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E159" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F159" t="s">
         <v>390</v>
@@ -7121,7 +7121,7 @@
         <v>527</v>
       </c>
       <c r="H159">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I159" t="s">
         <v>707</v>
@@ -7129,28 +7129,28 @@
     </row>
     <row r="160" spans="1:9">
       <c r="A160" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B160" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C160" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E160" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F160" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G160" t="s">
         <v>528</v>
       </c>
       <c r="H160">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I160" t="s">
         <v>707</v>
@@ -7158,28 +7158,28 @@
     </row>
     <row r="161" spans="1:9">
       <c r="A161" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B161" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C161" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D161" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E161" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F161" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G161" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H161">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I161" t="s">
         <v>707</v>
@@ -7193,7 +7193,7 @@
         <v>191</v>
       </c>
       <c r="C162" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D162" t="s">
         <v>318</v>
@@ -7202,13 +7202,13 @@
         <v>388</v>
       </c>
       <c r="F162" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="G162" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H162">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I162" t="s">
         <v>707</v>
@@ -7222,7 +7222,7 @@
         <v>191</v>
       </c>
       <c r="C163" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D163" t="s">
         <v>318</v>
@@ -7234,10 +7234,10 @@
         <v>390</v>
       </c>
       <c r="G163" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="H163">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="I163" t="s">
         <v>707</v>

</xml_diff>

<commit_message>
feat: initialize new Chrome user data profile and add scraping utility scripts
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3137" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="714">
   <si>
     <t>code</t>
   </si>
@@ -2513,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I392"/>
+  <dimension ref="A1:I389"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -13797,93 +13797,6 @@
         <v>713</v>
       </c>
     </row>
-    <row r="390" spans="1:9">
-      <c r="A390" t="s">
-        <v>92</v>
-      </c>
-      <c r="B390" t="s">
-        <v>218</v>
-      </c>
-      <c r="C390" t="s">
-        <v>260</v>
-      </c>
-      <c r="D390" t="s">
-        <v>346</v>
-      </c>
-      <c r="E390" t="s">
-        <v>389</v>
-      </c>
-      <c r="F390" t="s">
-        <v>389</v>
-      </c>
-      <c r="G390" t="s">
-        <v>604</v>
-      </c>
-      <c r="H390">
-        <v>1</v>
-      </c>
-      <c r="I390" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="391" spans="1:9">
-      <c r="A391" t="s">
-        <v>92</v>
-      </c>
-      <c r="B391" t="s">
-        <v>218</v>
-      </c>
-      <c r="C391" t="s">
-        <v>260</v>
-      </c>
-      <c r="D391" t="s">
-        <v>346</v>
-      </c>
-      <c r="E391" t="s">
-        <v>389</v>
-      </c>
-      <c r="F391" t="s">
-        <v>388</v>
-      </c>
-      <c r="G391" t="s">
-        <v>605</v>
-      </c>
-      <c r="H391">
-        <v>2</v>
-      </c>
-      <c r="I391" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="392" spans="1:9">
-      <c r="A392" t="s">
-        <v>92</v>
-      </c>
-      <c r="B392" t="s">
-        <v>218</v>
-      </c>
-      <c r="C392" t="s">
-        <v>260</v>
-      </c>
-      <c r="D392" t="s">
-        <v>346</v>
-      </c>
-      <c r="E392" t="s">
-        <v>389</v>
-      </c>
-      <c r="F392" t="s">
-        <v>390</v>
-      </c>
-      <c r="G392" t="s">
-        <v>606</v>
-      </c>
-      <c r="H392">
-        <v>3</v>
-      </c>
-      <c r="I392" t="s">
-        <v>713</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update daily submission statistics and remove completed cycle IDs
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3137" uniqueCount="714">
   <si>
     <t>code</t>
   </si>
@@ -2513,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I389"/>
+  <dimension ref="A1:I392"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -13797,6 +13797,93 @@
         <v>713</v>
       </c>
     </row>
+    <row r="390" spans="1:9">
+      <c r="A390" t="s">
+        <v>92</v>
+      </c>
+      <c r="B390" t="s">
+        <v>218</v>
+      </c>
+      <c r="C390" t="s">
+        <v>260</v>
+      </c>
+      <c r="D390" t="s">
+        <v>346</v>
+      </c>
+      <c r="E390" t="s">
+        <v>389</v>
+      </c>
+      <c r="F390" t="s">
+        <v>389</v>
+      </c>
+      <c r="G390" t="s">
+        <v>604</v>
+      </c>
+      <c r="H390">
+        <v>1</v>
+      </c>
+      <c r="I390" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="391" spans="1:9">
+      <c r="A391" t="s">
+        <v>92</v>
+      </c>
+      <c r="B391" t="s">
+        <v>218</v>
+      </c>
+      <c r="C391" t="s">
+        <v>260</v>
+      </c>
+      <c r="D391" t="s">
+        <v>346</v>
+      </c>
+      <c r="E391" t="s">
+        <v>389</v>
+      </c>
+      <c r="F391" t="s">
+        <v>388</v>
+      </c>
+      <c r="G391" t="s">
+        <v>605</v>
+      </c>
+      <c r="H391">
+        <v>2</v>
+      </c>
+      <c r="I391" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="392" spans="1:9">
+      <c r="A392" t="s">
+        <v>92</v>
+      </c>
+      <c r="B392" t="s">
+        <v>218</v>
+      </c>
+      <c r="C392" t="s">
+        <v>260</v>
+      </c>
+      <c r="D392" t="s">
+        <v>346</v>
+      </c>
+      <c r="E392" t="s">
+        <v>389</v>
+      </c>
+      <c r="F392" t="s">
+        <v>390</v>
+      </c>
+      <c r="G392" t="s">
+        <v>606</v>
+      </c>
+      <c r="H392">
+        <v>3</v>
+      </c>
+      <c r="I392" t="s">
+        <v>713</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update email interaction history and remove completed task tracker
</commit_message>
<xml_diff>
--- a/bounced_emails.xlsx
+++ b/bounced_emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3081" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3129" uniqueCount="721">
   <si>
     <t>code</t>
   </si>
@@ -2534,7 +2534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I385"/>
+  <dimension ref="A1:I391"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -13702,6 +13702,180 @@
         <v>720</v>
       </c>
     </row>
+    <row r="386" spans="1:9">
+      <c r="A386" t="s">
+        <v>88</v>
+      </c>
+      <c r="B386" t="s">
+        <v>212</v>
+      </c>
+      <c r="C386" t="s">
+        <v>258</v>
+      </c>
+      <c r="D386" t="s">
+        <v>340</v>
+      </c>
+      <c r="E386" t="s">
+        <v>387</v>
+      </c>
+      <c r="F386" t="s">
+        <v>390</v>
+      </c>
+      <c r="G386" t="s">
+        <v>595</v>
+      </c>
+      <c r="H386">
+        <v>1</v>
+      </c>
+      <c r="I386" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="387" spans="1:9">
+      <c r="A387" t="s">
+        <v>88</v>
+      </c>
+      <c r="B387" t="s">
+        <v>212</v>
+      </c>
+      <c r="C387" t="s">
+        <v>258</v>
+      </c>
+      <c r="D387" t="s">
+        <v>340</v>
+      </c>
+      <c r="E387" t="s">
+        <v>387</v>
+      </c>
+      <c r="F387" t="s">
+        <v>387</v>
+      </c>
+      <c r="G387" t="s">
+        <v>596</v>
+      </c>
+      <c r="H387">
+        <v>2</v>
+      </c>
+      <c r="I387" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="388" spans="1:9">
+      <c r="A388" t="s">
+        <v>88</v>
+      </c>
+      <c r="B388" t="s">
+        <v>212</v>
+      </c>
+      <c r="C388" t="s">
+        <v>258</v>
+      </c>
+      <c r="D388" t="s">
+        <v>340</v>
+      </c>
+      <c r="E388" t="s">
+        <v>387</v>
+      </c>
+      <c r="F388" t="s">
+        <v>388</v>
+      </c>
+      <c r="G388" t="s">
+        <v>597</v>
+      </c>
+      <c r="H388">
+        <v>3</v>
+      </c>
+      <c r="I388" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="389" spans="1:9">
+      <c r="A389" t="s">
+        <v>91</v>
+      </c>
+      <c r="B389" t="s">
+        <v>215</v>
+      </c>
+      <c r="C389" t="s">
+        <v>258</v>
+      </c>
+      <c r="D389" t="s">
+        <v>343</v>
+      </c>
+      <c r="E389" t="s">
+        <v>386</v>
+      </c>
+      <c r="F389" t="s">
+        <v>386</v>
+      </c>
+      <c r="G389" t="s">
+        <v>607</v>
+      </c>
+      <c r="H389">
+        <v>1</v>
+      </c>
+      <c r="I389" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="390" spans="1:9">
+      <c r="A390" t="s">
+        <v>91</v>
+      </c>
+      <c r="B390" t="s">
+        <v>215</v>
+      </c>
+      <c r="C390" t="s">
+        <v>258</v>
+      </c>
+      <c r="D390" t="s">
+        <v>343</v>
+      </c>
+      <c r="E390" t="s">
+        <v>386</v>
+      </c>
+      <c r="F390" t="s">
+        <v>387</v>
+      </c>
+      <c r="G390" t="s">
+        <v>608</v>
+      </c>
+      <c r="H390">
+        <v>2</v>
+      </c>
+      <c r="I390" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="391" spans="1:9">
+      <c r="A391" t="s">
+        <v>91</v>
+      </c>
+      <c r="B391" t="s">
+        <v>215</v>
+      </c>
+      <c r="C391" t="s">
+        <v>258</v>
+      </c>
+      <c r="D391" t="s">
+        <v>343</v>
+      </c>
+      <c r="E391" t="s">
+        <v>386</v>
+      </c>
+      <c r="F391" t="s">
+        <v>388</v>
+      </c>
+      <c r="G391" t="s">
+        <v>609</v>
+      </c>
+      <c r="H391">
+        <v>3</v>
+      </c>
+      <c r="I391" t="s">
+        <v>720</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>